<commit_message>
Multispeciality exposure: High / Medium / Low level tags (app + Excel)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -649,7 +649,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Multispeciality — label</t>
+          <t>Multispeciality exposure — level</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac)</t>
+          <t>Medium exposure (official: Cardiac)</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Critical care)</t>
+          <t>Medium exposure (official: Critical care)</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac, GI surgery, Critical care)</t>
+          <t>Medium exposure (official: Cardiac, GI surgery, Critical care)</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Critical care)</t>
+          <t>Medium exposure (official: Critical care)</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Neuro, Critical care)</t>
+          <t>Medium exposure (official: Neuro, Critical care)</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>Strong (official)</t>
+          <t>High exposure (4 core SS, official)</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>Strong (official)</t>
+          <t>High exposure (3 core SS, official)</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (3 SS depts on site)</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="N15" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (8 SS depts on site)</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac)</t>
+          <t>Medium exposure (official: Cardiac)</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (4 SS depts on site)</t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac, Neuro)</t>
+          <t>Medium exposure (official: Cardiac, Neuro)</t>
         </is>
       </c>
       <c r="O20" s="3" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Critical care)</t>
+          <t>Medium exposure (official: Critical care)</t>
         </is>
       </c>
       <c r="O21" s="3" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (5 SS depts on site)</t>
         </is>
       </c>
       <c r="O22" s="3" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Critical care, GI surgery)</t>
+          <t>Medium exposure (official: Critical care, GI surgery)</t>
         </is>
       </c>
       <c r="O23" s="3" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (8 SS depts on site)</t>
         </is>
       </c>
       <c r="O24" s="3" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (3 SS depts on site)</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Renal/Transplant)</t>
+          <t>Medium exposure (official: Renal/Transplant)</t>
         </is>
       </c>
       <c r="O26" s="3" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac, Neuro, Critical care)</t>
+          <t>Medium exposure (official: Cardiac, Neuro, Critical care)</t>
         </is>
       </c>
       <c r="O28" s="3" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac, Neuro)</t>
+          <t>Medium exposure (official: Cardiac, Neuro)</t>
         </is>
       </c>
       <c r="O30" s="3" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="N31" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O31" s="3" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="N32" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (3 SS depts on site)</t>
         </is>
       </c>
       <c r="O32" s="3" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="N34" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (5 SS depts on site)</t>
         </is>
       </c>
       <c r="O34" s="3" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="N35" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (6 SS depts on site)</t>
         </is>
       </c>
       <c r="O35" s="3" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (5 SS depts on site)</t>
         </is>
       </c>
       <c r="O37" s="3" t="inlineStr">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="N40" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (5 SS depts on site)</t>
         </is>
       </c>
       <c r="O40" s="3" t="inlineStr">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="N41" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (5 SS depts on site)</t>
         </is>
       </c>
       <c r="O41" s="3" t="inlineStr">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="N42" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac, Renal/Transplant, Critical care)</t>
+          <t>Medium exposure (official: Cardiac, Renal/Transplant, Critical care)</t>
         </is>
       </c>
       <c r="O42" s="3" t="inlineStr">
@@ -4034,7 +4034,7 @@
       </c>
       <c r="N43" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac)</t>
+          <t>Medium exposure (official: Cardiac)</t>
         </is>
       </c>
       <c r="O43" s="3" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="N44" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O44" s="3" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="N45" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (4 SS depts on site)</t>
         </is>
       </c>
       <c r="O45" s="3" t="inlineStr">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="N46" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O46" s="3" t="inlineStr">
@@ -4382,7 +4382,7 @@
       </c>
       <c r="N47" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (4 SS depts on site)</t>
         </is>
       </c>
       <c r="O47" s="3" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="N49" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O49" s="3" t="inlineStr">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="N50" s="5" t="inlineStr">
         <is>
-          <t>Strong (official)</t>
+          <t>High exposure (3 core SS, official)</t>
         </is>
       </c>
       <c r="O50" s="3" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="N51" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O51" s="3" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="N52" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Critical care)</t>
+          <t>Medium exposure (official: Critical care)</t>
         </is>
       </c>
       <c r="O52" s="3" t="inlineStr">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="N53" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (4 SS depts on site)</t>
         </is>
       </c>
       <c r="O53" s="3" t="inlineStr">
@@ -4937,7 +4937,7 @@
       </c>
       <c r="N54" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Critical care)</t>
+          <t>Medium exposure (official: Critical care)</t>
         </is>
       </c>
       <c r="O54" s="3" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="N55" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac, Critical care)</t>
+          <t>Medium exposure (official: Cardiac, Critical care)</t>
         </is>
       </c>
       <c r="O55" s="3" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="N56" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Critical care, Renal/Transplant)</t>
+          <t>Medium exposure (official: Critical care, Renal/Transplant)</t>
         </is>
       </c>
       <c r="O56" s="3" t="inlineStr">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="N57" s="5" t="inlineStr">
         <is>
-          <t>Strong (official)</t>
+          <t>High exposure (3 core SS, official)</t>
         </is>
       </c>
       <c r="O57" s="3" t="inlineStr">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="N58" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Vascular/Thoracic)</t>
+          <t>Medium exposure (official: Vascular/Thoracic)</t>
         </is>
       </c>
       <c r="O58" s="3" t="inlineStr">
@@ -5455,7 +5455,7 @@
       </c>
       <c r="N60" s="5" t="inlineStr">
         <is>
-          <t>Strong (official)</t>
+          <t>High exposure (4 core SS, official)</t>
         </is>
       </c>
       <c r="O60" s="3" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="N61" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O61" s="3" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="N62" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O62" s="3" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="N63" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O63" s="3" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="N64" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (5 SS depts on site)</t>
         </is>
       </c>
       <c r="O64" s="3" t="inlineStr">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="N65" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac)</t>
+          <t>Medium exposure (official: Cardiac)</t>
         </is>
       </c>
       <c r="O65" s="3" t="inlineStr">
@@ -5977,7 +5977,7 @@
       </c>
       <c r="N66" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O66" s="3" t="inlineStr">
@@ -6066,7 +6066,7 @@
       </c>
       <c r="N67" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (4 SS depts on site)</t>
         </is>
       </c>
       <c r="O67" s="3" t="inlineStr">
@@ -6153,7 +6153,7 @@
       </c>
       <c r="N68" s="5" t="inlineStr">
         <is>
-          <t>Strong (official)</t>
+          <t>High exposure (4 core SS, official)</t>
         </is>
       </c>
       <c r="O68" s="3" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="N69" s="6" t="inlineStr">
         <is>
-          <t>Claimed</t>
+          <t>Medium exposure (reported)</t>
         </is>
       </c>
       <c r="O69" s="3" t="inlineStr">
@@ -6432,7 +6432,7 @@
       </c>
       <c r="N73" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac, Renal/Transplant)</t>
+          <t>Medium exposure (official: Cardiac, Renal/Transplant)</t>
         </is>
       </c>
       <c r="O73" s="3" t="inlineStr">
@@ -6523,7 +6523,7 @@
       </c>
       <c r="N74" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (5 SS depts on site)</t>
         </is>
       </c>
       <c r="O74" s="3" t="inlineStr">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="N75" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (6 SS depts on site)</t>
         </is>
       </c>
       <c r="O75" s="3" t="inlineStr">
@@ -6701,7 +6701,7 @@
       </c>
       <c r="N76" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Critical care)</t>
+          <t>Medium exposure (official: Critical care)</t>
         </is>
       </c>
       <c r="O76" s="3" t="inlineStr">
@@ -6788,7 +6788,7 @@
       </c>
       <c r="N77" s="8" t="inlineStr">
         <is>
-          <t>Weak / unclear</t>
+          <t>Low exposure</t>
         </is>
       </c>
       <c r="O77" s="3" t="inlineStr">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="N78" s="5" t="inlineStr">
         <is>
-          <t>Strong (official)</t>
+          <t>High exposure (3 core SS, official)</t>
         </is>
       </c>
       <c r="O78" s="3" t="inlineStr">
@@ -6966,7 +6966,7 @@
       </c>
       <c r="N79" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac)</t>
+          <t>Medium exposure (official: Cardiac)</t>
         </is>
       </c>
       <c r="O79" s="3" t="inlineStr">
@@ -7053,7 +7053,7 @@
       </c>
       <c r="N80" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (6 SS depts on site)</t>
         </is>
       </c>
       <c r="O80" s="3" t="inlineStr">
@@ -7138,7 +7138,7 @@
       </c>
       <c r="N81" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac, Critical care)</t>
+          <t>Medium exposure (official: Cardiac, Critical care)</t>
         </is>
       </c>
       <c r="O81" s="3" t="inlineStr">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="N82" s="6" t="inlineStr">
         <is>
-          <t>Some (official: Cardiac, Neuro, Critical care)</t>
+          <t>Medium exposure (official: Cardiac, Neuro, Critical care)</t>
         </is>
       </c>
       <c r="O82" s="3" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="N84" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (6 SS depts on site)</t>
         </is>
       </c>
       <c r="O84" s="3" t="inlineStr">
@@ -7518,7 +7518,7 @@
       </c>
       <c r="N87" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (3 SS depts on site)</t>
         </is>
       </c>
       <c r="O87" s="3" t="inlineStr">
@@ -7675,7 +7675,7 @@
       </c>
       <c r="N90" s="6" t="inlineStr">
         <is>
-          <t>Claimed on site</t>
+          <t>Medium exposure (5 SS depts on site)</t>
         </is>
       </c>
       <c r="O90" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Shortlist: researched toxicity / hours / ICU for all 89, 13 missing hospitals added, decisive verdicts (no 'after checks')
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -766,12 +766,16 @@
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr"/>
-      <c r="R3" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr"/>
+      <c r="R3" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T3" s="3" t="inlineStr"/>
       <c r="U3" s="3" t="inlineStr"/>
     </row>
@@ -849,12 +853,16 @@
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr"/>
-      <c r="R4" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="inlineStr"/>
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T4" s="3" t="inlineStr"/>
       <c r="U4" s="3" t="inlineStr"/>
     </row>
@@ -930,12 +938,16 @@
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr"/>
-      <c r="R5" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S5" s="3" t="inlineStr"/>
+      <c r="R5" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online; aggregator lists DNB stipend Rs 15,000/mo (2025 MCC data)</t>
+        </is>
+      </c>
       <c r="T5" s="3" t="inlineStr"/>
       <c r="U5" s="3" t="inlineStr"/>
     </row>
@@ -960,9 +972,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1017,12 +1029,16 @@
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr"/>
-      <c r="R6" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S6" s="3" t="inlineStr"/>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T6" s="3" t="inlineStr"/>
       <c r="U6" s="3" t="inlineStr"/>
     </row>
@@ -1098,12 +1114,16 @@
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr"/>
-      <c r="R7" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S7" s="3" t="inlineStr"/>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T7" s="3" t="inlineStr"/>
       <c r="U7" s="3" t="inlineStr"/>
     </row>
@@ -1185,12 +1205,16 @@
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr"/>
-      <c r="R8" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S8" s="3" t="inlineStr"/>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T8" s="3" t="inlineStr"/>
       <c r="U8" s="3" t="inlineStr"/>
     </row>
@@ -1215,14 +1239,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1278,11 +1302,19 @@
       </c>
       <c r="R9" s="8" t="inlineStr">
         <is>
-          <t>Mixed / thin</t>
-        </is>
-      </c>
-      <c r="S9" s="3" t="inlineStr"/>
-      <c r="T9" s="3" t="inlineStr"/>
+          <t>Concerns reported</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>No suicide/strike found; 2017 NBE complaint: inhuman DNB duty hours (radiology); 2025 forum: meagre stipend ~50k</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>32 h/56 h stretches (radiology, 2017 complaint); WLB 5/5 (2025) [forum]</t>
+        </is>
+      </c>
       <c r="U9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1363,13 +1395,21 @@
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr"/>
-      <c r="R10" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S10" s="3" t="inlineStr"/>
-      <c r="T10" s="3" t="inlineStr"/>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>1 death(s) reported</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse 2019-26; radiology PG murdered in hospital duty room (Aug 2017, news)</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>Regular OT days + 6-9 emergency duties/month, weekly OT rotation [forum, 2021]</t>
+        </is>
+      </c>
       <c r="U10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1393,9 +1433,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1450,12 +1490,16 @@
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr"/>
-      <c r="R11" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S11" s="3" t="inlineStr"/>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse re residents; Delhi govt ordered action after probe flagged patient-care lapses (Jun 2026)</t>
+        </is>
+      </c>
       <c r="T11" s="3" t="inlineStr"/>
       <c r="U11" s="3" t="inlineStr"/>
     </row>
@@ -1480,14 +1524,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Join</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1541,12 +1585,16 @@
           <t>No resident or alumni account found. The hospital's DNB anaesthesiology page lists six senior-consultant faculty (MD/DNB qualified 1993-2009); it is a 242-bed private hospital (aggregator). The only 'review' text online is Meducate's generic boilerplate ('diverse clinical caseload ... procedural training'), which is not a resident account.</t>
         </is>
       </c>
-      <c r="R12" s="5" t="inlineStr">
-        <is>
-          <t>Reported OK</t>
-        </is>
-      </c>
-      <c r="S12" s="3" t="inlineStr"/>
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T12" s="3" t="inlineStr"/>
       <c r="U12" s="3" t="inlineStr"/>
     </row>
@@ -1571,14 +1619,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1628,12 +1676,16 @@
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr"/>
-      <c r="R13" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S13" s="3" t="inlineStr"/>
+      <c r="R13" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T13" s="3" t="inlineStr"/>
       <c r="U13" s="3" t="inlineStr"/>
     </row>
@@ -1709,12 +1761,16 @@
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr"/>
-      <c r="R14" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S14" s="3" t="inlineStr"/>
+      <c r="R14" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online (GMERS-wide JR pay cut 2023; Gotri stipend strike)</t>
+        </is>
+      </c>
       <c r="T14" s="3" t="inlineStr"/>
       <c r="U14" s="3" t="inlineStr"/>
     </row>
@@ -1739,14 +1795,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1798,14 +1854,22 @@
           <t>The hospital's own DNB page is unusually explicit: 3 seats a year, 'direct, hands-on involvement in operation-theatre anaesthesia, critical care, obstetric anaesthesia and pain management', 'exposure to regional blocks', structured critical-care rotations and 'close consultant mentorship' from three named senior consultants, in a 200-250-bed tertiary hospital opposite AIIMS Jodhpur (earlier pass: ~100 surgeries/day across 8 OTs). But the programme only started in 2025 (the hospital's own launch posts), so there are no seniors or alumni and no resident account.</t>
         </is>
       </c>
-      <c r="R15" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S15" s="3" t="inlineStr"/>
+      <c r="R15" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online (Jodhpur hits are AIIMS/SNMC, not Medipulse)</t>
+        </is>
+      </c>
       <c r="T15" s="3" t="inlineStr"/>
-      <c r="U15" s="3" t="inlineStr"/>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>Structured critical-care rotations; no duration given [official]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1828,14 +1892,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1885,12 +1949,16 @@
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr"/>
-      <c r="R16" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S16" s="3" t="inlineStr"/>
+      <c r="R16" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online (Jaipur hits are SMS/AIIMS Jodhpur, Rajasthan-wide strike Oct 2024)</t>
+        </is>
+      </c>
       <c r="T16" s="3" t="inlineStr"/>
       <c r="U16" s="3" t="inlineStr"/>
     </row>
@@ -1968,12 +2036,16 @@
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr"/>
-      <c r="R17" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S17" s="3" t="inlineStr"/>
+      <c r="R17" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online (Bikaner suicides were SP Medical College interns/residents, not Kothari)</t>
+        </is>
+      </c>
       <c r="T17" s="3" t="inlineStr"/>
       <c r="U17" s="3" t="inlineStr"/>
     </row>
@@ -2059,14 +2131,22 @@
           <t>No resident account found. meducate (aggregator) says hands-on is 'satisfactory, particularly in orthopaedic procedures and trauma' - a likely good source of regional blocks, but not verified.</t>
         </is>
       </c>
-      <c r="R18" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S18" s="3" t="inlineStr"/>
+      <c r="R18" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T18" s="3" t="inlineStr"/>
-      <c r="U18" s="3" t="inlineStr"/>
+      <c r="U18" s="3" t="inlineStr">
+        <is>
+          <t>25-bed ICU; dept trains anaesthesia+critical care together; no rota [official]</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -2140,12 +2220,16 @@
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr"/>
-      <c r="R19" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S19" s="3" t="inlineStr"/>
+      <c r="R19" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online (Lucknow hits are KGMU, not Max/Sahara)</t>
+        </is>
+      </c>
       <c r="T19" s="3" t="inlineStr"/>
       <c r="U19" s="3" t="inlineStr"/>
     </row>
@@ -2170,9 +2254,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -2231,14 +2315,22 @@
           <t>No resident account found. meducate (aggregator) says 'hands-on procedural opportunities in surgical specialties may be limited due to the consultant-led corporate practice model'. 2 DNB anaesthesia seats/yr.</t>
         </is>
       </c>
-      <c r="R20" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S20" s="3" t="inlineStr"/>
+      <c r="R20" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T20" s="3" t="inlineStr"/>
-      <c r="U20" s="3" t="inlineStr"/>
+      <c r="U20" s="3" t="inlineStr">
+        <is>
+          <t>ICU/critical-care rotations 'strong exposure'; no duration [forum]</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -2261,9 +2353,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -2322,14 +2414,22 @@
           <t>No resident account found. meducate (aggregator) says exposure is strongest in ICU/critical care and many procedures are consultant-led. 2 (+1) DNB anaesthesia seats/yr.</t>
         </is>
       </c>
-      <c r="R21" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S21" s="3" t="inlineStr"/>
+      <c r="R21" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online (Greater Noida trainee suicide Sept 2025 not linked to Kailash)</t>
+        </is>
+      </c>
       <c r="T21" s="3" t="inlineStr"/>
-      <c r="U21" s="3" t="inlineStr"/>
+      <c r="U21" s="3" t="inlineStr">
+        <is>
+          <t>ICU/critical-care exposure 'decent', cardiac+neuro ICU; no duration [forum]</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -2352,14 +2452,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -2413,22 +2513,26 @@
           <t>One anonymous DNB anaesthesia resident review (meducate, Aug 2022) is strongly positive on hands-on: 'Yes totally', 'all types of cases seen', patient load 'average', weekly case presentation and discussion for the next day's OT, 'far better than others for DNB'. Officially (2025 DNB brochure and department page): 300+ beds with 60 L4 ICU beds, 8 operation theatres (4 modular, 2 emergency, 2 minor), sub-speciality anaesthetists for transplant, paediatric, cardiac, neuro and obstetric work, cardiac-surgery anaesthesia and a pain clinic; 2 primary + 1 secondary DNB anaesthesia seats; HOD holds DA, DNB and FNB Critical Care. Single-source resident evidence, four years old.</t>
         </is>
       </c>
-      <c r="R22" s="8" t="inlineStr">
-        <is>
-          <t>Mixed / thin</t>
+      <c r="R22" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
         </is>
       </c>
       <c r="S22" s="3" t="inlineStr">
         <is>
-          <t>Recurrent violence/vandalism by patients' relatives after deaths (Sept 2025 and earlier), with hostile local press - personal-safety concern for residents · Mob violence after patient deaths and 'den of greed' coverage in local press (Sept 2025)</t>
+          <t>Nothing adverse found online; 2022 resident: 'dept very chill', no bond</t>
         </is>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>8 hrs a day compulsory rest choice', 'Department very chill', no · 8 hrs a day compulsory rest choice'</t>
-        </is>
-      </c>
-      <c r="U22" s="3" t="inlineStr"/>
+          <t>8 h/day, 'compulsory rest choice' [forum, 2022]</t>
+        </is>
+      </c>
+      <c r="U22" s="3" t="inlineStr">
+        <is>
+          <t>Dept runs 3 ICUs (Med/Surg/CCU), 60 L4 beds; no rota [official]</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -2451,14 +2555,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -2512,12 +2616,16 @@
           <t>No resident account found. The hospital's own (2012-13 era) anaesthesia page lists four round-the-clock OTs, an ICU, labour analgesia and ALS workshops for doctors/paramedics, with no USG-block, simulation or case-volume data. An aggregator's templated 'DNB review' says the ICU and dialysis units give hands-on critical-care exposure but that 'hands-on exposure in surgical specialties may be limited as many operative cases remain consultant-led' - unsourced, weak evidence.</t>
         </is>
       </c>
-      <c r="R23" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S23" s="3" t="inlineStr"/>
+      <c r="R23" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S23" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T23" s="3" t="inlineStr"/>
       <c r="U23" s="3" t="inlineStr"/>
     </row>
@@ -2597,12 +2705,16 @@
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr"/>
-      <c r="R24" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S24" s="3" t="inlineStr"/>
+      <c r="R24" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T24" s="3" t="inlineStr"/>
       <c r="U24" s="3" t="inlineStr"/>
     </row>
@@ -2689,7 +2801,11 @@
           <t>Unknown — ask</t>
         </is>
       </c>
-      <c r="S25" s="3" t="inlineStr"/>
+      <c r="S25" s="3" t="inlineStr">
+        <is>
+          <t>No resident incident found; consultant urologist suicide at sister college HIMS (Sept 2026, news)</t>
+        </is>
+      </c>
       <c r="T25" s="3" t="inlineStr"/>
       <c r="U25" s="3" t="inlineStr"/>
     </row>
@@ -2714,14 +2830,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -2775,13 +2891,21 @@
           <t>DNB Anaesthesiology at Chandan is brand new - the hospital announced its launch in Sept 2025 and the MCC DNB matrix lists 3 seats - so there are no alumni or senior residents to ask. The hospital's own page claims general/regional anaesthesia and regional-block-based post-operative pain management with a 24x7 intensivist-run ICU; the only 'review' is an aggregator saying exposure is moderate and hands-on depends on consultant involvement.</t>
         </is>
       </c>
-      <c r="R26" s="8" t="inlineStr">
-        <is>
-          <t>Mixed / thin</t>
-        </is>
-      </c>
-      <c r="S26" s="3" t="inlineStr"/>
-      <c r="T26" s="3" t="inlineStr"/>
+      <c r="R26" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="inlineStr">
+        <is>
+          <t>'structured working hours, balanced residency' (aggregator, no number) [snippet]</t>
+        </is>
+      </c>
       <c r="U26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
@@ -2856,12 +2980,16 @@
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr"/>
-      <c r="R27" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S27" s="3" t="inlineStr"/>
+      <c r="R27" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S27" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T27" s="3" t="inlineStr"/>
       <c r="U27" s="3" t="inlineStr"/>
     </row>
@@ -2886,14 +3014,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Join</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -2947,12 +3075,16 @@
           <t>Nothing from residents. The hospital is now branded 'CARE CHL Hospitals' (CARE Hospitals group); its anaesthesia HOD Dr Meenu Chadha is described as 42 years' experience in neuro, ortho, onco, paediatric and laparoscopic anaesthesia (hospital/aggregator snippets). Meducate lists 200 beds. Bing returned junk for every 'CHL' query; DuckDuckGo found no resident or workshop content.</t>
         </is>
       </c>
-      <c r="R28" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S28" s="3" t="inlineStr"/>
+      <c r="R28" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S28" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T28" s="3" t="inlineStr"/>
       <c r="U28" s="3" t="inlineStr"/>
     </row>
@@ -3026,12 +3158,16 @@
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr"/>
-      <c r="R29" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S29" s="3" t="inlineStr"/>
+      <c r="R29" s="8" t="inlineStr">
+        <is>
+          <t>Concerns reported</t>
+        </is>
+      </c>
+      <c r="S29" s="3" t="inlineStr">
+        <is>
+          <t>PG stipend strike (Apr 2026, 3 months unpaid); MP-wide JUDA strike (Mar 2026)</t>
+        </is>
+      </c>
       <c r="T29" s="3" t="inlineStr"/>
       <c r="U29" s="3" t="inlineStr"/>
     </row>
@@ -3056,9 +3192,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3113,12 +3249,16 @@
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr"/>
-      <c r="R30" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S30" s="3" t="inlineStr"/>
+      <c r="R30" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T30" s="3" t="inlineStr"/>
       <c r="U30" s="3" t="inlineStr"/>
     </row>
@@ -3203,8 +3343,16 @@
           <t>Some reports</t>
         </is>
       </c>
-      <c r="S31" s="3" t="inlineStr"/>
-      <c r="T31" s="3" t="inlineStr"/>
+      <c r="S31" s="3" t="inlineStr">
+        <is>
+          <t>Nothing hospital-specific; HP-wide resident strike (Dec 2025, IGMC termination)</t>
+        </is>
+      </c>
+      <c r="T31" s="3" t="inlineStr">
+        <is>
+          <t>Emergency duty 2-4 days/mo (roster Apr 2024) [official]; HP 12 h/shift cap</t>
+        </is>
+      </c>
       <c r="U31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
@@ -3288,8 +3436,16 @@
           <t>Some reports</t>
         </is>
       </c>
-      <c r="S32" s="3" t="inlineStr"/>
-      <c r="T32" s="3" t="inlineStr"/>
+      <c r="S32" s="3" t="inlineStr">
+        <is>
+          <t>Nothing hospital-specific; HP-wide resident strike (Dec 2025, IGMC termination)</t>
+        </is>
+      </c>
+      <c r="T32" s="3" t="inlineStr">
+        <is>
+          <t>HP policy: 12 h/shift cap for residents (Dec 2025) [news]; no local roster</t>
+        </is>
+      </c>
       <c r="U32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
@@ -3305,7 +3461,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
+          <t>not in app data (no MCC anaesthesia allotment 2024–25)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr"/>
@@ -3323,7 +3479,11 @@
       <c r="P33" s="3" t="inlineStr"/>
       <c r="Q33" s="3" t="inlineStr"/>
       <c r="R33" s="3" t="inlineStr"/>
-      <c r="S33" s="3" t="inlineStr"/>
+      <c r="S33" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online (resident-level); UMC negligence fine Rs 10L 2025 (patient case)</t>
+        </is>
+      </c>
       <c r="T33" s="3" t="inlineStr"/>
       <c r="U33" s="3" t="inlineStr"/>
     </row>
@@ -3405,12 +3565,16 @@
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr"/>
-      <c r="R34" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S34" s="3" t="inlineStr"/>
+      <c r="R34" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S34" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T34" s="3" t="inlineStr"/>
       <c r="U34" s="3" t="inlineStr"/>
     </row>
@@ -3435,14 +3599,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -3490,12 +3654,16 @@
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr"/>
-      <c r="R35" s="8" t="inlineStr">
-        <is>
-          <t>Mixed / thin</t>
-        </is>
-      </c>
-      <c r="S35" s="3" t="inlineStr"/>
+      <c r="R35" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S35" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T35" s="3" t="inlineStr"/>
       <c r="U35" s="3" t="inlineStr">
         <is>
@@ -3516,25 +3684,81 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr"/>
-      <c r="E36" s="3" t="inlineStr"/>
-      <c r="F36" s="3" t="inlineStr"/>
-      <c r="G36" s="3" t="inlineStr"/>
-      <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr"/>
-      <c r="J36" s="3" t="inlineStr"/>
-      <c r="K36" s="3" t="inlineStr"/>
-      <c r="L36" s="3" t="inlineStr"/>
-      <c r="M36" s="3" t="inlineStr"/>
-      <c r="N36" s="3" t="inlineStr"/>
-      <c r="O36" s="3" t="inlineStr"/>
-      <c r="P36" s="3" t="inlineStr"/>
+          <t>Satguru Partap Singh Hospital</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 37,887); not researched.</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>37887</v>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>29374</v>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>₹67,968</t>
+        </is>
+      </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>High exposure (3 core SS, official)</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: Critical care, Cardiac, Neuro, GI surgery</t>
+        </is>
+      </c>
+      <c r="P36" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q36" s="3" t="inlineStr"/>
-      <c r="R36" s="3" t="inlineStr"/>
-      <c r="S36" s="3" t="inlineStr"/>
+      <c r="R36" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S36" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T36" s="3" t="inlineStr"/>
       <c r="U36" s="3" t="inlineStr"/>
     </row>
@@ -3559,14 +3783,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -3620,12 +3844,16 @@
           <t>No trainee account found. Officially Livasa (formerly Ivy) Mohali is NBEMS-accredited for DNB in Anaesthesiology, Cardiology and Radiodiagnosis; the DNB Anaesthesiology / DrNB Critical Care programme director is the hospital's Director of Critical Care Medicine, which suggests an ICU-weighted programme. The hospital (227 beds per NBEMS data) publicises CABG/valve surgery, 500+ neuro-navigation surgeries, thrombectomy, aneurysm coiling and awake craniotomy, and the anaesthesia page lists nerve blocks, difficult-airway work and radiofrequency ablation - but no OT count, case numbers or resident testimony.</t>
         </is>
       </c>
-      <c r="R37" s="8" t="inlineStr">
-        <is>
-          <t>Mixed / thin</t>
-        </is>
-      </c>
-      <c r="S37" s="3" t="inlineStr"/>
+      <c r="R37" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S37" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T37" s="3" t="inlineStr"/>
       <c r="U37" s="3" t="inlineStr"/>
     </row>
@@ -3642,25 +3870,81 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr"/>
-      <c r="E38" s="3" t="inlineStr"/>
-      <c r="F38" s="3" t="inlineStr"/>
-      <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="3" t="inlineStr"/>
-      <c r="J38" s="3" t="inlineStr"/>
-      <c r="K38" s="3" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr"/>
-      <c r="M38" s="3" t="inlineStr"/>
-      <c r="N38" s="3" t="inlineStr"/>
-      <c r="O38" s="3" t="inlineStr"/>
-      <c r="P38" s="3" t="inlineStr"/>
+          <t>Mohandai Oswal Hospital</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 36,932); not researched.</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>36932</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>28910</v>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>₹67,968</t>
+        </is>
+      </c>
+      <c r="N38" s="6" t="inlineStr">
+        <is>
+          <t>Medium exposure (official: Onco)</t>
+        </is>
+      </c>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: Onco</t>
+        </is>
+      </c>
+      <c r="P38" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q38" s="3" t="inlineStr"/>
-      <c r="R38" s="3" t="inlineStr"/>
-      <c r="S38" s="3" t="inlineStr"/>
+      <c r="R38" s="8" t="inlineStr">
+        <is>
+          <t>Concerns reported</t>
+        </is>
+      </c>
+      <c r="S38" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse 2019-26; historical: 2007 DNB admit during lapsed accreditation, Rs 5L compensation (NCDRC 2018)</t>
+        </is>
+      </c>
       <c r="T38" s="3" t="inlineStr"/>
       <c r="U38" s="3" t="inlineStr"/>
     </row>
@@ -3677,25 +3961,81 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr"/>
-      <c r="G39" s="3" t="inlineStr"/>
-      <c r="H39" s="3" t="inlineStr"/>
-      <c r="I39" s="3" t="inlineStr"/>
-      <c r="J39" s="3" t="inlineStr"/>
-      <c r="K39" s="3" t="inlineStr"/>
-      <c r="L39" s="3" t="inlineStr"/>
-      <c r="M39" s="3" t="inlineStr"/>
-      <c r="N39" s="3" t="inlineStr"/>
-      <c r="O39" s="3" t="inlineStr"/>
-      <c r="P39" s="3" t="inlineStr"/>
+          <t>Fortis Hospital</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 37,505); not researched.</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>37505</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>28510</v>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>₹68,000</t>
+        </is>
+      </c>
+      <c r="N39" s="6" t="inlineStr">
+        <is>
+          <t>Medium exposure (official: GI surgery, Critical care)</t>
+        </is>
+      </c>
+      <c r="O39" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: GI surgery, Critical care</t>
+        </is>
+      </c>
+      <c r="P39" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q39" s="3" t="inlineStr"/>
-      <c r="R39" s="3" t="inlineStr"/>
-      <c r="S39" s="3" t="inlineStr"/>
+      <c r="R39" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S39" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T39" s="3" t="inlineStr"/>
       <c r="U39" s="3" t="inlineStr"/>
     </row>
@@ -3720,14 +4060,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -3779,14 +4119,22 @@
           <t>200-bed flagship of the Amandeep group, running DNB anaesthesia as a joint programme with Amandeep Medicity as secondary hospital (4 seats). The earlier pass recorded institutional claims of USG- and PNS-guided blocks, paediatric regional, TIVA, fibreoptic/video-laryngoscope intubation, POCUS and simulation; this pass could not re-locate that page (the hospital's DNB course URLs now return empty pages) and found no resident account. The group markets itself as a joint-replacement centre, which implies an orthopaedic, regional-anaesthesia-heavy case mix; the plastic-surgery DNB page shows daily morning academic sessions for trainees.</t>
         </is>
       </c>
-      <c r="R40" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S40" s="3" t="inlineStr"/>
+      <c r="R40" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S40" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T40" s="3" t="inlineStr"/>
-      <c r="U40" s="3" t="inlineStr"/>
+      <c r="U40" s="3" t="inlineStr">
+        <is>
+          <t>ICU rotation listed (RICU/CCU/Neuro/Septic ICU), no duration [official]</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -3870,12 +4218,16 @@
           <t>Not found online beyond the hospital's own marketing. In 2025 8 DNB anaesthesia seats were allotted (3 retained, 2 upgraded, 3 not reported per Formity), so about 8 trainees share a 158-bed hospital's case load.</t>
         </is>
       </c>
-      <c r="R41" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S41" s="3" t="inlineStr"/>
+      <c r="R41" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S41" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T41" s="3" t="inlineStr"/>
       <c r="U41" s="3" t="inlineStr"/>
     </row>
@@ -3900,14 +4252,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -3966,7 +4318,11 @@
           <t>Mixed / thin</t>
         </is>
       </c>
-      <c r="S42" s="3" t="inlineStr"/>
+      <c r="S42" s="3" t="inlineStr">
+        <is>
+          <t>No resident item; staff reviews allege unpaid salary/F&amp;F (2020-21), 'no job security' (3.0/5, 31 reviews)</t>
+        </is>
+      </c>
       <c r="T42" s="3" t="inlineStr"/>
       <c r="U42" s="3" t="inlineStr"/>
     </row>
@@ -4048,12 +4404,16 @@
         </is>
       </c>
       <c r="Q43" s="3" t="inlineStr"/>
-      <c r="R43" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S43" s="3" t="inlineStr"/>
+      <c r="R43" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S43" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T43" s="3" t="inlineStr"/>
       <c r="U43" s="3" t="inlineStr"/>
     </row>
@@ -4133,12 +4493,16 @@
         </is>
       </c>
       <c r="Q44" s="3" t="inlineStr"/>
-      <c r="R44" s="6" t="inlineStr">
-        <is>
-          <t>Some reports</t>
-        </is>
-      </c>
-      <c r="S44" s="3" t="inlineStr"/>
+      <c r="R44" s="8" t="inlineStr">
+        <is>
+          <t>Concerns reported</t>
+        </is>
+      </c>
+      <c r="S44" s="3" t="inlineStr">
+        <is>
+          <t>PCMSA doctors' strike (Sep 2024); 3 patient deaths, anaesthetist+SMO suspended (Jul 2025); no PG-specific item</t>
+        </is>
+      </c>
       <c r="T44" s="3" t="inlineStr"/>
       <c r="U44" s="3" t="inlineStr"/>
     </row>
@@ -4163,14 +4527,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -4224,12 +4588,16 @@
           <t>One first-hand account exists: a 2022 first-batch DNB/DA anaesthesia resident (Dr Rahul Marakana, LinkedIn, 2025) reports 60-70 adult + paediatric cardiac cases/month with 'full hands-on exposure', 300+ general surgeries/month (spine, ortho, gynae, trauma, paeds, high-risk), non-OR anaesthesia (MRI/CT/scopy/ECT), vascular and cath-lab work, and training in a 50+ bed Level-3 closed ICU (ventilation, sepsis, haemodynamics, CRRT/ECMO basics). Tone is strongly positive and the hospital's HR replied under it, so treat as a single enthusiastic (possibly curated) testimonial; NBEMS accredits 3 DNB specialities + DA here and a DNB Cardiothoracic (6-yr) seat is also listed, which supports the cardiac claim.</t>
         </is>
       </c>
-      <c r="R45" s="8" t="inlineStr">
-        <is>
-          <t>Mixed / thin</t>
-        </is>
-      </c>
-      <c r="S45" s="3" t="inlineStr"/>
+      <c r="R45" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S45" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T45" s="3" t="inlineStr"/>
       <c r="U45" s="3" t="inlineStr"/>
     </row>
@@ -4311,14 +4679,26 @@
         </is>
       </c>
       <c r="Q46" s="3" t="inlineStr"/>
-      <c r="R46" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S46" s="3" t="inlineStr"/>
-      <c r="T46" s="3" t="inlineStr"/>
-      <c r="U46" s="3" t="inlineStr"/>
+      <c r="R46" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S46" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
+      <c r="T46" s="3" t="inlineStr">
+        <is>
+          <t>OT 8am-2pm; 3-4 x 18 h night calls/month (yr1-2), 4-5 x 8 h (yr3) [forum]</t>
+        </is>
+      </c>
+      <c r="U46" s="3" t="inlineStr">
+        <is>
+          <t>2 months/yr ICU + 1 mo Raipur GMC SS + 1 mo cardiac OT (2021) [forum]</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -4396,12 +4776,16 @@
         </is>
       </c>
       <c r="Q47" s="3" t="inlineStr"/>
-      <c r="R47" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S47" s="3" t="inlineStr"/>
+      <c r="R47" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S47" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T47" s="3" t="inlineStr"/>
       <c r="U47" s="3" t="inlineStr"/>
     </row>
@@ -4418,25 +4802,81 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr"/>
-      <c r="E48" s="3" t="inlineStr"/>
-      <c r="F48" s="3" t="inlineStr"/>
-      <c r="G48" s="3" t="inlineStr"/>
-      <c r="H48" s="3" t="inlineStr"/>
-      <c r="I48" s="3" t="inlineStr"/>
-      <c r="J48" s="3" t="inlineStr"/>
-      <c r="K48" s="3" t="inlineStr"/>
-      <c r="L48" s="3" t="inlineStr"/>
-      <c r="M48" s="3" t="inlineStr"/>
-      <c r="N48" s="3" t="inlineStr"/>
-      <c r="O48" s="3" t="inlineStr"/>
-      <c r="P48" s="3" t="inlineStr"/>
+          <t>MMI Narayana Multispecialty Hospital</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 36,827); not researched.</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="n">
+        <v>36827</v>
+      </c>
+      <c r="J48" s="3" t="n">
+        <v>30158</v>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>₹67,500</t>
+        </is>
+      </c>
+      <c r="N48" s="6" t="inlineStr">
+        <is>
+          <t>Medium exposure (official: Neuro, Critical care)</t>
+        </is>
+      </c>
+      <c r="O48" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: Neuro, Critical care</t>
+        </is>
+      </c>
+      <c r="P48" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q48" s="3" t="inlineStr"/>
-      <c r="R48" s="3" t="inlineStr"/>
-      <c r="S48" s="3" t="inlineStr"/>
+      <c r="R48" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S48" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T48" s="3" t="inlineStr"/>
       <c r="U48" s="3" t="inlineStr"/>
     </row>
@@ -4512,14 +4952,14 @@
         </is>
       </c>
       <c r="Q49" s="3" t="inlineStr"/>
-      <c r="R49" s="6" t="inlineStr">
-        <is>
-          <t>Some reports</t>
+      <c r="R49" s="4" t="inlineStr">
+        <is>
+          <t>1 death(s) reported</t>
         </is>
       </c>
       <c r="S49" s="3" t="inlineStr">
         <is>
-          <t>Statewide JDA strike threat over stipend (Aug 2026)</t>
+          <t>1 MBBS student suicide (Aug 2025, not PG); intern+PG stipend strike (Aug 2026); JDA OPD boycott (Sep 2026)</t>
         </is>
       </c>
       <c r="T49" s="3" t="inlineStr"/>
@@ -4612,7 +5052,11 @@
           <t>Reported OK</t>
         </is>
       </c>
-      <c r="S50" s="3" t="inlineStr"/>
+      <c r="S50" s="3" t="inlineStr">
+        <is>
+          <t>JR reviews: 'toxic environment, poor work-life balance, manpower crisis' (2023/25); MTMC MBBS suicide (Aug 2025)</t>
+        </is>
+      </c>
       <c r="T50" s="3" t="inlineStr"/>
       <c r="U50" s="3" t="inlineStr"/>
     </row>
@@ -4694,12 +5138,16 @@
         </is>
       </c>
       <c r="Q51" s="3" t="inlineStr"/>
-      <c r="R51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S51" s="3" t="inlineStr"/>
+      <c r="R51" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S51" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T51" s="3" t="inlineStr"/>
       <c r="U51" s="3" t="inlineStr"/>
     </row>
@@ -4724,14 +5172,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -4781,12 +5229,16 @@
         </is>
       </c>
       <c r="Q52" s="3" t="inlineStr"/>
-      <c r="R52" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S52" s="3" t="inlineStr"/>
+      <c r="R52" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S52" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T52" s="3" t="inlineStr"/>
       <c r="U52" s="3" t="inlineStr"/>
     </row>
@@ -4864,12 +5316,16 @@
         </is>
       </c>
       <c r="Q53" s="3" t="inlineStr"/>
-      <c r="R53" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S53" s="3" t="inlineStr"/>
+      <c r="R53" s="4" t="inlineStr">
+        <is>
+          <t>1 death(s) reported</t>
+        </is>
+      </c>
+      <c r="S53" s="3" t="inlineStr">
+        <is>
+          <t>1 DNB resident suicide (1st-yr OBGYN, Mar 2025; note cited course dissatisfaction)</t>
+        </is>
+      </c>
       <c r="T53" s="3" t="inlineStr"/>
       <c r="U53" s="3" t="inlineStr"/>
     </row>
@@ -4951,12 +5407,16 @@
         </is>
       </c>
       <c r="Q54" s="3" t="inlineStr"/>
-      <c r="R54" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S54" s="3" t="inlineStr"/>
+      <c r="R54" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S54" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse for PGs found online (Apr 2025 staff-member suicide off-campus, not a resident)</t>
+        </is>
+      </c>
       <c r="T54" s="3" t="inlineStr"/>
       <c r="U54" s="3" t="inlineStr"/>
     </row>
@@ -5038,12 +5498,16 @@
         </is>
       </c>
       <c r="Q55" s="3" t="inlineStr"/>
-      <c r="R55" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S55" s="3" t="inlineStr"/>
+      <c r="R55" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S55" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T55" s="3" t="inlineStr"/>
       <c r="U55" s="3" t="inlineStr"/>
     </row>
@@ -5125,12 +5589,16 @@
         </is>
       </c>
       <c r="Q56" s="3" t="inlineStr"/>
-      <c r="R56" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S56" s="3" t="inlineStr"/>
+      <c r="R56" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S56" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T56" s="3" t="inlineStr"/>
       <c r="U56" s="3" t="inlineStr"/>
     </row>
@@ -5212,12 +5680,16 @@
         </is>
       </c>
       <c r="Q57" s="3" t="inlineStr"/>
-      <c r="R57" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S57" s="3" t="inlineStr"/>
+      <c r="R57" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S57" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T57" s="3" t="inlineStr"/>
       <c r="U57" s="3" t="inlineStr"/>
     </row>
@@ -5299,12 +5771,16 @@
         </is>
       </c>
       <c r="Q58" s="3" t="inlineStr"/>
-      <c r="R58" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S58" s="3" t="inlineStr"/>
+      <c r="R58" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S58" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T58" s="3" t="inlineStr"/>
       <c r="U58" s="3" t="inlineStr"/>
     </row>
@@ -5382,13 +5858,21 @@
         </is>
       </c>
       <c r="Q59" s="3" t="inlineStr"/>
-      <c r="R59" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S59" s="3" t="inlineStr"/>
-      <c r="T59" s="3" t="inlineStr"/>
+      <c r="R59" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S59" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
+      <c r="T59" s="3" t="inlineStr">
+        <is>
+          <t>8 h shifts, 6-7 nights/mo, post-night off (radiology DNB, not anaes) [forum]</t>
+        </is>
+      </c>
       <c r="U59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
@@ -5412,9 +5896,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
@@ -5469,12 +5953,16 @@
         </is>
       </c>
       <c r="Q60" s="3" t="inlineStr"/>
-      <c r="R60" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S60" s="3" t="inlineStr"/>
+      <c r="R60" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S60" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T60" s="3" t="inlineStr"/>
       <c r="U60" s="3" t="inlineStr"/>
     </row>
@@ -5554,12 +6042,16 @@
           <t>Aggregator review (anecdotal/templated): 'balanced mix of structured academics and hands-on exposure'; 'manageable patient loads'.</t>
         </is>
       </c>
-      <c r="R61" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S61" s="3" t="inlineStr"/>
+      <c r="R61" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S61" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse for PGs found online (Jun 2025 data-entry staff salary-delay protest hit OPD, not residents)</t>
+        </is>
+      </c>
       <c r="T61" s="3" t="inlineStr"/>
       <c r="U61" s="3" t="inlineStr"/>
     </row>
@@ -5641,12 +6133,16 @@
         </is>
       </c>
       <c r="Q62" s="3" t="inlineStr"/>
-      <c r="R62" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S62" s="3" t="inlineStr"/>
+      <c r="R62" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S62" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T62" s="3" t="inlineStr"/>
       <c r="U62" s="3" t="inlineStr"/>
     </row>
@@ -5726,12 +6222,16 @@
         </is>
       </c>
       <c r="Q63" s="3" t="inlineStr"/>
-      <c r="R63" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S63" s="3" t="inlineStr"/>
+      <c r="R63" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S63" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T63" s="3" t="inlineStr"/>
       <c r="U63" s="3" t="inlineStr"/>
     </row>
@@ -5813,12 +6313,16 @@
         </is>
       </c>
       <c r="Q64" s="3" t="inlineStr"/>
-      <c r="R64" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S64" s="3" t="inlineStr"/>
+      <c r="R64" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S64" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T64" s="3" t="inlineStr"/>
       <c r="U64" s="3" t="inlineStr"/>
     </row>
@@ -5843,14 +6347,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E65" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F65" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F65" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -5904,12 +6408,16 @@
           <t>228-bed NABH/NABL hospital with 8 OTs (aggregator) in the Narayana Health group, with on-site 'Cardiac Sciences' and 'Neuro Sciences' centres, an 18-bed dialysis unit and 20 'advanced care' beds (official page; the unit began as Sahyadri Narayana Hrudayalaya, a cardiac hospital). The aggregator review is generic ('broad clinical exposure across OPD, IPD, emergency, ICUs, OTs and super-specialty rotations'); group-level AmbitionBox resident reviews (2) rate skill development 5/5. No Shimoga-specific anaesthesia-resident account.</t>
         </is>
       </c>
-      <c r="R65" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S65" s="3" t="inlineStr"/>
+      <c r="R65" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S65" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T65" s="3" t="inlineStr"/>
       <c r="U65" s="3" t="inlineStr"/>
     </row>
@@ -5995,12 +6503,16 @@
           <t>Aggregator review (anecdotal/templated): involvement in deliveries, neonatal care, emergency procedures and routine surgeries under supervision; high OPD load.</t>
         </is>
       </c>
-      <c r="R66" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S66" s="3" t="inlineStr"/>
+      <c r="R66" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S66" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T66" s="3" t="inlineStr"/>
       <c r="U66" s="3" t="inlineStr"/>
     </row>
@@ -6080,12 +6592,16 @@
         </is>
       </c>
       <c r="Q67" s="3" t="inlineStr"/>
-      <c r="R67" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S67" s="3" t="inlineStr"/>
+      <c r="R67" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S67" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T67" s="3" t="inlineStr"/>
       <c r="U67" s="3" t="inlineStr"/>
     </row>
@@ -6167,12 +6683,16 @@
         </is>
       </c>
       <c r="Q68" s="3" t="inlineStr"/>
-      <c r="R68" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S68" s="3" t="inlineStr"/>
+      <c r="R68" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S68" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T68" s="3" t="inlineStr"/>
       <c r="U68" s="3" t="inlineStr"/>
     </row>
@@ -6197,9 +6717,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E69" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
@@ -6254,14 +6774,22 @@
         </is>
       </c>
       <c r="Q69" s="3" t="inlineStr"/>
-      <c r="R69" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S69" s="3" t="inlineStr"/>
+      <c r="R69" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S69" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T69" s="3" t="inlineStr"/>
-      <c r="U69" s="3" t="inlineStr"/>
+      <c r="U69" s="3" t="inlineStr">
+        <is>
+          <t>Dept runs neuro/cardiac/liver-transplant ICUs; no PG posting length [official]</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -6276,25 +6804,77 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr"/>
-      <c r="E70" s="3" t="inlineStr"/>
-      <c r="F70" s="3" t="inlineStr"/>
-      <c r="G70" s="3" t="inlineStr"/>
-      <c r="H70" s="3" t="inlineStr"/>
-      <c r="I70" s="3" t="inlineStr"/>
-      <c r="J70" s="3" t="inlineStr"/>
-      <c r="K70" s="3" t="inlineStr"/>
-      <c r="L70" s="3" t="inlineStr"/>
-      <c r="M70" s="3" t="inlineStr"/>
-      <c r="N70" s="3" t="inlineStr"/>
+          <t>Apollo Specialty Hospital</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 36,668); not researched.</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="n">
+        <v>36668</v>
+      </c>
+      <c r="J70" s="3" t="n">
+        <v>25926</v>
+      </c>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M70" s="3" t="inlineStr">
+        <is>
+          <t>₹35,000</t>
+        </is>
+      </c>
+      <c r="N70" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="O70" s="3" t="inlineStr"/>
-      <c r="P70" s="3" t="inlineStr"/>
+      <c r="P70" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q70" s="3" t="inlineStr"/>
-      <c r="R70" s="3" t="inlineStr"/>
-      <c r="S70" s="3" t="inlineStr"/>
+      <c r="R70" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S70" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T70" s="3" t="inlineStr"/>
       <c r="U70" s="3" t="inlineStr"/>
     </row>
@@ -6311,25 +6891,79 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr"/>
-      <c r="E71" s="3" t="inlineStr"/>
-      <c r="F71" s="3" t="inlineStr"/>
-      <c r="G71" s="3" t="inlineStr"/>
-      <c r="H71" s="3" t="inlineStr"/>
-      <c r="I71" s="3" t="inlineStr"/>
+          <t>Billroth Hospital</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 36,823); not researched.</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="n">
+        <v>36823</v>
+      </c>
       <c r="J71" s="3" t="inlineStr"/>
-      <c r="K71" s="3" t="inlineStr"/>
-      <c r="L71" s="3" t="inlineStr"/>
-      <c r="M71" s="3" t="inlineStr"/>
-      <c r="N71" s="3" t="inlineStr"/>
-      <c r="O71" s="3" t="inlineStr"/>
-      <c r="P71" s="3" t="inlineStr"/>
+      <c r="K71" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M71" s="3" t="inlineStr">
+        <is>
+          <t>₹50,923</t>
+        </is>
+      </c>
+      <c r="N71" s="6" t="inlineStr">
+        <is>
+          <t>Medium exposure (official: Cardiac, GI surgery)</t>
+        </is>
+      </c>
+      <c r="O71" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: Cardiac, GI surgery</t>
+        </is>
+      </c>
+      <c r="P71" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q71" s="3" t="inlineStr"/>
-      <c r="R71" s="3" t="inlineStr"/>
-      <c r="S71" s="3" t="inlineStr"/>
+      <c r="R71" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S71" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T71" s="3" t="inlineStr"/>
       <c r="U71" s="3" t="inlineStr"/>
     </row>
@@ -6346,25 +6980,79 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="inlineStr"/>
-      <c r="E72" s="3" t="inlineStr"/>
-      <c r="F72" s="3" t="inlineStr"/>
-      <c r="G72" s="3" t="inlineStr"/>
-      <c r="H72" s="3" t="inlineStr"/>
-      <c r="I72" s="3" t="inlineStr"/>
+          <t>Kongunad Hospitals Private Limited</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 37,022); not researched.</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="n">
+        <v>37022</v>
+      </c>
       <c r="J72" s="3" t="inlineStr"/>
-      <c r="K72" s="3" t="inlineStr"/>
-      <c r="L72" s="3" t="inlineStr"/>
-      <c r="M72" s="3" t="inlineStr"/>
-      <c r="N72" s="3" t="inlineStr"/>
-      <c r="O72" s="3" t="inlineStr"/>
-      <c r="P72" s="3" t="inlineStr"/>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L72" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M72" s="3" t="inlineStr">
+        <is>
+          <t>₹50,000</t>
+        </is>
+      </c>
+      <c r="N72" s="6" t="inlineStr">
+        <is>
+          <t>Medium exposure (official: Cardiac)</t>
+        </is>
+      </c>
+      <c r="O72" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: Cardiac</t>
+        </is>
+      </c>
+      <c r="P72" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q72" s="3" t="inlineStr"/>
-      <c r="R72" s="3" t="inlineStr"/>
-      <c r="S72" s="3" t="inlineStr"/>
+      <c r="R72" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S72" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T72" s="3" t="inlineStr"/>
       <c r="U72" s="3" t="inlineStr"/>
     </row>
@@ -6389,14 +7077,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E73" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F73" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F73" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -6450,12 +7138,16 @@
           <t>Nothing from trainees. Directory data list 8 anaesthesiologists, 2 cardiothoracic surgeons, 3 nephrologists and 3 critical-care specialists - a comparatively large anaesthesia team for a 4-speciality, 10-seat DNB hospital. The Hindu (9 Oct 2026) reports the hospital felicitating staff on completing 125 kidney transplants, confirming an active renal transplant programme (the input's Renal/Transplant exposure). A DNB/EDAIC-qualified consultant joined anaesthesia in Aug 2024 (Instagram). No OT count, case numbers or academics page.</t>
         </is>
       </c>
-      <c r="R73" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S73" s="3" t="inlineStr"/>
+      <c r="R73" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S73" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T73" s="3" t="inlineStr"/>
       <c r="U73" s="3" t="inlineStr"/>
     </row>
@@ -6480,14 +7172,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E74" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F74" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F74" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -6541,12 +7233,16 @@
           <t>60-year-old NABH trust hospital (founded 1965) with about 200-214 beds; recent additions are a NICU, a chemotherapy suite and a kidney-transplant surgery (site banner). The anaesthesia department page is a JavaScript app whose text could not be extracted and the DNB page on jeyasekharanhospital.edu.in is offline. The aggregator review praises 'robust hands-on exposure in labour rooms, emergency care and minor surgical procedures' and supportive faculty, but that is written for medicine/OBG/paediatrics residents, not anaesthesia.</t>
         </is>
       </c>
-      <c r="R74" s="8" t="inlineStr">
-        <is>
-          <t>Mixed / thin</t>
-        </is>
-      </c>
-      <c r="S74" s="3" t="inlineStr"/>
+      <c r="R74" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S74" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T74" s="3" t="inlineStr"/>
       <c r="U74" s="3" t="inlineStr"/>
     </row>
@@ -6628,12 +7324,16 @@
         </is>
       </c>
       <c r="Q75" s="3" t="inlineStr"/>
-      <c r="R75" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S75" s="3" t="inlineStr"/>
+      <c r="R75" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S75" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T75" s="3" t="inlineStr"/>
       <c r="U75" s="3" t="inlineStr"/>
     </row>
@@ -6715,12 +7415,16 @@
         </is>
       </c>
       <c r="Q76" s="3" t="inlineStr"/>
-      <c r="R76" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S76" s="3" t="inlineStr"/>
+      <c r="R76" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S76" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T76" s="3" t="inlineStr"/>
       <c r="U76" s="3" t="inlineStr"/>
     </row>
@@ -6802,14 +7506,22 @@
         </is>
       </c>
       <c r="Q77" s="3" t="inlineStr"/>
-      <c r="R77" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S77" s="3" t="inlineStr"/>
+      <c r="R77" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S77" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T77" s="3" t="inlineStr"/>
-      <c r="U77" s="3" t="inlineStr"/>
+      <c r="U77" s="3" t="inlineStr">
+        <is>
+          <t>10-bed closed ICU, 1 consultant + 1 resident round the clock [official]</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -6832,14 +7544,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E78" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F78" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Join</t>
+        </is>
+      </c>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -6893,12 +7605,16 @@
           <t>230-bed unit (aggregator) running DNB Anaesthesiology (post-MBBS and post-diploma) under Apollo's academic programme. One Glassdoor review titled 'DNB residency at Apollo Guwahati' by a DNB resident doctor says 'Brand, patient exposure is good' (only the snippet is readable). No other resident account; DNB Anaesthesiology closing rank 38,993 (2025) vs 31,709 (2024).</t>
         </is>
       </c>
-      <c r="R78" s="5" t="inlineStr">
-        <is>
-          <t>Reported OK</t>
-        </is>
-      </c>
-      <c r="S78" s="3" t="inlineStr"/>
+      <c r="R78" s="8" t="inlineStr">
+        <is>
+          <t>Concerns reported</t>
+        </is>
+      </c>
+      <c r="S78" s="3" t="inlineStr">
+        <is>
+          <t>Consultants' 2-day OPD/elective strike vs management, senior doctors 'humiliated' (Jun 2026)</t>
+        </is>
+      </c>
       <c r="T78" s="3" t="inlineStr"/>
       <c r="U78" s="3" t="inlineStr"/>
     </row>
@@ -6980,12 +7696,16 @@
         </is>
       </c>
       <c r="Q79" s="3" t="inlineStr"/>
-      <c r="R79" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S79" s="3" t="inlineStr"/>
+      <c r="R79" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S79" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T79" s="3" t="inlineStr"/>
       <c r="U79" s="3" t="inlineStr"/>
     </row>
@@ -7010,14 +7730,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E80" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F80" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -7067,12 +7787,16 @@
         </is>
       </c>
       <c r="Q80" s="3" t="inlineStr"/>
-      <c r="R80" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S80" s="3" t="inlineStr"/>
+      <c r="R80" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S80" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T80" s="3" t="inlineStr"/>
       <c r="U80" s="3" t="inlineStr"/>
     </row>
@@ -7156,12 +7880,16 @@
           <t>5 OTs + burn OT in a 100-bed hospital - modest volume. No resident account found.</t>
         </is>
       </c>
-      <c r="R81" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S81" s="3" t="inlineStr"/>
+      <c r="R81" s="4" t="inlineStr">
+        <is>
+          <t>1 death(s) reported</t>
+        </is>
+      </c>
+      <c r="S81" s="3" t="inlineStr">
+        <is>
+          <t>ICU doctor (EMO, not PG) died by suicide on duty inside ICU (Sep 2026); family cites personal harassment</t>
+        </is>
+      </c>
       <c r="T81" s="3" t="inlineStr"/>
       <c r="U81" s="3" t="inlineStr"/>
     </row>
@@ -7186,14 +7914,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E82" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F82" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>Join</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -7245,12 +7973,16 @@
           <t>200-bed private hospital (neetvantage) whose academics page lists DNB Anaesthesiology alongside DNB/DrNB programmes in neurosurgery and others; the anaesthesia faculty block shows MD/DNB anaesthetists including FNB (Critical Care) and DrNB (Critical Care) qualified consultants and a paediatric-anaesthesia fellow, a 'Neuro Anaesthesia' service, and a GI &amp; liver-transplant unit with its own critical-care/anaesthesia consultant (ex-PGIMER/ILBS, per LinkedIn). No resident account of what DNB trainees actually do, and no OT/case numbers published.</t>
         </is>
       </c>
-      <c r="R82" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S82" s="3" t="inlineStr"/>
+      <c r="R82" s="8" t="inlineStr">
+        <is>
+          <t>Concerns reported</t>
+        </is>
+      </c>
+      <c r="S82" s="3" t="inlineStr">
+        <is>
+          <t>Nurse suicide on premises (Aug 2025): staff allege senior harassment + 'heart attack' cover-up; no PG incident</t>
+        </is>
+      </c>
       <c r="T82" s="3" t="inlineStr"/>
       <c r="U82" s="3" t="inlineStr"/>
     </row>
@@ -7267,25 +7999,81 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr"/>
-      <c r="E83" s="3" t="inlineStr"/>
-      <c r="F83" s="3" t="inlineStr"/>
-      <c r="G83" s="3" t="inlineStr"/>
-      <c r="H83" s="3" t="inlineStr"/>
-      <c r="I83" s="3" t="inlineStr"/>
-      <c r="J83" s="3" t="inlineStr"/>
-      <c r="K83" s="3" t="inlineStr"/>
-      <c r="L83" s="3" t="inlineStr"/>
-      <c r="M83" s="3" t="inlineStr"/>
-      <c r="N83" s="3" t="inlineStr"/>
-      <c r="O83" s="3" t="inlineStr"/>
-      <c r="P83" s="3" t="inlineStr"/>
+          <t>Jaiprakash Hospital and Research Centre Pvt. Ltd</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 37,321); not researched.</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="n">
+        <v>37321</v>
+      </c>
+      <c r="J83" s="3" t="n">
+        <v>28677</v>
+      </c>
+      <c r="K83" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L83" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M83" s="3" t="inlineStr">
+        <is>
+          <t>₹90,000</t>
+        </is>
+      </c>
+      <c r="N83" s="6" t="inlineStr">
+        <is>
+          <t>Medium exposure (official: Neuro, Critical care)</t>
+        </is>
+      </c>
+      <c r="O83" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: Neuro, Critical care</t>
+        </is>
+      </c>
+      <c r="P83" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q83" s="3" t="inlineStr"/>
-      <c r="R83" s="3" t="inlineStr"/>
-      <c r="S83" s="3" t="inlineStr"/>
+      <c r="R83" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S83" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T83" s="3" t="inlineStr"/>
       <c r="U83" s="3" t="inlineStr"/>
     </row>
@@ -7373,12 +8161,12 @@
       </c>
       <c r="R84" s="6" t="inlineStr">
         <is>
-          <t>Some reports</t>
+          <t>Nothing adverse online</t>
         </is>
       </c>
       <c r="S84" s="3" t="inlineStr">
         <is>
-          <t>Manipur ethnic conflict since May 2023 with deaths, displacement, internet blackouts and President's Rule</t>
+          <t>Nothing adverse found online</t>
         </is>
       </c>
       <c r="T84" s="3" t="inlineStr"/>
@@ -7397,25 +8185,79 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="inlineStr"/>
-      <c r="E85" s="3" t="inlineStr"/>
-      <c r="F85" s="3" t="inlineStr"/>
-      <c r="G85" s="3" t="inlineStr"/>
-      <c r="H85" s="3" t="inlineStr"/>
-      <c r="I85" s="3" t="inlineStr"/>
+          <t>Medicover Hospitals MVP</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 36,924); not researched.</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="n">
+        <v>36924</v>
+      </c>
       <c r="J85" s="3" t="inlineStr"/>
-      <c r="K85" s="3" t="inlineStr"/>
-      <c r="L85" s="3" t="inlineStr"/>
-      <c r="M85" s="3" t="inlineStr"/>
-      <c r="N85" s="3" t="inlineStr"/>
-      <c r="O85" s="3" t="inlineStr"/>
-      <c r="P85" s="3" t="inlineStr"/>
+      <c r="K85" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L85" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M85" s="3" t="inlineStr">
+        <is>
+          <t>₹60,823</t>
+        </is>
+      </c>
+      <c r="N85" s="6" t="inlineStr">
+        <is>
+          <t>Medium exposure (official: Cardiac, Renal/Transplant, Critical care)</t>
+        </is>
+      </c>
+      <c r="O85" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: Cardiac, Renal/Transplant, Critical care</t>
+        </is>
+      </c>
+      <c r="P85" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q85" s="3" t="inlineStr"/>
-      <c r="R85" s="3" t="inlineStr"/>
-      <c r="S85" s="3" t="inlineStr"/>
+      <c r="R85" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S85" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T85" s="3" t="inlineStr"/>
       <c r="U85" s="3" t="inlineStr"/>
     </row>
@@ -7432,25 +8274,77 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D86" s="3" t="inlineStr"/>
-      <c r="E86" s="3" t="inlineStr"/>
-      <c r="F86" s="3" t="inlineStr"/>
-      <c r="G86" s="3" t="inlineStr"/>
-      <c r="H86" s="3" t="inlineStr"/>
-      <c r="I86" s="3" t="inlineStr"/>
-      <c r="J86" s="3" t="inlineStr"/>
-      <c r="K86" s="3" t="inlineStr"/>
-      <c r="L86" s="3" t="inlineStr"/>
-      <c r="M86" s="3" t="inlineStr"/>
-      <c r="N86" s="3" t="inlineStr"/>
+          <t>APOLLO SPECIALITY HOSPITALS</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 35,956); not researched.</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>35956</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>29669</v>
+      </c>
+      <c r="K86" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L86" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M86" s="3" t="inlineStr">
+        <is>
+          <t>₹48,000</t>
+        </is>
+      </c>
+      <c r="N86" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="O86" s="3" t="inlineStr"/>
-      <c r="P86" s="3" t="inlineStr"/>
+      <c r="P86" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q86" s="3" t="inlineStr"/>
-      <c r="R86" s="3" t="inlineStr"/>
-      <c r="S86" s="3" t="inlineStr"/>
+      <c r="R86" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S86" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T86" s="3" t="inlineStr"/>
       <c r="U86" s="3" t="inlineStr"/>
     </row>
@@ -7475,14 +8369,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E87" s="6" t="inlineStr">
-        <is>
-          <t>Join, after checks</t>
-        </is>
-      </c>
-      <c r="F87" s="5" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -7534,10 +8428,14 @@
       <c r="Q87" s="3" t="inlineStr"/>
       <c r="R87" s="6" t="inlineStr">
         <is>
-          <t>Some reports</t>
-        </is>
-      </c>
-      <c r="S87" s="3" t="inlineStr"/>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S87" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T87" s="3" t="inlineStr"/>
       <c r="U87" s="3" t="inlineStr"/>
     </row>
@@ -7554,25 +8452,81 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D88" s="3" t="inlineStr"/>
-      <c r="E88" s="3" t="inlineStr"/>
-      <c r="F88" s="3" t="inlineStr"/>
-      <c r="G88" s="3" t="inlineStr"/>
-      <c r="H88" s="3" t="inlineStr"/>
-      <c r="I88" s="3" t="inlineStr"/>
-      <c r="J88" s="3" t="inlineStr"/>
-      <c r="K88" s="3" t="inlineStr"/>
-      <c r="L88" s="3" t="inlineStr"/>
-      <c r="M88" s="3" t="inlineStr"/>
-      <c r="N88" s="3" t="inlineStr"/>
-      <c r="O88" s="3" t="inlineStr"/>
-      <c r="P88" s="3" t="inlineStr"/>
+          <t>KIMS Saveera Hospital</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 37,913); not researched.</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="n">
+        <v>37913</v>
+      </c>
+      <c r="J88" s="3" t="n">
+        <v>29579</v>
+      </c>
+      <c r="K88" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L88" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M88" s="3" t="inlineStr">
+        <is>
+          <t>₹60,000</t>
+        </is>
+      </c>
+      <c r="N88" s="6" t="inlineStr">
+        <is>
+          <t>Medium exposure (official: Cardiac)</t>
+        </is>
+      </c>
+      <c r="O88" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: Cardiac</t>
+        </is>
+      </c>
+      <c r="P88" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q88" s="3" t="inlineStr"/>
-      <c r="R88" s="3" t="inlineStr"/>
-      <c r="S88" s="3" t="inlineStr"/>
+      <c r="R88" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S88" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T88" s="3" t="inlineStr"/>
       <c r="U88" s="3" t="inlineStr"/>
     </row>
@@ -7589,25 +8543,81 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr"/>
-      <c r="E89" s="3" t="inlineStr"/>
-      <c r="F89" s="3" t="inlineStr"/>
-      <c r="G89" s="3" t="inlineStr"/>
-      <c r="H89" s="3" t="inlineStr"/>
-      <c r="I89" s="3" t="inlineStr"/>
-      <c r="J89" s="3" t="inlineStr"/>
-      <c r="K89" s="3" t="inlineStr"/>
-      <c r="L89" s="3" t="inlineStr"/>
-      <c r="M89" s="3" t="inlineStr"/>
-      <c r="N89" s="3" t="inlineStr"/>
-      <c r="O89" s="3" t="inlineStr"/>
-      <c r="P89" s="3" t="inlineStr"/>
+          <t>Seven Hills Hospital</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 36,925); not researched.</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>36925</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>28991</v>
+      </c>
+      <c r="K89" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>₹60,823</t>
+        </is>
+      </c>
+      <c r="N89" s="6" t="inlineStr">
+        <is>
+          <t>Medium exposure (official: Cardiac, Neuro)</t>
+        </is>
+      </c>
+      <c r="O89" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: Cardiac, Neuro</t>
+        </is>
+      </c>
+      <c r="P89" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q89" s="3" t="inlineStr"/>
-      <c r="R89" s="3" t="inlineStr"/>
-      <c r="S89" s="3" t="inlineStr"/>
+      <c r="R89" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S89" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T89" s="3" t="inlineStr"/>
       <c r="U89" s="3" t="inlineStr"/>
     </row>
@@ -7689,12 +8699,16 @@
         </is>
       </c>
       <c r="Q90" s="3" t="inlineStr"/>
-      <c r="R90" s="7" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="S90" s="3" t="inlineStr"/>
+      <c r="R90" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S90" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T90" s="3" t="inlineStr"/>
       <c r="U90" s="3" t="inlineStr"/>
     </row>
@@ -7711,25 +8725,81 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>not in app data (no 2024–25 allotment near your rank)</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="inlineStr"/>
-      <c r="E91" s="3" t="inlineStr"/>
-      <c r="F91" s="3" t="inlineStr"/>
-      <c r="G91" s="3" t="inlineStr"/>
-      <c r="H91" s="3" t="inlineStr"/>
-      <c r="I91" s="3" t="inlineStr"/>
-      <c r="J91" s="3" t="inlineStr"/>
-      <c r="K91" s="3" t="inlineStr"/>
-      <c r="L91" s="3" t="inlineStr"/>
-      <c r="M91" s="3" t="inlineStr"/>
-      <c r="N91" s="3" t="inlineStr"/>
-      <c r="O91" s="3" t="inlineStr"/>
-      <c r="P91" s="3" t="inlineStr"/>
+          <t>Lalitha Super Specialty Hospital</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Private hospital · DNB</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>Leave out</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>Not reachable at your AIR (2025 closing 37,019); not researched.</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>Unlikely</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="n">
+        <v>37019</v>
+      </c>
+      <c r="J91" s="3" t="n">
+        <v>29626</v>
+      </c>
+      <c r="K91" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L91" s="3" t="inlineStr">
+        <is>
+          <t>None (NBEMS rule)</t>
+        </is>
+      </c>
+      <c r="M91" s="3" t="inlineStr">
+        <is>
+          <t>₹60,900</t>
+        </is>
+      </c>
+      <c r="N91" s="6" t="inlineStr">
+        <is>
+          <t>Medium exposure (official: Cardiac, Neuro)</t>
+        </is>
+      </c>
+      <c r="O91" s="3" t="inlineStr">
+        <is>
+          <t>Official courses: Cardiac, Neuro</t>
+        </is>
+      </c>
+      <c r="P91" s="7" t="inlineStr">
+        <is>
+          <t>Unknown — ask</t>
+        </is>
+      </c>
       <c r="Q91" s="3" t="inlineStr"/>
-      <c r="R91" s="3" t="inlineStr"/>
-      <c r="S91" s="3" t="inlineStr"/>
+      <c r="R91" s="6" t="inlineStr">
+        <is>
+          <t>Nothing adverse online</t>
+        </is>
+      </c>
+      <c r="S91" s="3" t="inlineStr">
+        <is>
+          <t>Nothing adverse found online</t>
+        </is>
+      </c>
       <c r="T91" s="3" t="inlineStr"/>
       <c r="U91" s="3" t="inlineStr"/>
     </row>
@@ -7764,7 +8834,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Verdict: Join / Join after checks / Backup only / Avoid — from official data + web/resident research on her 5 priorities.</t>
+          <t>Verdict: Join / Backup only / Avoid — a decision, not a hedge; the "Confirm before locking" questions still live in the app drawer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore 'Put high' for Join verdicts after removing the hedged verdict
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -1529,9 +1529,9 @@
           <t>Join</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Backup only</t>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Put high</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -3019,9 +3019,9 @@
           <t>Join</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>Backup only</t>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Put high</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -4991,9 +4991,9 @@
           <t>Join</t>
         </is>
       </c>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>Backup only</t>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Put high</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -7549,9 +7549,9 @@
           <t>Join</t>
         </is>
       </c>
-      <c r="F78" s="8" t="inlineStr">
-        <is>
-          <t>Backup only</t>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Put high</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -7919,9 +7919,9 @@
           <t>Join</t>
         </is>
       </c>
-      <c r="F82" s="8" t="inlineStr">
-        <is>
-          <t>Backup only</t>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Put high</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Shortlist: verdicts + resident research for the 13 added hospitals — every sheet college now has a verdict
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -3692,9 +3692,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 37,887); not researched.</t>
+          <t>Established Ludhiana teaching hospital with cardiac, paeds cardiac, neuro, transplant and a large ICU.</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
@@ -3743,12 +3743,16 @@
           <t>Official courses: Critical care, Cardiac, Neuro, GI surgery</t>
         </is>
       </c>
-      <c r="P36" s="4" t="inlineStr">
-        <is>
-          <t>Dept page only</t>
-        </is>
-      </c>
-      <c r="Q36" s="3" t="inlineStr"/>
+      <c r="P36" s="6" t="inlineStr">
+        <is>
+          <t>Good (reported)</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>No resident account, but SPS has the largest anaesthesia cohort in this list - DNB Anaesthesia 4 post-MBBS + 4 post-diploma seats, plus DrNB Critical Care (2), DrNB Neurology, IDCCM/IFCCM and emergency-medicine fellowships - and its academics page names the four current anaesthesia trainees. 350-bed NABH hospital with cardiology, neurosciences and critical care. Meducate has no review text for it.</t>
+        </is>
+      </c>
       <c r="R36" s="7" t="inlineStr">
         <is>
           <t>Nothing adverse online</t>
@@ -3878,9 +3882,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -3890,7 +3894,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 36,932); not researched.</t>
+          <t>Running DNB programme with named faculty, but oncology is the only proven super-speciality.</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
@@ -3931,10 +3935,14 @@
       </c>
       <c r="P38" s="4" t="inlineStr">
         <is>
-          <t>Dept page only</t>
-        </is>
-      </c>
-      <c r="Q38" s="3" t="inlineStr"/>
+          <t>Some reports (weak)</t>
+        </is>
+      </c>
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>Two named DNB anaesthesia residents (Dr Gokkulavani T, Dr Gazi Mahveen Tasaduq) give testimonials on the hospital's own academic site: 'hands-on experience and interactive discussions... exposed to a wide range of cases... regular academic sessions and workshops'. These are hospital-curated and near-identical in wording, so weak as independent evidence, but they confirm anaesthesia residents are in place (2 per intake per the DNB trainee list). 300-bed hospital (Meducate) with orthopaedics, oncology (radiation oncology DNB), respiratory medicine and radiology programmes.</t>
+        </is>
+      </c>
       <c r="R38" s="4" t="inlineStr">
         <is>
           <t>Concerns reported</t>
@@ -3969,9 +3977,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -3981,7 +3989,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 37,505); not researched.</t>
+          <t>Small Fortis unit that lists cardiac and transplant surgery, but nothing is known about its anaesthesia training.</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
@@ -4022,10 +4030,14 @@
       </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>Dept page only</t>
-        </is>
-      </c>
-      <c r="Q39" s="3" t="inlineStr"/>
+          <t>Some reports (weak)</t>
+        </is>
+      </c>
+      <c r="Q39" s="3" t="inlineStr">
+        <is>
+          <t>No Ludhiana-specific resident account. Fortis Ludhiana is a small unit (175 beds per Meducate; 2 DNB specialities, 6 seats per formity) with cardiac sciences, neurosciences, oncology and an 8-bed NICU. The Fortis group DNB page promises supervised hands-on work, journal clubs, audits and mock tests, generically. The only Fortis DNB-resident voices (AmbitionBox, 2 reviews, Mohali and Bengaluru, 2022) say 'good exposure, variety of cases' and 'good infrastructure... only few people have powers rather than a system'.</t>
+        </is>
+      </c>
       <c r="R39" s="7" t="inlineStr">
         <is>
           <t>Nothing adverse online</t>
@@ -4810,9 +4822,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -4822,7 +4834,7 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 36,827); not researched.</t>
+          <t>Mid-size Narayana unit in Raipur; super-speciality claims are unsupported chain template text.</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
@@ -4861,12 +4873,16 @@
           <t>Official courses: Neuro, Critical care</t>
         </is>
       </c>
-      <c r="P48" s="8" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="Q48" s="3" t="inlineStr"/>
+      <c r="P48" s="4" t="inlineStr">
+        <is>
+          <t>Some reports (weak)</t>
+        </is>
+      </c>
+      <c r="Q48" s="3" t="inlineStr">
+        <is>
+          <t>No resident account (neetlogiq empty, AmbitionBox has no Narayana DNB-resident reviews, no Reddit hit). Officially a Narayana Health unit since 2011 with cardiac sciences, cancer (LINAC), neurosciences, robotic surgery, solid-organ and bone-marrow transplant, ECMO and cath lab - but only '105+ advanced care beds' / 265 beds (Meducate) and 70+ consultants, so it is a mid-size tertiary unit. Do not confuse with Shree Narayana Hospital, Raipur (a different DNB hospital).</t>
+        </is>
+      </c>
       <c r="R48" s="7" t="inlineStr">
         <is>
           <t>Nothing adverse online</t>
@@ -6812,9 +6828,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Avoid</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
@@ -6824,7 +6840,7 @@
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 36,668); not researched.</t>
+          <t>Declared stipend ₹35,000 is below the NBEMS minimum, and hands-on is described as limited.</t>
         </is>
       </c>
       <c r="H70" s="5" t="inlineStr">
@@ -6863,12 +6879,16 @@
           <t>Site lists: neurosurgery (unit doctor: MCh Neurosurgery), nephrology/urology (unit doctor: MCh Urology), GI surgery (unit doctor: MCh GI Surgery), cardiac sciences (unit doctor listed), interventional radiology (unit doctor: FNVIR), medical gastroenterology, rheumatology, NICU/PICU (listed under procedures)</t>
         </is>
       </c>
-      <c r="P70" s="8" t="inlineStr">
-        <is>
-          <t>Unknown — ask</t>
-        </is>
-      </c>
-      <c r="Q70" s="3" t="inlineStr"/>
+      <c r="P70" s="5" t="inlineStr">
+        <is>
+          <t>Observation-heavy</t>
+        </is>
+      </c>
+      <c r="Q70" s="3" t="inlineStr">
+        <is>
+          <t>The one non-templated review text in this set: Meducate's highlights for Apollo Madurai say 'DNB students get access to advanced clinical scenarios, particularly in oncology and critical care. Academics are well-structured. Surgical hands-on is consultant-led and sometimes limited. Ideal for residents focused on academics and sub-specialty exposure.' Unsigned, so weak, but it is the only explicit statement on hands-on limits found for any of these hospitals. 300-bed Apollo unit (est. 1997) with cardiac sciences, neurosciences, oncology, transplant and interventional radiology; 4 DNB specialities, 12 seats.</t>
+        </is>
+      </c>
       <c r="R70" s="7" t="inlineStr">
         <is>
           <t>Nothing adverse online</t>
@@ -6903,9 +6923,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
@@ -6915,7 +6935,7 @@
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 36,823); not researched.</t>
+          <t>Chennai hospital with official cardiac anaesthesia and surgical gastro programmes, so the cardiac and GI work is real.</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr">
@@ -6954,10 +6974,14 @@
       </c>
       <c r="P71" s="4" t="inlineStr">
         <is>
-          <t>Dept page only</t>
-        </is>
-      </c>
-      <c r="Q71" s="3" t="inlineStr"/>
+          <t>Some reports (weak)</t>
+        </is>
+      </c>
+      <c r="Q71" s="3" t="inlineStr">
+        <is>
+          <t>No resident account; Meducate has no page. Billroth (Shenoy Nagar) is a 330-bed Chennai hospital (NeetVantage) advertising a multi-organ transplant institute (heart, liver, lung, kidney, hand), cardiac surgery, neurosurgery and critical care; only 2 DNB courses here (anaesthesia, radiology). AmbitionBox has 9 'Duty Medical Officer' reviews - the closest thing to a junior-doctor voice - split between 'skills development' and 'simply waste / management'.</t>
+        </is>
+      </c>
       <c r="R71" s="7" t="inlineStr">
         <is>
           <t>Nothing adverse online</t>
@@ -6992,9 +7016,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E72" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
@@ -7004,7 +7028,7 @@
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 37,022); not researched.</t>
+          <t>Older Coimbatore hospital with a cardiac anaesthesia course, but thin anaesthesia faculty and moderate volume.</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -7043,10 +7067,14 @@
       </c>
       <c r="P72" s="4" t="inlineStr">
         <is>
-          <t>Dept page only</t>
-        </is>
-      </c>
-      <c r="Q72" s="3" t="inlineStr"/>
+          <t>Some reports (weak)</t>
+        </is>
+      </c>
+      <c r="Q72" s="3" t="inlineStr">
+        <is>
+          <t>No resident account, but two non-templated hints: Meducate's highlights say 'Moderate patient volume... Academics present but not highly structured. Hands-on procedural work is possible but depends on initiative. Suitable for those wanting to train in a smaller hospital environment', and an AmbitionBox DMO (Jan 2024) calls it 'a great training ground... working in all departments'. Officially 425 beds, 10,000 surgeries/yr, cath lab, renal transplant centre, MICU/CCU; no cardiac surgery or neurosurgery programme is listed.</t>
+        </is>
+      </c>
       <c r="R72" s="7" t="inlineStr">
         <is>
           <t>Nothing adverse online</t>
@@ -8011,9 +8039,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E83" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
@@ -8023,7 +8051,7 @@
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 37,321); not researched.</t>
+          <t>Well-equipped Rourkela tertiary centre with neuro, cardiac, trauma and big ICUs, plus the highest stipend here.</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr">
@@ -8062,12 +8090,16 @@
           <t>Official courses: Neuro, Critical care</t>
         </is>
       </c>
-      <c r="P83" s="4" t="inlineStr">
-        <is>
-          <t>Dept page only</t>
-        </is>
-      </c>
-      <c r="Q83" s="3" t="inlineStr"/>
+      <c r="P83" s="6" t="inlineStr">
+        <is>
+          <t>Good (reported)</t>
+        </is>
+      </c>
+      <c r="Q83" s="3" t="inlineStr">
+        <is>
+          <t>The hospital publishes an NBEMS-style DNB FAQ (Aug 2026): 307 beds, NABH+NABL, 21 accredited programmes incl. DrNB Neurosurgery and DrNB Critical Care and FNB Trauma - so neuro and ICU exposure is structurally present; anaesthesia has 1 post-MBBS + 1 post-diploma seat. The hospital posts its own resident-testimonial videos ('DNB doctors share their experience', farewell batch 2026) - hospital-curated, not independent. No third-party resident account found.</t>
+        </is>
+      </c>
       <c r="R83" s="7" t="inlineStr">
         <is>
           <t>Nothing adverse online</t>
@@ -8197,9 +8229,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E85" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F85" s="5" t="inlineStr">
@@ -8209,7 +8241,7 @@
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 36,924); not researched.</t>
+          <t>Biggest hospital in this list: 700 beds, 200 ICU beds, 28 OTs, with cardiac, neuro and transplant work.</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr">
@@ -8248,10 +8280,14 @@
       </c>
       <c r="P85" s="4" t="inlineStr">
         <is>
-          <t>Dept page only</t>
-        </is>
-      </c>
-      <c r="Q85" s="3" t="inlineStr"/>
+          <t>Some reports (weak)</t>
+        </is>
+      </c>
+      <c r="Q85" s="3" t="inlineStr">
+        <is>
+          <t>Nothing from residents. The hospital is large (listings say 650-700 beds, NABH) with cath labs, 'advanced ICUs', kidney and liver transplant surgeons, neurosurgery and robotic surgeons on the roster, and 13 DNB seats across 4 specialities (formity). Its anaesthesiology page is patient-facing marketing with no training content; Meducate has no page for this unit. A LinkedIn profile of a 'DNB resident PGY1' at Medicover Vizag exists but says nothing about training.</t>
+        </is>
+      </c>
       <c r="R85" s="7" t="inlineStr">
         <is>
           <t>Nothing adverse online</t>
@@ -8286,9 +8322,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E86" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr">
@@ -8298,7 +8334,7 @@
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 35,956); not researched.</t>
+          <t>200-bed Apollo unit focused on ortho, trauma and cardiology; no proven super-speciality depth.</t>
         </is>
       </c>
       <c r="H86" s="5" t="inlineStr">
@@ -8472,9 +8508,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E88" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E88" s="6" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
@@ -8484,7 +8520,7 @@
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 37,913); not researched.</t>
+          <t>Busy KIMS hospital in Anantapur with real cardiac, neuro, transplant and trauma numbers and 10 anaesthetists.</t>
         </is>
       </c>
       <c r="H88" s="5" t="inlineStr">
@@ -8567,9 +8603,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E89" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E89" s="6" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
@@ -8579,7 +8615,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 36,925); not researched.</t>
+          <t>Official cardiac anaesthesia and neurosurgery programmes in Vizag; hospital changed owners after insolvency in 2024.</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr">
@@ -8753,9 +8789,9 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E91" s="3" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
@@ -8765,7 +8801,7 @@
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>Not reachable at your AIR (2025 closing 37,019); not researched.</t>
+          <t>Guntur DNB centre since 2008 whose anaesthesia page details transplant, neuro and cardiothoracic work.</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr">
@@ -8804,12 +8840,16 @@
           <t>Official courses: Cardiac, Neuro</t>
         </is>
       </c>
-      <c r="P91" s="4" t="inlineStr">
-        <is>
-          <t>Dept page only</t>
-        </is>
-      </c>
-      <c r="Q91" s="3" t="inlineStr"/>
+      <c r="P91" s="6" t="inlineStr">
+        <is>
+          <t>Good (reported)</t>
+        </is>
+      </c>
+      <c r="Q91" s="3" t="inlineStr">
+        <is>
+          <t>No resident account, but the department's own DNB page is unusually specific: anaesthesia for liver and kidney transplant, neurosurgery, neuro-/vascular intervention, thoracic/vascular surgery, labour analgesia and out-of-OT work, with BIS depth monitoring, LiDCO cardiac output and SVV-guided fluids in routine use; DNB running since 2008 (3 anaesthesia seats + 1 diploma). Meducate's templated blurb adds nothing resident-sourced. Lalitha opened a new 600-bed 'Lalitha PVS Institute' campus in June 2026 and says DNB training continues - which campus residents rotate through is not stated.</t>
+        </is>
+      </c>
       <c r="R91" s="7" t="inlineStr">
         <is>
           <t>Nothing adverse online</t>

</xml_diff>

<commit_message>
Toxicity rule: Join with hospital-named strike/harassment or resident 'toxic' reports -> Backup only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -5002,14 +5002,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>Join</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -7576,14 +7576,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E78" s="6" t="inlineStr">
-        <is>
-          <t>Join</t>
-        </is>
-      </c>
-      <c r="F78" s="6" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -7946,14 +7946,14 @@
           <t>Private hospital · DNB</t>
         </is>
       </c>
-      <c r="E82" s="6" t="inlineStr">
-        <is>
-          <t>Join</t>
-        </is>
-      </c>
-      <c r="F82" s="6" t="inlineStr">
-        <is>
-          <t>Put high</t>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Backup only</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Labels: 'Missing' instead of 'Unknown — ask'
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -762,7 +762,7 @@
       </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr"/>
@@ -843,13 +843,13 @@
       </c>
       <c r="N4" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr"/>
       <c r="P4" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr"/>
@@ -928,13 +928,13 @@
       </c>
       <c r="N5" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr"/>
       <c r="P5" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr"/>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr"/>
@@ -1104,13 +1104,13 @@
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr"/>
       <c r="P7" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr"/>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="P8" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr"/>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr"/>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr"/>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr"/>
@@ -1736,7 +1736,7 @@
       <c r="J14" s="3" t="inlineStr"/>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr"/>
@@ -1757,7 +1757,7 @@
       </c>
       <c r="P14" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr"/>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr"/>
@@ -2026,13 +2026,13 @@
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr"/>
       <c r="P17" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr"/>
@@ -2210,13 +2210,13 @@
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr"/>
       <c r="P19" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr"/>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
       <c r="Q25" s="3" t="inlineStr"/>
       <c r="R25" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr">
@@ -2970,13 +2970,13 @@
       </c>
       <c r="N27" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr"/>
       <c r="P27" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr"/>
@@ -3148,13 +3148,13 @@
       </c>
       <c r="N29" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="O29" s="3" t="inlineStr"/>
       <c r="P29" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr"/>
@@ -3245,7 +3245,7 @@
       </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr"/>
@@ -3334,7 +3334,7 @@
       </c>
       <c r="P31" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr"/>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="P44" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q44" s="3" t="inlineStr"/>
@@ -4943,7 +4943,7 @@
       <c r="J49" s="3" t="inlineStr"/>
       <c r="K49" s="8" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr"/>
@@ -5307,7 +5307,7 @@
       </c>
       <c r="K53" s="8" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr"/>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="P53" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q53" s="3" t="inlineStr"/>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="P54" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q54" s="3" t="inlineStr"/>
@@ -5510,7 +5510,7 @@
       </c>
       <c r="P55" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q55" s="3" t="inlineStr"/>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="P56" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q56" s="3" t="inlineStr"/>
@@ -5692,7 +5692,7 @@
       </c>
       <c r="P57" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q57" s="3" t="inlineStr"/>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="P58" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q58" s="3" t="inlineStr"/>
@@ -5864,13 +5864,13 @@
       </c>
       <c r="N59" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="O59" s="3" t="inlineStr"/>
       <c r="P59" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q59" s="3" t="inlineStr"/>
@@ -5965,7 +5965,7 @@
       </c>
       <c r="P60" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q60" s="3" t="inlineStr"/>
@@ -6029,7 +6029,7 @@
       <c r="J61" s="3" t="inlineStr"/>
       <c r="K61" s="8" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="L61" s="3" t="inlineStr"/>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="P62" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q62" s="3" t="inlineStr"/>
@@ -6234,7 +6234,7 @@
       </c>
       <c r="P63" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q63" s="3" t="inlineStr"/>
@@ -6604,7 +6604,7 @@
       </c>
       <c r="P67" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q67" s="3" t="inlineStr"/>
@@ -6695,7 +6695,7 @@
       </c>
       <c r="P68" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q68" s="3" t="inlineStr"/>
@@ -6786,7 +6786,7 @@
       </c>
       <c r="P69" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q69" s="3" t="inlineStr"/>
@@ -8751,7 +8751,7 @@
       </c>
       <c r="P90" s="8" t="inlineStr">
         <is>
-          <t>Unknown — ask</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="Q90" s="3" t="inlineStr"/>
@@ -8915,7 +8915,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Labels: green = good, blue = acceptable, amber = caution, red = problem, grey "Unknown — ask" = nothing verified online (only seniors can answer).</t>
+          <t>Labels: green = good, blue = acceptable, amber = caution, red = problem, grey "Missing" = nothing verified online.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
JLN Bhilai (SAIL) is a public-sector DNB hospital, not private: OBC quota applies, bond not verified
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -4581,7 +4581,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Private hospital · DNB</t>
+          <t>Government hospital · DNB</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -4610,16 +4610,12 @@
       <c r="J45" s="2" t="n">
         <v>27369</v>
       </c>
-      <c r="K45" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>None (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
           <t>₹53,550</t>

</xml_diff>

<commit_message>
Shortlist: Show more / full details toggle, research notes rewritten in plain English, labels match their text
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -896,7 +896,7 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse found online; aggregator lists DNB stipend Rs 15,000/mo (2025 MCC data)</t>
+          <t>Nothing bad found. One review site says the stipend is ₹15,000/month, but the hospital told MCC ₹43,000. (review site)</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr"/>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
@@ -1241,17 +1241,17 @@
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>Caution — strike / harassment reported</t>
+          <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>No suicide/strike found; 2017 NBE complaint: inhuman DNB duty hours (radiology); 2025 forum: meagre stipend ~50k</t>
+          <t>No suicide or strike found. 2017: complaint to the DNB board about inhuman duty hours (radiology). 2025: a resident called the ~₹50k stipend low. (news + resident post)</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>32 h/56 h stretches (radiology, 2017 complaint); WLB 5/5 (2025) [forum]</t>
+          <t>A 2017 complaint said radiology residents worked 32–56 hours at a stretch. A 2025 resident rated work-life balance 5 out of 5. No anaesthesia-specific info. (complaint + review site)</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr"/>
@@ -1334,19 +1334,19 @@
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="4" t="inlineStr">
-        <is>
-          <t>Red flag — a death reported</t>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse 2019-26; radiology PG murdered in hospital duty room (Aug 2017, news)</t>
+          <t>Nothing bad found for 2019–26. 2017: a radiology PG was murdered in the hospital duty room. (news)</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>Regular OT days + 6-9 emergency duties/month, weekly OT rotation [forum, 2021]</t>
+          <t>Normal OT days plus 6–9 emergency duties a month; OT changes every week. (one anaesthesia resident, 2021)</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr"/>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse re residents; Delhi govt ordered action after probe flagged patient-care lapses (Jun 2026)</t>
+          <t>Nothing bad found about residents. June 2026: Delhi govt ordered action after finding patient-care lapses. (news)</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr"/>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse found online (GMERS-wide JR pay cut 2023; Gotri stipend strike)</t>
+          <t>Nothing about this hospital itself. GMERS colleges cut junior-doctor pay in 2023 and had a stipend strike at another GMERS college. (news)</t>
         </is>
       </c>
       <c r="T13" s="2" t="inlineStr"/>
@@ -1792,13 +1792,13 @@
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse found online (Jodhpur hits are AIIMS/SNMC, not Medipulse)</t>
+          <t>Nothing bad found about this hospital. (Jodhpur news was about AIIMS and SN Medical College.)</t>
         </is>
       </c>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>Structured critical-care rotations; no duration given [official]</t>
+          <t>Hospital says PGs do planned critical-care rotations. Length not stated. (hospital website)</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse found online (Jaipur hits are SMS/AIIMS Jodhpur, Rajasthan-wide strike Oct 2024)</t>
+          <t>Nothing bad found about this hospital. (Jaipur news about strikes and suicides was about other colleges.)</t>
         </is>
       </c>
       <c r="T15" s="2" t="inlineStr"/>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse found online (Bikaner suicides were SP Medical College interns/residents, not Kothari)</t>
+          <t>Nothing bad found about this hospital. (Bikaner suicide news was about SP Medical College, not Kothari.)</t>
         </is>
       </c>
       <c r="T16" s="2" t="inlineStr"/>
@@ -2071,7 +2071,7 @@
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>25-bed ICU; dept trains anaesthesia+critical care together; no rota [official]</t>
+          <t>25-bed ICU; anaesthesia and critical-care trainees are trained together. Posting length not stated. (hospital website)</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse found online (Lucknow hits are KGMU, not Max/Sahara)</t>
+          <t>Nothing bad found about this hospital. (Lucknow news was about KGMU.)</t>
         </is>
       </c>
       <c r="T18" s="2" t="inlineStr"/>
@@ -2251,7 +2251,7 @@
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>ICU/critical-care rotations 'strong exposure'; no duration [forum]</t>
+          <t>Review says ICU exposure is 'strong'. Posting length not stated. (review site)</t>
         </is>
       </c>
     </row>
@@ -2344,13 +2344,13 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse found online (Greater Noida trainee suicide Sept 2025 not linked to Kailash)</t>
+          <t>Nothing bad found about this hospital. (A Sept 2025 trainee suicide in Greater Noida was at another place.)</t>
         </is>
       </c>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>ICU/critical-care exposure 'decent', cardiac+neuro ICU; no duration [forum]</t>
+          <t>Review says ICU exposure is 'decent', with cardiac and neuro ICUs. Posting length not stated. (review site)</t>
         </is>
       </c>
     </row>
@@ -2428,7 +2428,7 @@
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
@@ -2443,17 +2443,17 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse found online; 2022 resident: 'dept very chill', no bond</t>
+          <t>Nothing bad found. A 2022 resident called the department 'very chill'.</t>
         </is>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>8 h/day, 'compulsory rest choice' [forum, 2022]</t>
+          <t>About 8 hours a day; residents get rest after duty. (one resident review, 2022)</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>Dept runs 3 ICUs (Med/Surg/CCU), 60 L4 beds; no rota [official]</t>
+          <t>Anaesthesia runs 3 ICUs (medical, surgical, cardiac) with 60 beds. Posting length not stated. (hospital website)</t>
         </is>
       </c>
     </row>
@@ -2711,14 +2711,14 @@
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="7" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
+      <c r="R24" s="6" t="inlineStr">
+        <is>
+          <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>No resident incident found; consultant urologist suicide at sister college HIMS (Sept 2026, news)</t>
+          <t>Nothing about residents. Sep 2026: a consultant at its sister medical college died by suicide. (news)</t>
         </is>
       </c>
       <c r="T24" s="2" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr">
@@ -2814,7 +2814,7 @@
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>'structured working hours, balanced residency' (aggregator, no number) [snippet]</t>
+          <t>A review site says 'structured working hours'. No actual numbers. (review site)</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="P27" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr">
@@ -3063,12 +3063,12 @@
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="3" t="inlineStr">
         <is>
-          <t>Caution — strike / harassment reported</t>
+          <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>PG stipend strike (Apr 2026, 3 months unpaid); MP-wide JUDA strike (Mar 2026)</t>
+          <t>April 2026: about 175 PG residents went on strike — stipend not paid for 3 months. Also a state-wide junior doctors' strike in March 2026. (news)</t>
         </is>
       </c>
       <c r="T28" s="2" t="inlineStr"/>
@@ -3239,17 +3239,17 @@
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="6" t="inlineStr">
         <is>
-          <t>Unclear — some reports, read the text</t>
+          <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>Nothing hospital-specific; HP-wide resident strike (Dec 2025, IGMC termination)</t>
+          <t>Nothing about this college itself. All Himachal residents went on strike in Dec 2025 after a doctor was sacked at IGMC Shimla. (news)</t>
         </is>
       </c>
       <c r="T30" s="2" t="inlineStr">
         <is>
-          <t>Emergency duty 2-4 days/mo (roster Apr 2024) [official]; HP 12 h/shift cap</t>
+          <t>2–4 emergency duties a month per resident (official duty roster, 2024). State rule since Dec 2025: max 12 hours per shift.</t>
         </is>
       </c>
       <c r="U30" s="2" t="inlineStr"/>
@@ -3332,17 +3332,17 @@
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="6" t="inlineStr">
         <is>
-          <t>Unclear — some reports, read the text</t>
+          <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>Nothing hospital-specific; HP-wide resident strike (Dec 2025, IGMC termination)</t>
+          <t>Nothing about this college itself. All Himachal residents went on strike in Dec 2025 after a doctor was sacked at IGMC Shimla. (news)</t>
         </is>
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>HP policy: 12 h/shift cap for residents (Dec 2025) [news]; no local roster</t>
+          <t>State rule since Dec 2025: residents work max 12 hours per shift. No hospital roster found. (news)</t>
         </is>
       </c>
       <c r="U31" s="2" t="inlineStr"/>
@@ -3380,7 +3380,7 @@
       <c r="R32" s="2" t="inlineStr"/>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse found online (resident-level); UMC negligence fine Rs 10L 2025 (patient case)</t>
+          <t>Nothing bad found about residents. Hospital was fined ₹10 lakh in 2025 for a patient-care case (news).</t>
         </is>
       </c>
       <c r="T32" s="2" t="inlineStr"/>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="P36" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="P37" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr">
@@ -3826,14 +3826,14 @@
           <t>Two named DNB anaesthesia residents (Dr Gokkulavani T, Dr Gazi Mahveen Tasaduq) give testimonials on the hospital's own academic site: 'hands-on experience and interactive discussions... exposed to a wide range of cases... regular academic sessions and workshops'. These are hospital-curated and near-identical in wording, so weak as independent evidence, but they confirm anaesthesia residents are in place (2 per intake per the DNB trainee list). 300-bed hospital (Meducate) with orthopaedics, oncology (radiation oncology DNB), respiratory medicine and radiology programmes.</t>
         </is>
       </c>
-      <c r="R37" s="3" t="inlineStr">
-        <is>
-          <t>Caution — strike / harassment reported</t>
+      <c r="R37" s="6" t="inlineStr">
+        <is>
+          <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse 2019-26; historical: 2007 DNB admit during lapsed accreditation, Rs 5L compensation (NCDRC 2018)</t>
+          <t>Nothing bad found for 2019–26. Old case: in 2007 it took a DNB resident while its accreditation had lapsed; court ordered ₹5 lakh compensation in 2018. (court record)</t>
         </is>
       </c>
       <c r="T37" s="2" t="inlineStr"/>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="P38" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
@@ -4002,7 +4002,7 @@
       </c>
       <c r="P39" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr">
@@ -4019,7 +4019,7 @@
       <c r="T39" s="2" t="inlineStr"/>
       <c r="U39" s="2" t="inlineStr">
         <is>
-          <t>ICU rotation listed (RICU/CCU/Neuro/Septic ICU), no duration [official]</t>
+          <t>PGs rotate through several ICUs (respiratory, cardiac, neuro, septic). How long is not stated. (hospital website)</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr">
@@ -4196,14 +4196,14 @@
           <t>Ivy Amritsar has been rebranded Livasa Hospital. The group's academic page (official) says it is NBE-recognised for DNB Anaesthesiology, Radiodiagnosis and Cardiology and names three DNB-qualified anaesthesia faculty (Dr Rajiv Dhunna - also programme director for DrNB critical care per LinkedIn - Dr Shalini S, Dr Sunny Rupal), though the page text refers to 'Livasa Hospital, Mohali' so unit-level detail is unclear. 180 beds (aggregator). No resident account found.</t>
         </is>
       </c>
-      <c r="R41" s="3" t="inlineStr">
-        <is>
-          <t>Unclear — just one anonymous post</t>
+      <c r="R41" s="6" t="inlineStr">
+        <is>
+          <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t>No resident item; staff reviews allege unpaid salary/F&amp;F (2020-21), 'no job security' (3.0/5, 31 reviews)</t>
+          <t>Nothing about residents. Staff reviews (2020–21) complain of unpaid salary and no job security. (job-review site)</t>
         </is>
       </c>
       <c r="T41" s="2" t="inlineStr"/>
@@ -4374,12 +4374,12 @@
       <c r="Q43" s="2" t="inlineStr"/>
       <c r="R43" s="3" t="inlineStr">
         <is>
-          <t>Caution — strike / harassment reported</t>
+          <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="S43" s="2" t="inlineStr">
         <is>
-          <t>PCMSA doctors' strike (Sep 2024); 3 patient deaths, anaesthetist+SMO suspended (Jul 2025); no PG-specific item</t>
+          <t>Sep 2024: government doctors' strike shut the OPD. July 2025: 3 patients died after an oxygen fault; an anaesthetist was suspended. Nothing about PGs. (news)</t>
         </is>
       </c>
       <c r="T43" s="2" t="inlineStr"/>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="P44" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q44" s="2" t="inlineStr">
@@ -4558,12 +4558,12 @@
       <c r="S45" s="2" t="inlineStr"/>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t>OT 8am-2pm; 3-4 x 18 h night calls/month (yr1-2), 4-5 x 8 h (yr3) [forum]</t>
+          <t>OT 8 am–2 pm. 1st–2nd year: 3–4 night calls a month, 18 hours each. 3rd year: 4–5 calls of 8 hours. (one resident, 2021)</t>
         </is>
       </c>
       <c r="U45" s="2" t="inlineStr">
         <is>
-          <t>2 months/yr ICU + 1 mo Raipur GMC SS + 1 mo cardiac OT (2021) [forum]</t>
+          <t>2 months a year in ICU, plus 1 month at Raipur medical college and 1 month in cardiac OT. (one resident, 2021)</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="P47" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q47" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="S48" s="2" t="inlineStr">
         <is>
-          <t>1 MBBS student suicide (Aug 2025, not PG); intern+PG stipend strike (Aug 2026); JDA OPD boycott (Sep 2026)</t>
+          <t>Aug 2026: interns and PGs struck over unpaid stipend. Sep 2026: junior doctors threatened to stop OPD. Aug 2025: an MBBS student (not a PG) died by suicide. (news)</t>
         </is>
       </c>
       <c r="T48" s="2" t="inlineStr"/>
@@ -4910,14 +4910,14 @@
           <t>Official DNB page: 983-bed NABH hospital, 76 critical-care/ICU beds plus separate cardiac CCU, PICU, NICU and burns unit, 13 modular OTs with a PACU, and 'academic rotations in superspecialities' incl. cardiology, critical care, neurosurgery, neuroanaesthesia, onco-surgery, plastic and paediatric surgery; anaesthesia DNB since 1999 (2 primary + 2 secondary seats/yr), FNB critical care since 2013, interventional pain procedures in the main OT. Resident evidence is mixed: AmbitionBox DNB residents (3 reviews, 4.8/5) praise an 'excellent academic environment and work culture', while a DNB-medicine forum post says first-year residents do 'all the clerical work and blood sampling which isn't the case with other DNB institutes'.</t>
         </is>
       </c>
-      <c r="R49" s="5" t="inlineStr">
-        <is>
-          <t>Good — residents report sane hours</t>
+      <c r="R49" s="3" t="inlineStr">
+        <is>
+          <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="S49" s="2" t="inlineStr">
         <is>
-          <t>JR reviews: 'toxic environment, poor work-life balance, manpower crisis' (2023/25); MTMC MBBS suicide (Aug 2025)</t>
+          <t>Junior doctors' reviews (2023, 2025) say 'toxic environment, poor work-life balance, too few staff'. A student at the linked medical college died by suicide in Aug 2025. (job-review site + news)</t>
         </is>
       </c>
       <c r="T49" s="2" t="inlineStr"/>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="S52" s="2" t="inlineStr">
         <is>
-          <t>1 DNB resident suicide (1st-yr OBGYN, Mar 2025; note cited course dissatisfaction)</t>
+          <t>March 2025: a 1st-year DNB resident (Obs &amp; Gynae) died by suicide in the hostel. Her note mentioned unhappiness with the course. (news)</t>
         </is>
       </c>
       <c r="T52" s="2" t="inlineStr"/>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="S53" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse for PGs found online (Apr 2025 staff-member suicide off-campus, not a resident)</t>
+          <t>Nothing bad found about PGs. April 2025: a staff member (not a resident) died by suicide off campus. (news)</t>
         </is>
       </c>
       <c r="T53" s="2" t="inlineStr"/>
@@ -5705,7 +5705,7 @@
       <c r="S58" s="2" t="inlineStr"/>
       <c r="T58" s="2" t="inlineStr">
         <is>
-          <t>8 h shifts, 6-7 nights/mo, post-night off (radiology DNB, not anaes) [forum]</t>
+          <t>8-hour shifts, 6–7 night duties a month, day off after a night — but this is from a radiology resident, not anaesthesia. (resident post)</t>
         </is>
       </c>
       <c r="U58" s="2" t="inlineStr"/>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="S60" s="2" t="inlineStr">
         <is>
-          <t>Nothing adverse for PGs found online (Jun 2025 data-entry staff salary-delay protest hit OPD, not residents)</t>
+          <t>Nothing bad found about PGs. June 2025: data-entry staff protested late salary. (news)</t>
         </is>
       </c>
       <c r="T60" s="2" t="inlineStr"/>
@@ -6219,7 +6219,7 @@
       </c>
       <c r="P64" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
@@ -6586,7 +6586,7 @@
       <c r="T68" s="2" t="inlineStr"/>
       <c r="U68" s="2" t="inlineStr">
         <is>
-          <t>Dept runs neuro/cardiac/liver-transplant ICUs; no PG posting length [official]</t>
+          <t>Department runs neuro, cardiac and liver-transplant ICUs. Posting length not stated. (hospital website)</t>
         </is>
       </c>
     </row>
@@ -6753,7 +6753,7 @@
       </c>
       <c r="P70" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q70" s="2" t="inlineStr">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="P71" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q71" s="2" t="inlineStr">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="P72" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q72" s="2" t="inlineStr">
@@ -7024,7 +7024,7 @@
       </c>
       <c r="P73" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q73" s="2" t="inlineStr">
@@ -7302,7 +7302,7 @@
       <c r="T76" s="2" t="inlineStr"/>
       <c r="U76" s="2" t="inlineStr">
         <is>
-          <t>10-bed closed ICU, 1 consultant + 1 resident round the clock [official]</t>
+          <t>10-bed ICU with 1 consultant and 1 resident on duty round the clock. Posting length not stated. (hospital website)</t>
         </is>
       </c>
     </row>
@@ -7380,7 +7380,7 @@
       </c>
       <c r="P77" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q77" s="2" t="inlineStr">
@@ -7390,12 +7390,12 @@
       </c>
       <c r="R77" s="3" t="inlineStr">
         <is>
-          <t>Caution — strike / harassment reported</t>
+          <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="S77" s="2" t="inlineStr">
         <is>
-          <t>Consultants' 2-day OPD/elective strike vs management, senior doctors 'humiliated' (Jun 2026)</t>
+          <t>June 2026: senior doctors stopped OPD and planned surgery for 2 days, saying management humiliated them. (news)</t>
         </is>
       </c>
       <c r="T77" s="2" t="inlineStr"/>
@@ -7662,7 +7662,7 @@
       </c>
       <c r="S80" s="2" t="inlineStr">
         <is>
-          <t>ICU doctor (EMO, not PG) died by suicide on duty inside ICU (Sep 2026); family cites personal harassment</t>
+          <t>Sep 2026: an ICU doctor (staff, not a PG) died by suicide on duty. Family blamed personal harassment, not the hospital. (news)</t>
         </is>
       </c>
       <c r="T80" s="2" t="inlineStr"/>
@@ -7740,7 +7740,7 @@
       </c>
       <c r="P81" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q81" s="2" t="inlineStr">
@@ -7750,12 +7750,12 @@
       </c>
       <c r="R81" s="3" t="inlineStr">
         <is>
-          <t>Caution — strike / harassment reported</t>
+          <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="S81" s="2" t="inlineStr">
         <is>
-          <t>Nurse suicide on premises (Aug 2025): staff allege senior harassment + 'heart attack' cover-up; no PG incident</t>
+          <t>Aug 2025: a nurse died by suicide at the hospital; staff alleged harassment by seniors and a cover-up. Nothing about PGs. (news)</t>
         </is>
       </c>
       <c r="T81" s="2" t="inlineStr"/>
@@ -8019,7 +8019,7 @@
       </c>
       <c r="P84" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q84" s="2" t="inlineStr">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="P85" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q85" s="2" t="inlineStr">
@@ -8296,7 +8296,7 @@
       </c>
       <c r="P87" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q87" s="2" t="inlineStr">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="P88" s="3" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="Q88" s="2" t="inlineStr">
@@ -8951,12 +8951,12 @@
       <c r="A26" s="10" t="inlineStr"/>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Unclear — just one anonymous post</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Too little to trust either way.</t>
+          <t>No one who trained there has written about it; only the hospital or review sites say anything. Searched: Reddit, Quora, review sites, Google.</t>
         </is>
       </c>
     </row>
@@ -9007,12 +9007,12 @@
       <c r="A30" s="10" t="inlineStr"/>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Caution — strike / harassment reported</t>
+          <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>A strike, harassment complaint or resignation naming the hospital (see detail).</t>
+          <t>A strike, unpaid stipend, harassment or duty-hour complaint naming the hospital (see detail).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multispeciality: plain list of departments (officially confirmed vs website claim) instead of raw notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -716,7 +716,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac</t>
+          <t>Officially confirmed: Heart.</t>
         </is>
       </c>
       <c r="P2" s="7" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Critical care</t>
+          <t>Officially confirmed: Critical care (ICU).</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, GI surgery, Critical care</t>
+          <t>Officially confirmed: Heart, Stomach &amp; liver (GI) surgery, Critical care (ICU).</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Critical care</t>
+          <t>Officially confirmed: Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Neuro, Critical care</t>
+          <t>Officially confirmed: Brain &amp; spine, Critical care (ICU).</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Onco, Cardiac, Renal/Transplant, GI surgery, Critical care</t>
+          <t>Officially confirmed: Cancer, Heart, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery, Critical care (ICU).</t>
         </is>
       </c>
       <c r="P10" s="7" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Renal/Transplant, GI surgery</t>
+          <t>Officially confirmed: Heart, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Children's surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiology/cath lab ('third generation state of the art Cath Labs'), neurosurgery (Neurology &amp; Neurosurgery), nephrology/dialysis (nephrology dept + dialysis centre), urology, oncology ('surgical and clinical expertise in treating cancer' - no separate surgical oncology dept), NICU (Pediatrics &amp; Neonatology), emergency ('24-hour emergency services'; no trauma centre stated)</t>
+          <t>Hospital website lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P12" s="7" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Site lists: broad clinical departments only: Medicine, Surgery, OBGY, Paediatrics, Orthopaedics, Ophthalmology, ENT, Dermatology, Psychiatry, Anaesthesia, Radiodiagnosis, Dentistry, Forensic, Community Medicine, no CTVS, cardiology, neurosurgery, nephrology/dialysis, urology, transplant, GI surgery, oncology, paediatric surgery, NICU/PICU, burns, trauma unit or pain clinic appears on the site, hospital 'Facilities' page lists only 'OPD, Wards, Laboratory, Pharmacy, Canteen'</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P13" s="7" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac surgery ('Cardiology &amp; Cardiac Surgery' centre of excellence; class-100 laminar-flow cardiac OT; TAVI), cardiology/cath lab (24x7 cath lab, 'Asia's 1st Artis-1' Siemens; primary PCI), neurosurgery (aneurysm clipping; Neurology &amp; Neurosurgery CoE), nephrology/dialysis (28-station dialysis unit), kidney transplant ('newly active' programme), urology (urology procedures, holmium laser), oncology (department listed; surgical oncology not separately named), NICU</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P14" s="5" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac</t>
+          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P15" s="7" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiology/cath lab ('Interventional Cardiology'; 'Advance Flat Panel Cath Lab'), neurosurgery ('Neuro &amp; Spine Surgery'), nephrology/dialysis ('6 Hemodialysis' stations), urology ('Urology &amp; Kidney Transplant' headed by an MCh urologist; TURP, PCNL, URSL listed - no transplant activity documented), trauma/emergency ('24*7 Emergency &amp; Trauma Care', '4 Emergency &amp; Trauma Beds'), pain clinic (DNB anaesthesia page: spine blocks, face blocks, intra-articular procedures, PRP, ozone, C-arm), paediatrics &amp; neonatology (no NICU beds stated), cardiac surgery - NOT working: homepage lists 'Cardiac Surgery' as coming soon; infrastructure page lists 'CTVS &amp; Neuro Modular OTs'; DNB page promised a 'Cardiac &amp; Neuro Surgery department by September 2023'</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Newborn / child ICU, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P17" s="6" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Neuro</t>
+          <t>Officially confirmed: Heart, Brain &amp; spine.</t>
         </is>
       </c>
       <c r="P19" s="6" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Critical care</t>
+          <t>Officially confirmed: Critical care (ICU).</t>
         </is>
       </c>
       <c r="P20" s="6" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac surgery/CTVS (doctor list: Dr Mohit Saxena MCh CTVS, Prof Dr Damyanti Agarwal MCh CTVS; anaesthesia page: 'Anaesthesia for Cardiac Surgery') - NOT on the specialities menu, cardiology ('Cardiology Care' page; cath lab not stated), neurosurgery (3 MS/MCh/DNB neurosurgeons on doctor list) - only 'Neurology' on the specialities menu, nephrology/dialysis ('Urology and Nephrology Unit'; 1 DNB nephrologist; dialysis not explicitly stated), urology (2 MCh urologists), kidney transplant (homepage mention 'Nephrology &amp; Urology with kidney transplant program'; no detail), surgical oncology (4 surgical oncologists incl. MCh; 'Cancer Care' + Radiation Oncology DNB), NICU and PICU ('Surgical ICU, Medical ICU, PICU, NICU, Burn ICU, CCU')</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P21" s="3" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Critical care, GI surgery</t>
+          <t>Officially confirmed: Critical care (ICU), Stomach &amp; liver (GI) surgery. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P22" s="4" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiology/cath lab (angiography, angioplasty, pacemaker, cardiac catheterisation; ICCU), cardiac surgery (CLAIMED on cardiology page: valve replacement, off-pump bypass, robotic-assisted, '10,000+ heart surgeries' - no cardiac surgeon named), neurosurgery (cranial, spinal, endoscopic brain/spine surgery listed; no surgeon named), GI surgery (surgical gastro: laparoscopic, hepatobiliary-pancreatic, colorectal, GI-oncology), paediatric surgery, surgical oncology ('Cancer Specialist' dept), NICU, PICU</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P23" s="7" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiology/cath lab ('low dose flat panel Cardiac Cath Lab'), neurosurgery (2 neurosurgeons on doctors page), nephrology/dialysis ('dialysis therapies offered'), urology (2 urologists on doctors page), surgical oncology (listed as department; no surgical oncologist on doctors page), plastic surgery &amp; burn, pain management clinic, anaesthesia (department page)</t>
+          <t>Hospital website lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Burns, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P24" s="3" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Renal/Transplant</t>
+          <t>Officially confirmed: Kidney &amp; transplant. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P25" s="3" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Neuro, Critical care</t>
+          <t>Officially confirmed: Heart, Brain &amp; spine, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
         </is>
       </c>
       <c r="P27" s="3" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Neuro</t>
+          <t>Officially confirmed: Heart, Brain &amp; spine.</t>
         </is>
       </c>
       <c r="P29" s="7" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiology (OPD-level only: one assistant professor, OPD Tue/Thu, echo Wed/Fri; no cath lab stated), trauma/emergency (Emergency Services phone line listed; no department page)</t>
+          <t>Hospital website lists: Cardiology, Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P30" s="7" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>Site lists: 22 departments listed; clinical: Medicine, Surgery, OBGY, Paediatrics, Orthopaedics, Ophthalmology, ENT, Dermatology, Psychiatry, Anaesthesiology, Radiology, Radiotherapy, TB &amp; Respiratory Diseases, Dentistry, ICU, cardiac care and paediatric care units exist within the 500 sanctioned beds (counts not given); anaesthesia dept runs its own 10-bed ICU and 13-bed PACU, nephrology/dialysis: 'a Dialysis Unit' (no nephrology department), trauma/emergency: 24-h emergency OT and maternity OT, pain clinic (acute and chronic pain referrals), no CTVS, cardiology, neurosurgery, urology, transplant, GI surgery, surgical oncology, paediatric surgery or burns unit - 'Superspeciality Departments ... in the pipeline'</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P31" s="3" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac sciences (Director + Sr Consultant; CTVS not explicitly listed), neurosurgery (Sr Consultant), urology (2 Sr Consultants), renal sciences &amp; kidney transplant (1 Sr Consultant; transplant activity at this unit not evidenced), gastro sciences (medical), cancer care (HOD + Sr Consultant), intervention radiology, critical care &amp; anaesthesiology (Head + 3 Sr Consultants) and critical care (1 Sr Consultant)</t>
+          <t>Hospital website lists: Heart surgery, Brain &amp; spine surgery, Kidney transplant, Urology, Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac sciences (procedures listed: CABG, minimally invasive cardiac surgery, ECMO, EP study, angiography), neuro sciences brain &amp; spine (neurosurgery consultant listed), renal sciences &amp; kidney transplant, gastro sciences (medical and surgical gastroenterology), cancer care (Director-level surgical oncology; nuclear medicine), critical care (7 named doctors), paediatrics and paediatric surgery, bariatric surgery</t>
+          <t>Hospital website lists: Heart surgery, Brain &amp; spine surgery, Kidney transplant, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P34" s="3" t="inlineStr">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Critical care, Cardiac, Neuro, GI surgery</t>
+          <t>Officially confirmed: Critical care (ICU), Heart, Brain &amp; spine, Stomach &amp; liver (GI) surgery. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic.</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac surgery/CTVS (Mohali page: 'Cardiac/Thoracic Surgery'; group speciality index: Cardiac Surgery, CTVS), cardiology (Mohali page; 'Interventional Cardiology' on group index), neurosurgery (Mohali page), nephrology (Mohali page), urology (Mohali page), kidney transplant ('Renal Transplant Surgery' on Mohali page), surgical oncology ('Oncology' on Mohali page; 'Surgical Oncology' on group index, not location-tagged), vascular surgery (Mohali page)</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P36" s="3" t="inlineStr">
@@ -3813,7 +3813,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Onco</t>
+          <t>Officially confirmed: Cancer. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P37" s="3" t="inlineStr">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>Official courses: GI surgery, Critical care</t>
+          <t>Officially confirmed: Stomach &amp; liver (GI) surgery, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Pain clinic.</t>
         </is>
       </c>
       <c r="P38" s="3" t="inlineStr">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiothoracic and vascular surgery (speciality page; 'CTVS surgeries' on DNB page), cardiology (CCU / ICCU), neuro &amp; spine surgery (neurosurgery; 'Neuro ICU'), nephrology, urology, surgical oncology ('onco-surgeries'), NICU, emergency &amp; trauma care 24x7</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P39" s="3" t="inlineStr">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac surgery (CTVS page: CABG, valve replacement, congenital heart repair, pericardectomy, vascular/AV-fistula, thoracic; one surgeon listed), cardiology/cath lab ('fully equipped Cardiac Cath Lab' - About page; angioplasty testimonial), neurosurgery (trauma EDH/SDH, aneurysm, minimally invasive spine, neuro-endoscopy, stroke unit; 'dedicated ICU' and 'neuro-anesthetists'), nephrology/dialysis (dialysis unit with CRRT and CAPD), urology (speciality page listed), oncology (department page listed; surgical vs medical not specified), NICU-level neonatal care (Paediatrics &amp; Neonatology: 'well equipped ICU with ventilators ... premature and full term infants'), trauma/emergency (24-hour emergency services)</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P40" s="6" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Renal/Transplant, Critical care</t>
+          <t>Officially confirmed: Heart, Kidney &amp; transplant, Critical care (ICU).</t>
         </is>
       </c>
       <c r="P41" s="3" t="inlineStr">
@@ -4278,7 +4278,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac</t>
+          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
         </is>
       </c>
       <c r="P42" s="3" t="inlineStr">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac surgery incl. paediatric ('Adult CABG and valve surgeries', 'Pediatric and congenital cardiac surgery', 'Heart failure surgery and transplantation', ECMO; 3 CTVS surgeons named), cardiology/cath lab ('equipped with Cath Labs'; Institute of Cardiac Sciences), neurosurgery (department + Institute of Neurosciences), nephrology/dialysis ('Nephrology' and 'Dialysis' departments; Institute of Nephrology and Urology), urology, oncology (Institute of Oncology + 'Oncology' dept; surgical oncology not separately named; Nuclear Medicine listed), trauma/emergency ('Emergency Medicine'), pain (anaesthesia page: 'pain medicine', 'Epidurals, Labour analgesia')</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P44" s="3" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>Site lists: [forum 2021] OTs for general surgery, obstetrics, ENT, orthopaedics, ophthalmology, plastic surgery and urosurgery, [forum 2021] 20-bed emergency/trauma unit, [forum 2021] paediatric surgery, neurosurgery and cardiac surgery are NOT on site - covered by 4 months/yr of outside postings at affiliated centres</t>
+          <t>Hospital website lists: Heart surgery, Brain &amp; spine surgery, Children's surgery, Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P45" s="3" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiology/cath lab (cath lab listed with the OTs; Cardiology department), neurosurgery ('Neuro Surgery' on specialities page) and neurology, urology and oncology (specialities list), nephrology: dialysis unit only (no nephrology department named), trauma/emergency ('Traumatology' department; '4 bedded Emergency with 2 bedded Observation'; ACLS ambulance), ICU types named: 'ICU (Medical/ Surgical/ Cardiac/ Burns/ Neonatal)' - no bed counts, paediatrics; blood &amp; component bank (only one in region); apheresis unit, 'Anaesthesiology &amp; Intensive Care Unit' listed as a speciality</t>
+          <t>Hospital website lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P46" s="3" t="inlineStr">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Neuro, Critical care</t>
+          <t>Officially confirmed: Brain &amp; spine, Critical care (ICU). Website also lists: Cardiology, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P47" s="3" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>Site lists: emergency ('24-hour emergency obstetric care' only; no trauma centre page), critical care (anaesthesia page mentions 'critical care medicine' in the curriculum; no ICU page)</t>
+          <t>Hospital website lists: Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P48" s="3" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Neuro, Critical care, Paeds</t>
+          <t>Officially confirmed: Heart, Brain &amp; spine, Critical care (ICU), Children's surgery. Website also lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
         </is>
       </c>
       <c r="P49" s="4" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>Site lists: nephrology/dialysis (24-hour dialysis listed; no nephrology department), NICU (level 2), PICU, trauma/emergency (Accident &amp; Emergency department), pain clinic (Pain OPD Tuesdays with interventions; acute &amp; chronic pain management, labour analgesia), cardiology-type procedures only (temporary/permanent pacing, thrombolysis; no cath lab or cardiology department)</t>
+          <t>Hospital website lists: Cardiology, Kidney (dialysis), Newborn / child ICU, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P50" s="3" t="inlineStr">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Critical care</t>
+          <t>Officially confirmed: Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
         </is>
       </c>
       <c r="P51" s="3" t="inlineStr">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>Site lists: critical care ('Critical Care Unit'), cardiology ('Intensive Coronary Care Unit'; no cath lab mentioned), nephrology/dialysis ('Haemodialysis'), burns ('Intensive Burns Unit'), NICU-equivalent ('Special Care Baby Unit'), neurosurgery (listed), oncology ('Cancer Therapy'; surgical oncology not specified), nuclear medicine, MRI, CT, psychiatry, rehabilitation, 'Ultramodern Operation Theatre', Eye OT</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P52" s="7" t="inlineStr">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Critical care</t>
+          <t>Officially confirmed: Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P53" s="7" t="inlineStr">
@@ -5344,7 +5344,7 @@
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Critical care</t>
+          <t>Officially confirmed: Heart, Critical care (ICU).</t>
         </is>
       </c>
       <c r="P54" s="7" t="inlineStr">
@@ -5431,7 +5431,7 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Critical care, Renal/Transplant</t>
+          <t>Officially confirmed: Critical care (ICU), Kidney &amp; transplant.</t>
         </is>
       </c>
       <c r="P55" s="7" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>Official courses: GI surgery, Cardiac, Neuro, Critical care</t>
+          <t>Officially confirmed: Stomach &amp; liver (GI) surgery, Heart, Brain &amp; spine, Critical care (ICU).</t>
         </is>
       </c>
       <c r="P56" s="7" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Vascular/Thoracic</t>
+          <t>Officially confirmed: Blood vessel &amp; chest surgery.</t>
         </is>
       </c>
       <c r="P57" s="7" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Neuro, Renal/Transplant, GI surgery, Critical care</t>
+          <t>Officially confirmed: Heart, Brain &amp; spine, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery, Critical care (ICU).</t>
         </is>
       </c>
       <c r="P59" s="7" t="inlineStr">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac surgery/CTVS (peopletreehospitals.co.in: CABG, minimally invasive cardiac surgery - 'one of the five hospitals in the city capable of performing MICS', open-heart surgery, valve repair/replacement; cardiovascular surgeon Dr Akshay Kumar Singh), cardiology/cath lab ('Modular Cathlab'; angioplasty, pacemaker, AICD, CRT, RF ablation, electrophysiology, 3D mapping, 128-slice CT, cardiac MRI; interventional cardiologist Dr Karthik Naidu K C, non-interventional Dr Manjunath Kadakol), paediatric cardiology, cardiac anaesthesia (Dr Suma K Rao, cardiac anaesthesiologist), not shown on any reachable official page: neurosurgery, nephrology/dialysis, urology, transplant, GI surgery, surgical oncology, paediatric surgery, NICU, PICU, trauma/emergency, burns, pain clinic</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P63" s="3" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac</t>
+          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU.</t>
         </is>
       </c>
       <c r="P64" s="3" t="inlineStr">
@@ -6394,7 +6394,7 @@
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac surgery (listed as a speciality on the homepage only; cardiology page describes cath-lab work, no CABG/valve, no cardiac surgeon named), cardiology/cath lab ('State-of-the-art Cath Lab', 24/7; coronary angiography &amp; angioplasty; Dr Krishna Kumar B R, Dr Balakrishna G T), neurosurgery (Dr Pratham R Bysani; tumour, aneurysm, awake craniotomy, endoscopic spine, thrombectomy), nephrology/dialysis (nephrology listed), urology, GI surgery (surgical gastroenterology), surgical oncology, NICU ('Level-3 NICU')</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P66" s="7" t="inlineStr">
@@ -6481,7 +6481,7 @@
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Onco, Cardiac, Renal/Transplant, GI surgery, Critical care</t>
+          <t>Officially confirmed: Cancer, Heart, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery, Critical care (ICU).</t>
         </is>
       </c>
       <c r="P67" s="7" t="inlineStr">
@@ -6659,7 +6659,7 @@
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>Site lists: neurosurgery (unit doctor: MCh Neurosurgery), nephrology/urology (unit doctor: MCh Urology), GI surgery (unit doctor: MCh GI Surgery), cardiac sciences (unit doctor listed), interventional radiology (unit doctor: FNVIR), medical gastroenterology, rheumatology, NICU/PICU (listed under procedures)</t>
+          <t>Hospital website lists: Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Newborn / child ICU. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P69" s="4" t="inlineStr">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, GI surgery</t>
+          <t>Officially confirmed: Heart, Stomach &amp; liver (GI) surgery. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns.</t>
         </is>
       </c>
       <c r="P70" s="3" t="inlineStr">
@@ -6837,7 +6837,7 @@
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac</t>
+          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P71" s="3" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Renal/Transplant</t>
+          <t>Officially confirmed: Heart, Kidney &amp; transplant. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
         </is>
       </c>
       <c r="P72" s="3" t="inlineStr">
@@ -7019,7 +7019,7 @@
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiology incl. interventional cardiology; 'cardiac surgery' claimed in home-page Centers of Excellence text; vascular surgery (menu), neurology/neurosurgery (menu), nephrology/haemodialysis; urology 'incl. dialysis' (menu + home text), kidney transplant (news banner: 'Successful Kidney Transplant Surgery'), surgical gastroenterology (menu), oncology + new chemotherapy suite (banner), paediatrics/paediatric surgery; new NICU (banner), trauma care unit 24/7 with advanced life support; accident &amp; emergency (home text/menu)</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P73" s="3" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiology (no CTVS/cardiac surgery page on either the live or archived site), neurosurgery (live: Department of Neurosurgery; archived: Neurology &amp; Neuro Surgery), nephrology (dialysis not quantified), urology, GI surgery (live: Surgical Gastroenterology), surgical oncology (live: Oncosurgery), paediatric surgery (live), vascular surgery, plastic surgery (live)</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P74" s="3" t="inlineStr">
@@ -7197,7 +7197,7 @@
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Critical care</t>
+          <t>Officially confirmed: Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
         </is>
       </c>
       <c r="P75" s="3" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiology (department page), neurosurgery (department page), nephrology/dialysis ('Dialysis Unit' on about page; no nephrology dept), NICU ('Neonatal ICU'; Paediatrics &amp; Neonatology dept), trauma/emergency (Accident &amp; Emergency dept), ICU ('10 beds (closed unit)', 8 ventilators)</t>
+          <t>Hospital website lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P76" s="3" t="inlineStr">
@@ -7375,7 +7375,7 @@
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>Official courses: GI surgery, Critical care, Neuro, Renal/Transplant</t>
+          <t>Officially confirmed: Stomach &amp; liver (GI) surgery, Critical care (ICU), Brain &amp; spine, Kidney &amp; transplant. Website also lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P77" s="3" t="inlineStr">
@@ -7470,7 +7470,7 @@
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac</t>
+          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P78" s="3" t="inlineStr">
@@ -7557,7 +7557,7 @@
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac surgery/CTVS (Dr Suraj Kumar Pradhan, MCh, 'Director, CTVS Department'; CABG, valve MVR/AVR/DVR, children's heart surgery, minimally invasive heart surgery; 'dedicated 24x7 Cardiac ICU'; cardiac anaesthesiologist Dr Hrishikesh Bharali, MD with fellowship in cardiac anaesthesia), cardiology/cath lab (cath lab listed), neurosurgery (Dr Mayukh Kamal Goswami, MCh; craniotomy for TBI/bleeds, brain tumour, minimally invasive spine), nephrology/dialysis (dialysis unit), urology (listed), oncology &amp; onco-surgery (listed), NICU (listed), ICU/HDU; trauma ICU, neuro ICU and surgical ICU referenced (no numbers)</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P79" s="3" t="inlineStr">
@@ -7642,7 +7642,7 @@
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Critical care</t>
+          <t>Officially confirmed: Heart, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
         </is>
       </c>
       <c r="P80" s="6" t="inlineStr">
@@ -7735,7 +7735,7 @@
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Neuro, Critical care</t>
+          <t>Officially confirmed: Heart, Brain &amp; spine, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
         </is>
       </c>
       <c r="P81" s="3" t="inlineStr">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Neuro, Critical care</t>
+          <t>Officially confirmed: Brain &amp; spine, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns.</t>
         </is>
       </c>
       <c r="P82" s="5" t="inlineStr">
@@ -7921,7 +7921,7 @@
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac surgery ('Cardio-Thoracic &amp; Vascular Surgery' department; anaesthesia page: anaesthesia for 'Cardiac Surgery'), cardiology ('Shija Heart Beat', Department of Cardiology; cath lab not stated), neurosurgery (department; Neurosciences centre of excellence), nephrology/dialysis ('150+ per day' dialysis), urology ('with transplantation services'), kidney transplant ('135' kidney transplants done), surgical oncology (department), paediatrics &amp; neonatology (NICU not explicit)</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P83" s="6" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Renal/Transplant, Critical care</t>
+          <t>Officially confirmed: Heart, Kidney &amp; transplant, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic.</t>
         </is>
       </c>
       <c r="P84" s="3" t="inlineStr">
@@ -8109,7 +8109,7 @@
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>Site lists: trauma/emergency (unit page: 'special focus on Orthopaedics, Trauma and Cardiology'), cardiology, nephrology (unit doctor listed), surgical oncology (unit doctor listed: MCh Surgical Oncology), pain clinic (unit doctor: 'Pain &amp; Rehabilitation Medicine', MBBS DA DNB FPM)</t>
+          <t>Hospital website lists: Cardiology, Kidney (dialysis), Cancer surgery, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P85" s="3" t="inlineStr">
@@ -8204,7 +8204,7 @@
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiac surgery (CTVS): 'Cardiothoracic Vascular Surgery' - one consultant (Dr Shegu Gilbert); on/off-pump CABG, valve repair/replacement, Bentall, ASD/VSD/TOF corrections listed, cardiology/cath lab: 'Cardiology', 'Angiography &amp; Angioplasty', 'Cardiac ICU' (homepage), neurosurgery: listed (neurosurgery-hospital-tirupati/), nephrology/dialysis: 'Nephrology (with hemodialysis, peritoneal dialysis, CRRT)', urology: listed, GI surgery: 'Surgical Gastroenterology' (departments/), trauma/emergency: '24/7 Emergency &amp; Trauma Centre (Level 1)' (homepage); 'Emergency Medicine' dept, pain clinic: 'Pain Medicine' on anaesthesia page; 'Consultant, Pain Medicine' (Dr Rajesh Naidu B) on critical-care page</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P86" s="3" t="inlineStr">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac</t>
+          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P87" s="3" t="inlineStr">
@@ -8382,7 +8382,7 @@
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Neuro</t>
+          <t>Officially confirmed: Heart, Brain &amp; spine. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
         </is>
       </c>
       <c r="P88" s="3" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>Site lists: cardiology/cath lab ('flat panel cardiac Cath Lab') - Vizianagaram unit site, neurosurgery (centre of excellence) - Vizianagaram unit site, nephrology/dialysis ('Over 100 Dialysis per month') - Vizianagaram unit site, GI surgery and gastroenterology - Vizianagaram unit site, paediatric surgery, vascular surgery, plastic surgery - Vizianagaram unit site, urology, oncology, emergency medicine, anaesthesia &amp; critical care (department links) - Vizianagaram unit site, KIMS Seethammadhara (the ex-Queen's NRI Visakhapatnam unit) page lists KIMS group specialities generically (CTVS, neurosurgery, liver transplant, oncology...); unit doctors named: Clinical Director/HOD Anaesthesia-Critical Care-Pain &amp; Palliative Medicine, Clinical Lead Critical Care &amp; consultant anaesthesiologist, chief consultant critical care, senior consultant neurosurgeon, chief consultant gastroenterology/liver transplantation, medical oncology/BMT consultant</t>
+          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
         </is>
       </c>
       <c r="P89" s="7" t="inlineStr">
@@ -8560,7 +8560,7 @@
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>Official courses: Cardiac, Neuro</t>
+          <t>Officially confirmed: Heart, Brain &amp; spine. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
         </is>
       </c>
       <c r="P90" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Multispeciality label: no department count (matches the plain list)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -1597,7 +1597,7 @@
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>Medium — 3 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>Medium — 8 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>Medium — 4 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>Medium — 5 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>Medium — 8 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>Medium — 3 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="N31" s="6" t="inlineStr">
         <is>
-          <t>Medium — 3 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="N33" s="6" t="inlineStr">
         <is>
-          <t>Medium — 5 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="N34" s="6" t="inlineStr">
         <is>
-          <t>Medium — 6 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="N36" s="6" t="inlineStr">
         <is>
-          <t>Medium — 5 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
@@ -3992,7 +3992,7 @@
       </c>
       <c r="N39" s="6" t="inlineStr">
         <is>
-          <t>Medium — 5 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="N40" s="6" t="inlineStr">
         <is>
-          <t>Medium — 5 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
@@ -4449,7 +4449,7 @@
       </c>
       <c r="N44" s="6" t="inlineStr">
         <is>
-          <t>Medium — 4 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
@@ -4629,7 +4629,7 @@
       </c>
       <c r="N46" s="6" t="inlineStr">
         <is>
-          <t>Medium — 4 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="N52" s="6" t="inlineStr">
         <is>
-          <t>Medium — 4 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O52" s="2" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="N63" s="6" t="inlineStr">
         <is>
-          <t>Medium — 5 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O63" s="2" t="inlineStr">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="N66" s="6" t="inlineStr">
         <is>
-          <t>Medium — 4 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O66" s="2" t="inlineStr">
@@ -6654,7 +6654,7 @@
       </c>
       <c r="N69" s="6" t="inlineStr">
         <is>
-          <t>Medium — 3 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O69" s="2" t="inlineStr">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="N73" s="6" t="inlineStr">
         <is>
-          <t>Medium — 5 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O73" s="2" t="inlineStr">
@@ -7105,7 +7105,7 @@
       </c>
       <c r="N74" s="6" t="inlineStr">
         <is>
-          <t>Medium — 6 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O74" s="2" t="inlineStr">
@@ -7552,7 +7552,7 @@
       </c>
       <c r="N79" s="6" t="inlineStr">
         <is>
-          <t>Medium — 6 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O79" s="2" t="inlineStr">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="N83" s="6" t="inlineStr">
         <is>
-          <t>Medium — 6 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O83" s="2" t="inlineStr">
@@ -8199,7 +8199,7 @@
       </c>
       <c r="N86" s="6" t="inlineStr">
         <is>
-          <t>Medium — 3 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O86" s="2" t="inlineStr">
@@ -8468,7 +8468,7 @@
       </c>
       <c r="N89" s="6" t="inlineStr">
         <is>
-          <t>Medium — 5 super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="O89" s="2" t="inlineStr">
@@ -8882,12 +8882,12 @@
       <c r="A21" s="10" t="inlineStr"/>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Medium — N super-speciality depts, hospital's own claim</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Only the hospital website says so; nothing official confirms it.</t>
+          <t>The hospital website lists super-speciality departments (named in the detail); no official training course confirms them.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multispeciality field: department names only; source shown by the label
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -711,12 +711,12 @@
       </c>
       <c r="N2" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart.</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="P2" s="7" t="inlineStr">
@@ -966,12 +966,12 @@
       </c>
       <c r="N5" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Critical care (ICU).</t>
+          <t>Critical care (ICU)</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
@@ -1134,12 +1134,12 @@
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, GI surgery, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Stomach &amp; liver (GI) surgery, Critical care (ICU).</t>
+          <t>Heart, Stomach &amp; liver (GI) surgery, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
@@ -1221,12 +1221,12 @@
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
+          <t>Critical care (ICU)</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
@@ -1320,12 +1320,12 @@
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Neuro, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Brain &amp; spine, Critical care (ICU).</t>
+          <t>Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Cancer, Heart, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery, Critical care (ICU).</t>
+          <t>Cancer, Heart, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P10" s="7" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Children's surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
+          <t>Heart, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P12" s="7" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
       <c r="P13" s="7" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P14" s="5" t="inlineStr">
@@ -1866,12 +1866,12 @@
       </c>
       <c r="N15" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="P15" s="7" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Newborn / child ICU, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="P17" s="6" t="inlineStr">
@@ -2224,12 +2224,12 @@
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Neuro (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Brain &amp; spine.</t>
+          <t>Heart, Brain &amp; spine</t>
         </is>
       </c>
       <c r="P19" s="6" t="inlineStr">
@@ -2319,12 +2319,12 @@
       </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Critical care (ICU).</t>
+          <t>Critical care (ICU)</t>
         </is>
       </c>
       <c r="P20" s="6" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
       <c r="P21" s="3" t="inlineStr">
@@ -2521,12 +2521,12 @@
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Critical care, GI surgery (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Critical care (ICU), Stomach &amp; liver (GI) surgery. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
+          <t>Critical care (ICU), Stomach &amp; liver (GI) surgery</t>
         </is>
       </c>
       <c r="P22" s="4" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P23" s="7" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Burns, Pain clinic. Not officially confirmed.</t>
+          <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Burns, Pain clinic</t>
         </is>
       </c>
       <c r="P24" s="3" t="inlineStr">
@@ -2788,12 +2788,12 @@
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Renal/Transplant (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Kidney &amp; transplant. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
+          <t>Kidney &amp; transplant</t>
         </is>
       </c>
       <c r="P25" s="3" t="inlineStr">
@@ -2964,12 +2964,12 @@
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Neuro, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Brain &amp; spine, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
+          <t>Heart, Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P27" s="3" t="inlineStr">
@@ -3138,12 +3138,12 @@
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Neuro (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Brain &amp; spine.</t>
+          <t>Heart, Brain &amp; spine</t>
         </is>
       </c>
       <c r="P29" s="7" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Cardiology, Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Cardiology, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P30" s="7" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
       <c r="P31" s="3" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Brain &amp; spine surgery, Kidney transplant, Urology, Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Heart surgery, Brain &amp; spine surgery, Kidney transplant, Urology, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Brain &amp; spine surgery, Kidney transplant, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Heart surgery, Brain &amp; spine surgery, Kidney transplant, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P34" s="3" t="inlineStr">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Critical care (ICU), Heart, Brain &amp; spine, Stomach &amp; liver (GI) surgery. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic.</t>
+          <t>Critical care (ICU), Heart, Brain &amp; spine, Stomach &amp; liver (GI) surgery</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Pain clinic</t>
         </is>
       </c>
       <c r="P36" s="3" t="inlineStr">
@@ -3808,12 +3808,12 @@
       </c>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Onco (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Cancer. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
+          <t>Cancer</t>
         </is>
       </c>
       <c r="P37" s="3" t="inlineStr">
@@ -3903,12 +3903,12 @@
       </c>
       <c r="N38" s="6" t="inlineStr">
         <is>
-          <t>Medium — only GI surgery, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Stomach &amp; liver (GI) surgery, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Pain clinic.</t>
+          <t>Stomach &amp; liver (GI) surgery, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P38" s="3" t="inlineStr">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
       <c r="P39" s="3" t="inlineStr">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="P40" s="6" t="inlineStr">
@@ -4178,12 +4178,12 @@
       </c>
       <c r="N41" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Renal/Transplant, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Kidney &amp; transplant, Critical care (ICU).</t>
+          <t>Heart, Kidney &amp; transplant, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P41" s="3" t="inlineStr">
@@ -4273,12 +4273,12 @@
       </c>
       <c r="N42" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="P42" s="3" t="inlineStr">
@@ -4363,7 +4363,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>Not found online. A Punjab govt district civil hospital offering 7 DNB/diploma programmes (General Medicine, General Surgery, Family Medicine, Radiology, DCH, DGO, Anaesthesia). Exposure is likely general surgery, obstetrics, trauma and emergency; no evidence of super-speciality services.</t>
+          <t>Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P43" s="7" t="inlineStr">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="P44" s="3" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Brain &amp; spine surgery, Children's surgery, Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Heart surgery, Brain &amp; spine surgery, Children's surgery, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P45" s="3" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns. Not officially confirmed.</t>
+          <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns</t>
         </is>
       </c>
       <c r="P46" s="3" t="inlineStr">
@@ -4716,12 +4716,12 @@
       </c>
       <c r="N47" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Neuro, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Brain &amp; spine, Critical care (ICU). Website also lists: Cardiology, Trauma &amp; emergency.</t>
+          <t>Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P47" s="3" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P48" s="3" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Brain &amp; spine, Critical care (ICU), Children's surgery. Website also lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
+          <t>Heart, Brain &amp; spine, Critical care (ICU), Children's surgery</t>
         </is>
       </c>
       <c r="P49" s="4" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Cardiology, Kidney (dialysis), Newborn / child ICU, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
+          <t>Cardiology, Kidney (dialysis), Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="P50" s="3" t="inlineStr">
@@ -5074,12 +5074,12 @@
       </c>
       <c r="N51" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
+          <t>Critical care (ICU)</t>
         </is>
       </c>
       <c r="P51" s="3" t="inlineStr">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
       <c r="P52" s="7" t="inlineStr">
@@ -5248,12 +5248,12 @@
       </c>
       <c r="N53" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Trauma &amp; emergency.</t>
+          <t>Critical care (ICU)</t>
         </is>
       </c>
       <c r="P53" s="7" t="inlineStr">
@@ -5339,12 +5339,12 @@
       </c>
       <c r="N54" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Critical care (ICU).</t>
+          <t>Heart, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P54" s="7" t="inlineStr">
@@ -5426,12 +5426,12 @@
       </c>
       <c r="N55" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Critical care, Renal/Transplant (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Critical care (ICU), Kidney &amp; transplant.</t>
+          <t>Critical care (ICU), Kidney &amp; transplant</t>
         </is>
       </c>
       <c r="P55" s="7" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Stomach &amp; liver (GI) surgery, Heart, Brain &amp; spine, Critical care (ICU).</t>
+          <t>Stomach &amp; liver (GI) surgery, Heart, Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P56" s="7" t="inlineStr">
@@ -5600,12 +5600,12 @@
       </c>
       <c r="N57" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Vascular/Thoracic (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Blood vessel &amp; chest surgery.</t>
+          <t>Blood vessel &amp; chest surgery</t>
         </is>
       </c>
       <c r="P57" s="7" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Brain &amp; spine, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery, Critical care (ICU).</t>
+          <t>Heart, Brain &amp; spine, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P59" s="7" t="inlineStr">
@@ -5858,11 +5858,7 @@
           <t>Low — little super-speciality work</t>
         </is>
       </c>
-      <c r="O60" s="2" t="inlineStr">
-        <is>
-          <t>Government General Hospital, Jayanagar, Bengaluru (state Health dept); DNB centre since 2018 with 2 Anaesthesia seats (prior notes). Aggregator lists Anaesthesia, Medicine, OBG, Paeds, Ortho, Radiology; ICU and labour/maternity. No super-speciality surgery found.</t>
-        </is>
-      </c>
+      <c r="O60" s="2" t="inlineStr"/>
       <c r="P60" s="6" t="inlineStr">
         <is>
           <t>Some — reported, but not by residents</t>
@@ -5955,7 +5951,7 @@
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>Aggregator: NABH/NABL hospital with 30+ specialities incl. cardiology, neurology, orthopaedics, urology, oncology, paediatrics; 128-slice CT. Official unit-level detail (CTVS, transplant, NICU level) could not be retrieved (sagarhospitals.in page did not render).</t>
+          <t>Heart surgery, Cardiology, Urology, Cancer surgery, Newborn / child ICU</t>
         </is>
       </c>
       <c r="P61" s="7" t="inlineStr">
@@ -6040,7 +6036,7 @@
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>Kauvery group (12 hospitals) lists heart-lung, kidney, liver and BMT transplant, neurosurgery, oncology, mother &amp; child, vascular surgery and runs DNB courses, but which of these run at the Electronic City unit could not be confirmed from the unit page.</t>
+          <t>Brain &amp; spine surgery, Cancer surgery</t>
         </is>
       </c>
       <c r="P62" s="7" t="inlineStr">
@@ -6127,7 +6123,7 @@
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
       <c r="P63" s="3" t="inlineStr">
@@ -6209,12 +6205,12 @@
       </c>
       <c r="N64" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU.</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="P64" s="3" t="inlineStr">
@@ -6305,7 +6301,7 @@
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>Government SNR District Hospital, Kolar. Aggregator lists DNB Anaesthesia, Paediatrics, OBG plus diplomas, a 24-bed neonatal SNCU, expanding CT/MRI and a new mother-and-child block. No super-speciality surgery found.</t>
+          <t>Newborn / child ICU</t>
         </is>
       </c>
       <c r="P65" s="6" t="inlineStr">
@@ -6394,7 +6390,7 @@
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P66" s="7" t="inlineStr">
@@ -6481,7 +6477,7 @@
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Cancer, Heart, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery, Critical care (ICU).</t>
+          <t>Cancer, Heart, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P67" s="7" t="inlineStr">
@@ -6568,7 +6564,7 @@
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>Official site lists centres for Cardiac Sciences (cardiology + CTVS), Brain &amp; Spine (neurosurgery; also runs DNB Neurosurgery), GI Surgery &amp; Liver Transplantation, Renal Sciences &amp; transplant, cancer care, paediatric super-speciality incl. NICU, obstetrics, rehab and 24x7 emergency. NABH/JCI-standard infrastructure; Japanese-Indian (Secom/Toyota Tsusho) MNC hospital.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Liver transplant, GI surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P68" s="7" t="inlineStr">
@@ -6659,7 +6655,7 @@
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Newborn / child ICU. Not officially confirmed.</t>
+          <t>Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Newborn / child ICU</t>
         </is>
       </c>
       <c r="P69" s="4" t="inlineStr">
@@ -6743,12 +6739,12 @@
       </c>
       <c r="N70" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, GI surgery (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Stomach &amp; liver (GI) surgery. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns.</t>
+          <t>Heart, Stomach &amp; liver (GI) surgery</t>
         </is>
       </c>
       <c r="P70" s="3" t="inlineStr">
@@ -6832,12 +6828,12 @@
       </c>
       <c r="N71" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="P71" s="3" t="inlineStr">
@@ -6923,12 +6919,12 @@
       </c>
       <c r="N72" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Renal/Transplant (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Kidney &amp; transplant. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
+          <t>Heart, Kidney &amp; transplant</t>
         </is>
       </c>
       <c r="P72" s="3" t="inlineStr">
@@ -7019,7 +7015,7 @@
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P73" s="3" t="inlineStr">
@@ -7110,7 +7106,7 @@
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
       <c r="P74" s="3" t="inlineStr">
@@ -7192,12 +7188,12 @@
       </c>
       <c r="N75" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
+          <t>Critical care (ICU)</t>
         </is>
       </c>
       <c r="P75" s="3" t="inlineStr">
@@ -7284,7 +7280,7 @@
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Newborn / child ICU, Trauma &amp; emergency. Not officially confirmed.</t>
+          <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P76" s="3" t="inlineStr">
@@ -7375,7 +7371,7 @@
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Stomach &amp; liver (GI) surgery, Critical care (ICU), Brain &amp; spine, Kidney &amp; transplant. Website also lists: Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Trauma &amp; emergency.</t>
+          <t>Stomach &amp; liver (GI) surgery, Critical care (ICU), Brain &amp; spine, Kidney &amp; transplant</t>
         </is>
       </c>
       <c r="P77" s="3" t="inlineStr">
@@ -7465,12 +7461,12 @@
       </c>
       <c r="N78" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="P78" s="3" t="inlineStr">
@@ -7557,7 +7553,7 @@
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
       <c r="P79" s="3" t="inlineStr">
@@ -7637,12 +7633,12 @@
       </c>
       <c r="N80" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
+          <t>Heart, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P80" s="6" t="inlineStr">
@@ -7730,12 +7726,12 @@
       </c>
       <c r="N81" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Neuro, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Brain &amp; spine, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
+          <t>Heart, Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P81" s="3" t="inlineStr">
@@ -7825,12 +7821,12 @@
       </c>
       <c r="N82" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Neuro, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Brain &amp; spine, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns.</t>
+          <t>Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P82" s="5" t="inlineStr">
@@ -7921,7 +7917,7 @@
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns</t>
         </is>
       </c>
       <c r="P83" s="6" t="inlineStr">
@@ -8009,12 +8005,12 @@
       </c>
       <c r="N84" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Renal/Transplant, Critical care (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Kidney &amp; transplant, Critical care (ICU). Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic.</t>
+          <t>Heart, Kidney &amp; transplant, Critical care (ICU)</t>
         </is>
       </c>
       <c r="P84" s="3" t="inlineStr">
@@ -8109,7 +8105,7 @@
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Cardiology, Kidney (dialysis), Cancer surgery, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
+          <t>Cardiology, Kidney (dialysis), Cancer surgery, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="P85" s="3" t="inlineStr">
@@ -8204,7 +8200,7 @@
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="P86" s="3" t="inlineStr">
@@ -8286,12 +8282,12 @@
       </c>
       <c r="N87" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="P87" s="3" t="inlineStr">
@@ -8377,12 +8373,12 @@
       </c>
       <c r="N88" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Neuro (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Brain &amp; spine. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic.</t>
+          <t>Heart, Brain &amp; spine</t>
         </is>
       </c>
       <c r="P88" s="3" t="inlineStr">
@@ -8473,7 +8469,7 @@
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>Hospital website lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency, Pain clinic. Not officially confirmed.</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="P89" s="7" t="inlineStr">
@@ -8555,12 +8551,12 @@
       </c>
       <c r="N90" s="6" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac, Neuro (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>Officially confirmed: Heart, Brain &amp; spine. Website also lists: Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency.</t>
+          <t>Heart, Brain &amp; spine</t>
         </is>
       </c>
       <c r="P90" s="5" t="inlineStr">
@@ -8869,12 +8865,12 @@
       <c r="A20" s="10" t="inlineStr"/>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Medium — only Cardiac … (officially confirmed)</t>
+          <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Officially confirmed, but in only 1–2 areas (named in the label).</t>
+          <t>Official super-speciality training runs here, but in only 1–2 areas (listed under the label).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Shortlist: facts-only short text in every column (source shown by label); website notes saying a dept is absent no longer counted
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -699,11 +699,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
           <t>₹64,000</t>
@@ -786,11 +782,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
           <t>₹51,000</t>
@@ -867,11 +859,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
           <t>₹43,000/month</t>
@@ -896,7 +884,7 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>Nothing bad found. One review site says the stipend is ₹15,000/month, but the hospital told MCC ₹43,000. (review site)</t>
+          <t>Stipend ₹15,000/month reported vs ₹43,000 declared</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr"/>
@@ -954,11 +942,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
           <t>₹75,000</t>
@@ -1039,11 +1023,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr">
         <is>
           <t>₹43,000/month</t>
@@ -1122,11 +1102,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
           <t>₹57,000</t>
@@ -1209,11 +1185,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr">
         <is>
           <t>₹58,900</t>
@@ -1236,7 +1208,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>The official page shows a 6-OT, 210-bed multispecialty set-up giving anaesthesia for neurosurgery, cardiothoracic, paediatric, gastro and urological surgery plus IVF, with a pre-anaesthetic clinic and 7-bed post-op room, which implies a broad case mix, but says nothing about USG-guided blocks, simulation or resident case numbers. The only resident voice is one anonymous AmbitionBox rating (skill development 4/5) - weak evidence.</t>
+          <t>6 OTs, 210 beds; neuro, cardiothoracic, paeds, gastro, uro and IVF cases</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
@@ -1246,12 +1218,12 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>No suicide or strike found. 2017: complaint to the DNB board about inhuman duty hours (radiology). 2025: a resident called the ~₹50k stipend low. (news + resident post)</t>
+          <t>2017 duty-hours complaint (radiology); ~₹50k stipend called low (2025)</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>A 2017 complaint said radiology residents worked 32–56 hours at a stretch. A 2025 resident rated work-life balance 5 out of 5. No anaesthesia-specific info. (complaint + review site)</t>
+          <t>2017: radiology residents worked 32–56 h at a stretch</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr"/>
@@ -1308,11 +1280,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
           <t>₹58,000</t>
@@ -1341,12 +1309,12 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Nothing bad found for 2019–26. 2017: a radiology PG was murdered in the hospital duty room. (news)</t>
+          <t>2017: radiology PG murdered in hospital duty room</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>Normal OT days plus 6–9 emergency duties a month; OT changes every week. (one anaesthesia resident, 2021)</t>
+          <t>OT days plus 6–9 emergency duties a month (2021)</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr"/>
@@ -1403,11 +1371,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr">
         <is>
           <t>₹63,000</t>
@@ -1436,7 +1400,7 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Nothing bad found about residents. June 2026: Delhi govt ordered action after finding patient-care lapses. (news)</t>
+          <t>June 2026: Delhi govt ordered action over patient-care lapses</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr"/>
@@ -1494,11 +1458,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr">
         <is>
           <t>₹70,000</t>
@@ -1521,7 +1481,7 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>No resident or alumni account found. The hospital's DNB anaesthesiology page lists six senior-consultant faculty (MD/DNB qualified 1993-2009); it is a 242-bed private hospital (aggregator). The only 'review' text online is Meducate's generic boilerplate ('diverse clinical caseload ... procedural training'), which is not a resident account.</t>
+          <t>242 beds; six senior consultant faculty</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -1585,11 +1545,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr">
         <is>
           <t>₹72,000</t>
@@ -1678,14 +1634,10 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
-        </is>
-      </c>
+          <t>Low — little or no super-speciality work</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
@@ -1699,7 +1651,7 @@
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>Nothing about this hospital itself. GMERS colleges cut junior-doctor pay in 2023 and had a stipend strike at another GMERS college. (news)</t>
+          <t>GMERS group cut junior-doctor pay (2023)</t>
         </is>
       </c>
       <c r="T13" s="2" t="inlineStr"/>
@@ -1755,11 +1707,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
           <t>₹ 40,000/month</t>
@@ -1782,7 +1730,7 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>The hospital's own DNB page is unusually explicit: 3 seats a year, 'direct, hands-on involvement in operation-theatre anaesthesia, critical care, obstetric anaesthesia and pain management', 'exposure to regional blocks', structured critical-care rotations and 'close consultant mentorship' from three named senior consultants, in a 200-250-bed tertiary hospital opposite AIIMS Jodhpur (earlier pass: ~100 surgeries/day across 8 OTs). But the programme only started in 2025 (the hospital's own launch posts), so there are no seniors or alumni and no resident account.</t>
+          <t>Hands-on OT, ICU, obstetric, pain work and regional blocks; ~100 surgeries/day; started 2025</t>
         </is>
       </c>
       <c r="R14" s="6" t="inlineStr">
@@ -1790,15 +1738,11 @@
           <t>OK — nothing bad found online</t>
         </is>
       </c>
-      <c r="S14" s="2" t="inlineStr">
-        <is>
-          <t>Nothing bad found about this hospital. (Jodhpur news was about AIIMS and SN Medical College.)</t>
-        </is>
-      </c>
+      <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>Hospital says PGs do planned critical-care rotations. Length not stated. (hospital website)</t>
+          <t>Planned critical-care rotations</t>
         </is>
       </c>
     </row>
@@ -1854,11 +1798,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
           <t>₹56,100</t>
@@ -1885,11 +1825,7 @@
           <t>OK — nothing bad found online</t>
         </is>
       </c>
-      <c r="S15" s="2" t="inlineStr">
-        <is>
-          <t>Nothing bad found about this hospital. (Jaipur news about strikes and suicides was about other colleges.)</t>
-        </is>
-      </c>
+      <c r="S15" s="2" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
     </row>
@@ -1945,11 +1881,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr">
         <is>
           <t>₹55,200</t>
@@ -1972,11 +1904,7 @@
           <t>OK — nothing bad found online</t>
         </is>
       </c>
-      <c r="S16" s="2" t="inlineStr">
-        <is>
-          <t>Nothing bad found about this hospital. (Bikaner suicide news was about SP Medical College, not Kothari.)</t>
-        </is>
-      </c>
+      <c r="S16" s="2" t="inlineStr"/>
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
     </row>
@@ -2032,11 +1960,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
           <t>₹60,000</t>
@@ -2049,7 +1973,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="P17" s="6" t="inlineStr">
@@ -2059,7 +1983,7 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>No resident account found. meducate (aggregator) says hands-on is 'satisfactory, particularly in orthopaedic procedures and trauma' - a likely good source of regional blocks, but not verified.</t>
+          <t>Satisfactory hands-on, especially orthopaedic and trauma cases</t>
         </is>
       </c>
       <c r="R17" s="6" t="inlineStr">
@@ -2071,7 +1995,7 @@
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>25-bed ICU; anaesthesia and critical-care trainees are trained together. Posting length not stated. (hospital website)</t>
+          <t>25-bed ICU; trained alongside critical-care trainees</t>
         </is>
       </c>
     </row>
@@ -2125,11 +2049,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
           <t>₹60,000</t>
@@ -2152,11 +2072,7 @@
           <t>OK — nothing bad found online</t>
         </is>
       </c>
-      <c r="S18" s="2" t="inlineStr">
-        <is>
-          <t>Nothing bad found about this hospital. (Lucknow news was about KGMU.)</t>
-        </is>
-      </c>
+      <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
     </row>
@@ -2212,11 +2128,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
           <t>₹70,000</t>
@@ -2239,7 +2151,7 @@
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>No resident account found. meducate (aggregator) says 'hands-on procedural opportunities in surgical specialties may be limited due to the consultant-led corporate practice model'. 2 DNB anaesthesia seats/yr.</t>
+          <t>Hands-on may be limited: consultant-led corporate model; 2 seats/yr</t>
         </is>
       </c>
       <c r="R19" s="6" t="inlineStr">
@@ -2251,7 +2163,7 @@
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>Review says ICU exposure is 'strong'. Posting length not stated. (review site)</t>
+          <t>Strong ICU exposure</t>
         </is>
       </c>
     </row>
@@ -2307,11 +2219,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr">
         <is>
           <t>₹60,000</t>
@@ -2334,7 +2242,7 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>No resident account found. meducate (aggregator) says exposure is strongest in ICU/critical care and many procedures are consultant-led. 2 (+1) DNB anaesthesia seats/yr.</t>
+          <t>Strongest in ICU; many procedures consultant-led; 2 (+1) seats/yr</t>
         </is>
       </c>
       <c r="R20" s="6" t="inlineStr">
@@ -2342,15 +2250,11 @@
           <t>OK — nothing bad found online</t>
         </is>
       </c>
-      <c r="S20" s="2" t="inlineStr">
-        <is>
-          <t>Nothing bad found about this hospital. (A Sept 2025 trainee suicide in Greater Noida was at another place.)</t>
-        </is>
-      </c>
+      <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>Review says ICU exposure is 'decent', with cardiac and neuro ICUs. Posting length not stated. (review site)</t>
+          <t>Decent ICU exposure; cardiac and neuro ICUs</t>
         </is>
       </c>
     </row>
@@ -2406,11 +2310,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr">
         <is>
           <t>₹56,100</t>
@@ -2433,7 +2333,7 @@
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>One anonymous DNB anaesthesia resident review (meducate, Aug 2022) is strongly positive on hands-on: 'Yes totally', 'all types of cases seen', patient load 'average', weekly case presentation and discussion for the next day's OT, 'far better than others for DNB'. Officially (2025 DNB brochure and department page): 300+ beds with 60 L4 ICU beds, 8 operation theatres (4 modular, 2 emergency, 2 minor), sub-speciality anaesthetists for transplant, paediatric, cardiac, neuro and obstetric work, cardiac-surgery anaesthesia and a pain clinic; 2 primary + 1 secondary DNB anaesthesia seats; HOD holds DA, DNB and FNB Critical Care. Single-source resident evidence, four years old.</t>
+          <t>All types of cases (2022); 8 OTs; transplant, cardiac, neuro, paeds, obstetric anaesthesia</t>
         </is>
       </c>
       <c r="R21" s="6" t="inlineStr">
@@ -2443,17 +2343,17 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>Nothing bad found. A 2022 resident called the department 'very chill'.</t>
+          <t>Department called 'very chill' (2022)</t>
         </is>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>About 8 hours a day; residents get rest after duty. (one resident review, 2022)</t>
+          <t>~8 h a day; rest after duty (2022)</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>Anaesthesia runs 3 ICUs (medical, surgical, cardiac) with 60 beds. Posting length not stated. (hospital website)</t>
+          <t>3 ICUs (medical, surgical, cardiac), 60 beds, run by anaesthesia</t>
         </is>
       </c>
     </row>
@@ -2509,11 +2409,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr">
         <is>
           <t>₹70,000</t>
@@ -2536,7 +2432,7 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>No resident account found. The hospital's own (2012-13 era) anaesthesia page lists four round-the-clock OTs, an ICU, labour analgesia and ALS workshops for doctors/paramedics, with no USG-block, simulation or case-volume data. An aggregator's templated 'DNB review' says the ICU and dialysis units give hands-on critical-care exposure but that 'hands-on exposure in surgical specialties may be limited as many operative cases remain consultant-led' - unsourced, weak evidence.</t>
+          <t>Hands-on mostly ICU; surgical cases largely consultant-led; 4 OTs</t>
         </is>
       </c>
       <c r="R22" s="6" t="inlineStr">
@@ -2598,11 +2494,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr">
         <is>
           <t>₹ 35,000/month</t>
@@ -2685,19 +2577,15 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr">
         <is>
           <t>₹56,100</t>
         </is>
       </c>
-      <c r="N24" s="6" t="inlineStr">
-        <is>
-          <t>Medium — only the hospital website claims them</t>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -2718,7 +2606,7 @@
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>Nothing about residents. Sep 2026: a consultant at its sister medical college died by suicide. (news)</t>
+          <t>Sep 2026: consultant at sister medical college died by suicide</t>
         </is>
       </c>
       <c r="T24" s="2" t="inlineStr"/>
@@ -2776,11 +2664,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
           <t>₹70,000</t>
@@ -2803,7 +2687,7 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>DNB Anaesthesiology at Chandan is brand new - the hospital announced its launch in Sept 2025 and the MCC DNB matrix lists 3 seats - so there are no alumni or senior residents to ask. The hospital's own page claims general/regional anaesthesia and regional-block-based post-operative pain management with a 24x7 intensivist-run ICU; the only 'review' is an aggregator saying exposure is moderate and hands-on depends on consultant involvement.</t>
+          <t>New programme (Sept 2025), 3 seats; regional blocks, 24x7 ICU; hands-on depends on consultants</t>
         </is>
       </c>
       <c r="R25" s="6" t="inlineStr">
@@ -2814,7 +2698,7 @@
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>A review site says 'structured working hours'. No actual numbers. (review site)</t>
+          <t>Structured working hours</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr"/>
@@ -2869,11 +2753,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr">
         <is>
           <t>₹ 70,000/month</t>
@@ -2952,11 +2832,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr">
         <is>
           <t>₹69,115</t>
@@ -2979,7 +2855,7 @@
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>Nothing from residents. The hospital is now branded 'CARE CHL Hospitals' (CARE Hospitals group); its anaesthesia HOD Dr Meenu Chadha is described as 42 years' experience in neuro, ortho, onco, paediatric and laparoscopic anaesthesia (hospital/aggregator snippets). Meducate lists 200 beds. Bing returned junk for every 'CHL' query; DuckDuckGo found no resident or workshop content.</t>
+          <t>200 beds; HOD experienced in neuro, ortho, onco, paeds cases</t>
         </is>
       </c>
       <c r="R27" s="6" t="inlineStr">
@@ -3068,7 +2944,7 @@
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>April 2026: about 175 PG residents went on strike — stipend not paid for 3 months. Also a state-wide junior doctors' strike in March 2026. (news)</t>
+          <t>Apr 2026: ~175 PGs struck over 3 months' unpaid stipend; state strike Mar 2026</t>
         </is>
       </c>
       <c r="T28" s="2" t="inlineStr"/>
@@ -3126,11 +3002,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
           <t>₹56,100</t>
@@ -3213,7 +3085,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>2 years (incl. mandatory 1 year field posting) · ₹40,00,000 (₹90 lakh if clubbed with super-specialty bond) · leaving: ₹10,00,000 + 18% interest p.a. + stipend drawn</t>
+          <t>2 years incl. 1-year field posting; ₹40 lakh; leaving: ₹10 lakh + 18% interest + stipend</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -3223,7 +3095,7 @@
       </c>
       <c r="N30" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
@@ -3244,12 +3116,12 @@
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>Nothing about this college itself. All Himachal residents went on strike in Dec 2025 after a doctor was sacked at IGMC Shimla. (news)</t>
+          <t>Dec 2025: state-wide resident strike after doctor sacked at IGMC Shimla</t>
         </is>
       </c>
       <c r="T30" s="2" t="inlineStr">
         <is>
-          <t>2–4 emergency duties a month per resident (official duty roster, 2024). State rule since Dec 2025: max 12 hours per shift.</t>
+          <t>2–4 emergency duties a month (2024); max 12 h shifts</t>
         </is>
       </c>
       <c r="U30" s="2" t="inlineStr"/>
@@ -3306,7 +3178,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>2 years (incl. 1 year field posting) · ₹40,00,000 · leaving: ₹10,00,000 + 18% p.a. interest + stipend drawn</t>
+          <t>2 years incl. 1-year field posting; ₹40 lakh; leaving: ₹10 lakh + 18% interest + stipend</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -3314,14 +3186,14 @@
           <t>₹40,000</t>
         </is>
       </c>
-      <c r="N31" s="6" t="inlineStr">
-        <is>
-          <t>Medium — only the hospital website claims them</t>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency, Burns, Pain clinic</t>
+          <t>Kidney (dialysis), Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="P31" s="3" t="inlineStr">
@@ -3337,12 +3209,12 @@
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>Nothing about this college itself. All Himachal residents went on strike in Dec 2025 after a doctor was sacked at IGMC Shimla. (news)</t>
+          <t>Dec 2025: state-wide resident strike after doctor sacked at IGMC Shimla</t>
         </is>
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>State rule since Dec 2025: residents work max 12 hours per shift. No hospital roster found. (news)</t>
+          <t>Max 12 h per shift (state rule since Dec 2025)</t>
         </is>
       </c>
       <c r="U31" s="2" t="inlineStr"/>
@@ -3380,7 +3252,7 @@
       <c r="R32" s="2" t="inlineStr"/>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>Nothing bad found about residents. Hospital was fined ₹10 lakh in 2025 for a patient-care case (news).</t>
+          <t>2025: hospital fined ₹10 lakh over a patient-care case</t>
         </is>
       </c>
       <c r="T32" s="2" t="inlineStr"/>
@@ -3438,24 +3310,20 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L33" s="2" t="inlineStr"/>
       <c r="M33" s="2" t="inlineStr">
         <is>
           <t>₹35,000</t>
         </is>
       </c>
-      <c r="N33" s="6" t="inlineStr">
-        <is>
-          <t>Medium — only the hospital website claims them</t>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Brain &amp; spine surgery, Kidney transplant, Urology, Trauma &amp; emergency</t>
+          <t>Brain &amp; spine surgery, Kidney transplant, Urology, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr">
@@ -3523,11 +3391,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr">
         <is>
           <t>₹70,000</t>
@@ -3535,12 +3399,12 @@
       </c>
       <c r="N34" s="6" t="inlineStr">
         <is>
-          <t>Medium — only the hospital website claims them</t>
+          <t>Medium — mentioned online, not confirmed</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Brain &amp; spine surgery, Kidney transplant, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency</t>
+          <t>Kidney transplant, Children's surgery, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P34" s="3" t="inlineStr">
@@ -3558,7 +3422,7 @@
       <c r="T34" s="2" t="inlineStr"/>
       <c r="U34" s="2" t="inlineStr">
         <is>
-          <t>y resident-level review is one 2020 AmbitionBox entry by an ICU 'Resident Medical Officer' (5/5, 'grecian support a lot', rotational schedule with flexible timings) - a s</t>
+          <t>Rotational ICU schedule, flexible timings (2020)</t>
         </is>
       </c>
     </row>
@@ -3614,11 +3478,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr">
         <is>
           <t>₹67,968</t>
@@ -3641,7 +3501,7 @@
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>No resident account, but SPS has the largest anaesthesia cohort in this list - DNB Anaesthesia 4 post-MBBS + 4 post-diploma seats, plus DrNB Critical Care (2), DrNB Neurology, IDCCM/IFCCM and emergency-medicine fellowships - and its academics page names the four current anaesthesia trainees. 350-bed NABH hospital with cardiology, neurosciences and critical care. Meducate has no review text for it.</t>
+          <t>8 DNB seats/yr (4 + 4 post-diploma); 350 beds; cardiac, neuro, critical care</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
@@ -3705,11 +3565,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr">
         <is>
           <t>₹76,000</t>
@@ -3732,7 +3588,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>No trainee account found. Officially Livasa (formerly Ivy) Mohali is NBEMS-accredited for DNB in Anaesthesiology, Cardiology and Radiodiagnosis; the DNB Anaesthesiology / DrNB Critical Care programme director is the hospital's Director of Critical Care Medicine, which suggests an ICU-weighted programme. The hospital (227 beds per NBEMS data) publicises CABG/valve surgery, 500+ neuro-navigation surgeries, thrombectomy, aneurysm coiling and awake craniotomy, and the anaesthesia page lists nerve blocks, difficult-airway work and radiofrequency ablation - but no OT count, case numbers or resident testimony.</t>
+          <t>227 beds; cardiac and neurosurgery; nerve blocks, difficult airway; director heads critical care</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
@@ -3796,11 +3652,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
           <t>₹67,968</t>
@@ -3823,7 +3675,7 @@
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>Two named DNB anaesthesia residents (Dr Gokkulavani T, Dr Gazi Mahveen Tasaduq) give testimonials on the hospital's own academic site: 'hands-on experience and interactive discussions... exposed to a wide range of cases... regular academic sessions and workshops'. These are hospital-curated and near-identical in wording, so weak as independent evidence, but they confirm anaesthesia residents are in place (2 per intake per the DNB trainee list). 300-bed hospital (Meducate) with orthopaedics, oncology (radiation oncology DNB), respiratory medicine and radiology programmes.</t>
+          <t>Wide range of cases, workshops; 2 seats/yr; 300 beds</t>
         </is>
       </c>
       <c r="R37" s="6" t="inlineStr">
@@ -3833,7 +3685,7 @@
       </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
-          <t>Nothing bad found for 2019–26. Old case: in 2007 it took a DNB resident while its accreditation had lapsed; court ordered ₹5 lakh compensation in 2018. (court record)</t>
+          <t>2007: took DNB resident during lapsed accreditation; ₹5 lakh compensation ordered 2018</t>
         </is>
       </c>
       <c r="T37" s="2" t="inlineStr"/>
@@ -3891,11 +3743,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr">
         <is>
           <t>₹68,000</t>
@@ -3918,7 +3766,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>No Ludhiana-specific resident account. Fortis Ludhiana is a small unit (175 beds per Meducate; 2 DNB specialities, 6 seats per formity) with cardiac sciences, neurosciences, oncology and an 8-bed NICU. The Fortis group DNB page promises supervised hands-on work, journal clubs, audits and mock tests, generically. The only Fortis DNB-resident voices (AmbitionBox, 2 reviews, Mohali and Bengaluru, 2022) say 'good exposure, variety of cases' and 'good infrastructure... only few people have powers rather than a system'.</t>
+          <t>175 beds; cardiac, neuro, oncology; journal clubs, audits, mock tests</t>
         </is>
       </c>
       <c r="R38" s="6" t="inlineStr">
@@ -3980,11 +3828,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L39" s="2" t="inlineStr"/>
       <c r="M39" s="2" t="inlineStr">
         <is>
           <t>₹76,000</t>
@@ -3997,7 +3841,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
       <c r="P39" s="3" t="inlineStr">
@@ -4007,7 +3851,7 @@
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>200-bed flagship of the Amandeep group, running DNB anaesthesia as a joint programme with Amandeep Medicity as secondary hospital (4 seats). The earlier pass recorded institutional claims of USG- and PNS-guided blocks, paediatric regional, TIVA, fibreoptic/video-laryngoscope intubation, POCUS and simulation; this pass could not re-locate that page (the hospital's DNB course URLs now return empty pages) and found no resident account. The group markets itself as a joint-replacement centre, which implies an orthopaedic, regional-anaesthesia-heavy case mix; the plastic-surgery DNB page shows daily morning academic sessions for trainees.</t>
+          <t>200 beds, 4 seats; USG/PNS blocks, TIVA, POCUS, simulation; joint-replacement focus</t>
         </is>
       </c>
       <c r="R39" s="6" t="inlineStr">
@@ -4019,7 +3863,7 @@
       <c r="T39" s="2" t="inlineStr"/>
       <c r="U39" s="2" t="inlineStr">
         <is>
-          <t>PGs rotate through several ICUs (respiratory, cardiac, neuro, septic). How long is not stated. (hospital website)</t>
+          <t>Rotations through respiratory, cardiac, neuro and septic ICUs</t>
         </is>
       </c>
     </row>
@@ -4075,11 +3919,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr">
         <is>
           <t>₹45,000</t>
@@ -4102,7 +3942,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>Not found online beyond the hospital's own marketing. In 2025 8 DNB anaesthesia seats were allotted (3 retained, 2 upgraded, 3 not reported per Formity), so about 8 trainees share a 158-bed hospital's case load.</t>
+          <t>8 seats allotted in 2025 in a 158-bed hospital</t>
         </is>
       </c>
       <c r="R40" s="6" t="inlineStr">
@@ -4166,11 +4006,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr">
         <is>
           <t>₹45,000</t>
@@ -4193,7 +4029,7 @@
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>Ivy Amritsar has been rebranded Livasa Hospital. The group's academic page (official) says it is NBE-recognised for DNB Anaesthesiology, Radiodiagnosis and Cardiology and names three DNB-qualified anaesthesia faculty (Dr Rajiv Dhunna - also programme director for DrNB critical care per LinkedIn - Dr Shalini S, Dr Sunny Rupal), though the page text refers to 'Livasa Hospital, Mohali' so unit-level detail is unclear. 180 beds (aggregator). No resident account found.</t>
+          <t>180 beds; three DNB-qualified anaesthesia faculty</t>
         </is>
       </c>
       <c r="R41" s="6" t="inlineStr">
@@ -4203,7 +4039,7 @@
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t>Nothing about residents. Staff reviews (2020–21) complain of unpaid salary and no job security. (job-review site)</t>
+          <t>Staff complaints of unpaid salary, no job security (2020–21)</t>
         </is>
       </c>
       <c r="T41" s="2" t="inlineStr"/>
@@ -4261,11 +4097,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr">
         <is>
           <t>₹76,000</t>
@@ -4348,7 +4180,7 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>1 year (AIQ); 2 years (State fresh candidates) · ₹10,00,000 (AIQ); ₹15,00,000 (State fresh candidates) · leaving: balance fee for the whole course (bond/bank guarantee may be sought)</t>
+          <t>AIQ: 1 yr, ₹10 lakh; state fresh: 2 yrs, ₹15 lakh; leaving: full-course fee balance</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
@@ -4358,7 +4190,7 @@
       </c>
       <c r="N43" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr">
@@ -4379,7 +4211,7 @@
       </c>
       <c r="S43" s="2" t="inlineStr">
         <is>
-          <t>Sep 2024: government doctors' strike shut the OPD. July 2025: 3 patients died after an oxygen fault; an anaesthetist was suspended. Nothing about PGs. (news)</t>
+          <t>Sep 2024 doctors' strike shut OPD; Jul 2025: 3 deaths after oxygen fault, anaesthetist suspended</t>
         </is>
       </c>
       <c r="T43" s="2" t="inlineStr"/>
@@ -4437,11 +4269,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr">
         <is>
           <t>₹76,000</t>
@@ -4464,7 +4292,7 @@
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>One first-hand account exists: a 2022 first-batch DNB/DA anaesthesia resident (Dr Rahul Marakana, LinkedIn, 2025) reports 60-70 adult + paediatric cardiac cases/month with 'full hands-on exposure', 300+ general surgeries/month (spine, ortho, gynae, trauma, paeds, high-risk), non-OR anaesthesia (MRI/CT/scopy/ECT), vascular and cath-lab work, and training in a 50+ bed Level-3 closed ICU (ventilation, sepsis, haemodynamics, CRRT/ECMO basics). Tone is strongly positive and the hospital's HR replied under it, so treat as a single enthusiastic (possibly curated) testimonial; NBEMS accredits 3 DNB specialities + DA here and a DNB Cardiothoracic (6-yr) seat is also listed, which supports the cardiac claim.</t>
+          <t>60–70 cardiac cases/month, 300+ surgeries/month; non-OR and cath-lab work (2022)</t>
         </is>
       </c>
       <c r="R44" s="6" t="inlineStr">
@@ -4474,7 +4302,11 @@
       </c>
       <c r="S44" s="2" t="inlineStr"/>
       <c r="T44" s="2" t="inlineStr"/>
-      <c r="U44" s="2" t="inlineStr"/>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>50+ bed Level-3 closed ICU; ventilation, sepsis, CRRT/ECMO basics</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4536,12 +4368,12 @@
       </c>
       <c r="N45" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Brain &amp; spine surgery, Children's surgery, Trauma &amp; emergency</t>
+          <t>Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P45" s="3" t="inlineStr">
@@ -4558,12 +4390,12 @@
       <c r="S45" s="2" t="inlineStr"/>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t>OT 8 am–2 pm. 1st–2nd year: 3–4 night calls a month, 18 hours each. 3rd year: 4–5 calls of 8 hours. (one resident, 2021)</t>
+          <t>OT 8 am–2 pm; yr 1–2: 3–4 18-h calls/month; yr 3: 4–5 8-h calls</t>
         </is>
       </c>
       <c r="U45" s="2" t="inlineStr">
         <is>
-          <t>2 months a year in ICU, plus 1 month at Raipur medical college and 1 month in cardiac OT. (one resident, 2021)</t>
+          <t>2 months ICU/year; also 1 month cardiac OT, 1 month Raipur medical college</t>
         </is>
       </c>
     </row>
@@ -4617,24 +4449,20 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr">
         <is>
           <t>₹50,000</t>
         </is>
       </c>
-      <c r="N46" s="6" t="inlineStr">
-        <is>
-          <t>Medium — only the hospital website claims them</t>
+      <c r="N46" s="3" t="inlineStr">
+        <is>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns</t>
+          <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P46" s="3" t="inlineStr">
@@ -4704,11 +4532,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr">
         <is>
           <t>₹67,500</t>
@@ -4731,7 +4555,7 @@
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>No resident account (neetlogiq empty, AmbitionBox has no Narayana DNB-resident reviews, no Reddit hit). Officially a Narayana Health unit since 2011 with cardiac sciences, cancer (LINAC), neurosciences, robotic surgery, solid-organ and bone-marrow transplant, ECMO and cath lab - but only '105+ advanced care beds' / 265 beds (Meducate) and 70+ consultants, so it is a mid-size tertiary unit. Do not confuse with Shree Narayana Hospital, Raipur (a different DNB hospital).</t>
+          <t>265 beds; cardiac, cancer, neuro, robotic, transplant, ECMO, cath lab</t>
         </is>
       </c>
       <c r="R47" s="6" t="inlineStr">
@@ -4801,7 +4625,7 @@
       </c>
       <c r="N48" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
@@ -4822,7 +4646,7 @@
       </c>
       <c r="S48" s="2" t="inlineStr">
         <is>
-          <t>Aug 2026: interns and PGs struck over unpaid stipend. Sep 2026: junior doctors threatened to stop OPD. Aug 2025: an MBBS student (not a PG) died by suicide. (news)</t>
+          <t>Aug 2026: PG stipend strike; Sep 2026 OPD-stop threat; Aug 2025 MBBS student suicide</t>
         </is>
       </c>
       <c r="T48" s="2" t="inlineStr"/>
@@ -4880,11 +4704,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L49" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr">
         <is>
           <t>₹52,000</t>
@@ -4907,7 +4727,7 @@
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>Official DNB page: 983-bed NABH hospital, 76 critical-care/ICU beds plus separate cardiac CCU, PICU, NICU and burns unit, 13 modular OTs with a PACU, and 'academic rotations in superspecialities' incl. cardiology, critical care, neurosurgery, neuroanaesthesia, onco-surgery, plastic and paediatric surgery; anaesthesia DNB since 1999 (2 primary + 2 secondary seats/yr), FNB critical care since 2013, interventional pain procedures in the main OT. Resident evidence is mixed: AmbitionBox DNB residents (3 reviews, 4.8/5) praise an 'excellent academic environment and work culture', while a DNB-medicine forum post says first-year residents do 'all the clerical work and blood sampling which isn't the case with other DNB institutes'.</t>
+          <t>983 beds, 13 OTs; first-year DNBs do clerical work and blood sampling</t>
         </is>
       </c>
       <c r="R49" s="3" t="inlineStr">
@@ -4917,11 +4737,15 @@
       </c>
       <c r="S49" s="2" t="inlineStr">
         <is>
-          <t>Junior doctors' reviews (2023, 2025) say 'toxic environment, poor work-life balance, too few staff'. A student at the linked medical college died by suicide in Aug 2025. (job-review site + news)</t>
+          <t>Toxic environment, understaffing (2023, 2025); Aug 2025 linked-college student suicide</t>
         </is>
       </c>
       <c r="T49" s="2" t="inlineStr"/>
-      <c r="U49" s="2" t="inlineStr"/>
+      <c r="U49" s="2" t="inlineStr">
+        <is>
+          <t>76 ICU beds plus CCU, PICU, NICU, burns unit</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4975,11 +4799,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L50" s="2" t="inlineStr"/>
       <c r="M50" s="2" t="inlineStr">
         <is>
           <t>₹53,000</t>
@@ -4987,7 +4807,7 @@
       </c>
       <c r="N50" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr">
@@ -5062,11 +4882,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L51" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr">
         <is>
           <t>₹68,000</t>
@@ -5162,7 +4978,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
+          <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Cancer surgery, Newborn / child ICU, Burns</t>
         </is>
       </c>
       <c r="P52" s="7" t="inlineStr">
@@ -5178,7 +4994,7 @@
       </c>
       <c r="S52" s="2" t="inlineStr">
         <is>
-          <t>March 2025: a 1st-year DNB resident (Obs &amp; Gynae) died by suicide in the hostel. Her note mentioned unhappiness with the course. (news)</t>
+          <t>Mar 2025: 1st-year DNB OBG resident suicide in hostel; note cited the course</t>
         </is>
       </c>
       <c r="T52" s="2" t="inlineStr"/>
@@ -5236,11 +5052,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L53" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr">
         <is>
           <t>₹53,000</t>
@@ -5269,7 +5081,7 @@
       </c>
       <c r="S53" s="2" t="inlineStr">
         <is>
-          <t>Nothing bad found about PGs. April 2025: a staff member (not a resident) died by suicide off campus. (news)</t>
+          <t>Apr 2025: staff member (not resident) suicide off campus</t>
         </is>
       </c>
       <c r="T53" s="2" t="inlineStr"/>
@@ -5327,11 +5139,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr">
         <is>
           <t>₹55,000</t>
@@ -5414,11 +5222,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L55" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L55" s="2" t="inlineStr"/>
       <c r="M55" s="2" t="inlineStr">
         <is>
           <t>₹58,000</t>
@@ -5501,11 +5305,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L56" s="2" t="inlineStr"/>
       <c r="M56" s="2" t="inlineStr">
         <is>
           <t>₹45,000</t>
@@ -5588,11 +5388,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L57" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr">
         <is>
           <t>₹56,250</t>
@@ -5675,11 +5471,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L58" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr">
         <is>
           <t>₹45,000</t>
@@ -5705,7 +5497,7 @@
       <c r="S58" s="2" t="inlineStr"/>
       <c r="T58" s="2" t="inlineStr">
         <is>
-          <t>8-hour shifts, 6–7 night duties a month, day off after a night — but this is from a radiology resident, not anaesthesia. (resident post)</t>
+          <t>8-h shifts, 6–7 nights/month, day off after night (radiology)</t>
         </is>
       </c>
       <c r="U58" s="2" t="inlineStr"/>
@@ -5762,11 +5554,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L59" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L59" s="2" t="inlineStr"/>
       <c r="M59" s="2" t="inlineStr">
         <is>
           <t>₹56,250</t>
@@ -5855,7 +5643,7 @@
       </c>
       <c r="N60" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O60" s="2" t="inlineStr"/>
@@ -5866,7 +5654,7 @@
       </c>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t>Aggregator review (anecdotal/templated): 'balanced mix of structured academics and hands-on exposure'; 'manageable patient loads'.</t>
+          <t>Balanced academics and hands-on; manageable patient load</t>
         </is>
       </c>
       <c r="R60" s="6" t="inlineStr">
@@ -5876,7 +5664,7 @@
       </c>
       <c r="S60" s="2" t="inlineStr">
         <is>
-          <t>Nothing bad found about PGs. June 2025: data-entry staff protested late salary. (news)</t>
+          <t>June 2025: data-entry staff protested late salary</t>
         </is>
       </c>
       <c r="T60" s="2" t="inlineStr"/>
@@ -5934,11 +5722,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L61" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L61" s="2" t="inlineStr"/>
       <c r="M61" s="2" t="inlineStr">
         <is>
           <t>₹56,250</t>
@@ -5946,7 +5730,7 @@
       </c>
       <c r="N61" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O61" s="2" t="inlineStr">
@@ -6019,11 +5803,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L62" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="2" t="inlineStr">
         <is>
           <t>₹35,000</t>
@@ -6031,7 +5811,7 @@
       </c>
       <c r="N62" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O62" s="2" t="inlineStr">
@@ -6106,24 +5886,20 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L63" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr">
         <is>
           <t>₹40,000</t>
         </is>
       </c>
-      <c r="N63" s="6" t="inlineStr">
-        <is>
-          <t>Medium — only the hospital website claims them</t>
+      <c r="N63" s="3" t="inlineStr">
+        <is>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
+          <t>Heart surgery, Cardiology</t>
         </is>
       </c>
       <c r="P63" s="3" t="inlineStr">
@@ -6193,11 +5969,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L64" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L64" s="2" t="inlineStr"/>
       <c r="M64" s="2" t="inlineStr">
         <is>
           <t>₹56,250</t>
@@ -6220,7 +5992,7 @@
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>228-bed NABH/NABL hospital with 8 OTs (aggregator) in the Narayana Health group, with on-site 'Cardiac Sciences' and 'Neuro Sciences' centres, an 18-bed dialysis unit and 20 'advanced care' beds (official page; the unit began as Sahyadri Narayana Hrudayalaya, a cardiac hospital). The aggregator review is generic ('broad clinical exposure across OPD, IPD, emergency, ICUs, OTs and super-specialty rotations'); group-level AmbitionBox resident reviews (2) rate skill development 5/5. No Shimoga-specific anaesthesia-resident account.</t>
+          <t>228 beds, 8 OTs; cardiac and neuro centres; broad exposure</t>
         </is>
       </c>
       <c r="R64" s="6" t="inlineStr">
@@ -6286,7 +6058,7 @@
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>1 year · ₹20,00,000 · leaving: ₹20,00,000</t>
+          <t>1 year; ₹20 lakh; leaving: ₹20 lakh</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
@@ -6296,7 +6068,7 @@
       </c>
       <c r="N65" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O65" s="2" t="inlineStr">
@@ -6311,7 +6083,7 @@
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>Aggregator review (anecdotal/templated): involvement in deliveries, neonatal care, emergency procedures and routine surgeries under supervision; high OPD load.</t>
+          <t>Deliveries, emergency procedures, routine surgeries under supervision; high OPD load</t>
         </is>
       </c>
       <c r="R65" s="6" t="inlineStr">
@@ -6373,11 +6145,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L66" s="2" t="inlineStr"/>
       <c r="M66" s="2" t="inlineStr">
         <is>
           <t>₹56,250</t>
@@ -6460,11 +6228,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L67" s="2" t="inlineStr"/>
       <c r="M67" s="2" t="inlineStr">
         <is>
           <t>₹56,250</t>
@@ -6547,11 +6311,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L68" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L68" s="2" t="inlineStr"/>
       <c r="M68" s="2" t="inlineStr">
         <is>
           <t>₹45,000</t>
@@ -6582,7 +6342,7 @@
       <c r="T68" s="2" t="inlineStr"/>
       <c r="U68" s="2" t="inlineStr">
         <is>
-          <t>Department runs neuro, cardiac and liver-transplant ICUs. Posting length not stated. (hospital website)</t>
+          <t>Neuro, cardiac and liver-transplant ICUs</t>
         </is>
       </c>
     </row>
@@ -6638,11 +6398,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L69" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L69" s="2" t="inlineStr"/>
       <c r="M69" s="2" t="inlineStr">
         <is>
           <t>₹35,000</t>
@@ -6665,7 +6421,7 @@
       </c>
       <c r="Q69" s="2" t="inlineStr">
         <is>
-          <t>The one non-templated review text in this set: Meducate's highlights for Apollo Madurai say 'DNB students get access to advanced clinical scenarios, particularly in oncology and critical care. Academics are well-structured. Surgical hands-on is consultant-led and sometimes limited. Ideal for residents focused on academics and sub-specialty exposure.' Unsigned, so weak, but it is the only explicit statement on hands-on limits found for any of these hospitals. 300-bed Apollo unit (est. 1997) with cardiac sciences, neurosciences, oncology, transplant and interventional radiology; 4 DNB specialities, 12 seats.</t>
+          <t>Surgical hands-on consultant-led, sometimes limited; strong oncology, critical care; 300 beds</t>
         </is>
       </c>
       <c r="R69" s="6" t="inlineStr">
@@ -6727,11 +6483,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L70" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L70" s="2" t="inlineStr"/>
       <c r="M70" s="2" t="inlineStr">
         <is>
           <t>₹50,923</t>
@@ -6754,7 +6506,7 @@
       </c>
       <c r="Q70" s="2" t="inlineStr">
         <is>
-          <t>No resident account; Meducate has no page. Billroth (Shenoy Nagar) is a 330-bed Chennai hospital (NeetVantage) advertising a multi-organ transplant institute (heart, liver, lung, kidney, hand), cardiac surgery, neurosurgery and critical care; only 2 DNB courses here (anaesthesia, radiology). AmbitionBox has 9 'Duty Medical Officer' reviews - the closest thing to a junior-doctor voice - split between 'skills development' and 'simply waste / management'.</t>
+          <t>330 beds; multi-organ transplant, cardiac surgery, neurosurgery, critical care</t>
         </is>
       </c>
       <c r="R70" s="6" t="inlineStr">
@@ -6816,11 +6568,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L71" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L71" s="2" t="inlineStr"/>
       <c r="M71" s="2" t="inlineStr">
         <is>
           <t>₹50,000</t>
@@ -6843,7 +6591,7 @@
       </c>
       <c r="Q71" s="2" t="inlineStr">
         <is>
-          <t>No resident account, but two non-templated hints: Meducate's highlights say 'Moderate patient volume... Academics present but not highly structured. Hands-on procedural work is possible but depends on initiative. Suitable for those wanting to train in a smaller hospital environment', and an AmbitionBox DMO (Jan 2024) calls it 'a great training ground... working in all departments'. Officially 425 beds, 10,000 surgeries/yr, cath lab, renal transplant centre, MICU/CCU; no cardiac surgery or neurosurgery programme is listed.</t>
+          <t>Hands-on possible but depends on initiative; 425 beds, 10,000 surgeries/yr; no cardiac/neurosurgery</t>
         </is>
       </c>
       <c r="R71" s="6" t="inlineStr">
@@ -6907,11 +6655,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L72" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L72" s="2" t="inlineStr"/>
       <c r="M72" s="2" t="inlineStr">
         <is>
           <t>₹39,500</t>
@@ -6934,7 +6678,7 @@
       </c>
       <c r="Q72" s="2" t="inlineStr">
         <is>
-          <t>Nothing from trainees. Directory data list 8 anaesthesiologists, 2 cardiothoracic surgeons, 3 nephrologists and 3 critical-care specialists - a comparatively large anaesthesia team for a 4-speciality, 10-seat DNB hospital. The Hindu (9 Oct 2026) reports the hospital felicitating staff on completing 125 kidney transplants, confirming an active renal transplant programme (the input's Renal/Transplant exposure). A DNB/EDAIC-qualified consultant joined anaesthesia in Aug 2024 (Instagram). No OT count, case numbers or academics page.</t>
+          <t>8 anaesthesiologists; active kidney transplant programme (125 done by Oct 2026)</t>
         </is>
       </c>
       <c r="R72" s="6" t="inlineStr">
@@ -6998,11 +6742,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L73" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L73" s="2" t="inlineStr"/>
       <c r="M73" s="2" t="inlineStr">
         <is>
           <t>₹48,000</t>
@@ -7015,7 +6755,7 @@
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency</t>
+          <t>Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P73" s="3" t="inlineStr">
@@ -7025,7 +6765,7 @@
       </c>
       <c r="Q73" s="2" t="inlineStr">
         <is>
-          <t>60-year-old NABH trust hospital (founded 1965) with about 200-214 beds; recent additions are a NICU, a chemotherapy suite and a kidney-transplant surgery (site banner). The anaesthesia department page is a JavaScript app whose text could not be extracted and the DNB page on jeyasekharanhospital.edu.in is offline. The aggregator review praises 'robust hands-on exposure in labour rooms, emergency care and minor surgical procedures' and supportive faculty, but that is written for medicine/OBG/paediatrics residents, not anaesthesia.</t>
+          <t>~200 beds; NICU, chemotherapy, kidney transplant</t>
         </is>
       </c>
       <c r="R73" s="6" t="inlineStr">
@@ -7089,11 +6829,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L74" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L74" s="2" t="inlineStr"/>
       <c r="M74" s="2" t="inlineStr">
         <is>
           <t>₹50,000</t>
@@ -7106,7 +6842,7 @@
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
+          <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="P74" s="3" t="inlineStr">
@@ -7176,11 +6912,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L75" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L75" s="2" t="inlineStr"/>
       <c r="M75" s="2" t="inlineStr">
         <is>
           <t>₹35,000</t>
@@ -7263,11 +6995,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L76" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L76" s="2" t="inlineStr"/>
       <c r="M76" s="2" t="inlineStr">
         <is>
           <t>₹48,000</t>
@@ -7275,7 +7003,7 @@
       </c>
       <c r="N76" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O76" s="2" t="inlineStr">
@@ -7298,7 +7026,7 @@
       <c r="T76" s="2" t="inlineStr"/>
       <c r="U76" s="2" t="inlineStr">
         <is>
-          <t>10-bed ICU with 1 consultant and 1 resident on duty round the clock. Posting length not stated. (hospital website)</t>
+          <t>10-bed ICU; 1 consultant + 1 resident on duty 24x7</t>
         </is>
       </c>
     </row>
@@ -7354,11 +7082,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L77" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L77" s="2" t="inlineStr"/>
       <c r="M77" s="2" t="inlineStr">
         <is>
           <t>₹51,500</t>
@@ -7381,7 +7105,7 @@
       </c>
       <c r="Q77" s="2" t="inlineStr">
         <is>
-          <t>230-bed unit (aggregator) running DNB Anaesthesiology (post-MBBS and post-diploma) under Apollo's academic programme. One Glassdoor review titled 'DNB residency at Apollo Guwahati' by a DNB resident doctor says 'Brand, patient exposure is good' (only the snippet is readable). No other resident account; DNB Anaesthesiology closing rank 38,993 (2025) vs 31,709 (2024).</t>
+          <t>230 beds; good patient exposure</t>
         </is>
       </c>
       <c r="R77" s="3" t="inlineStr">
@@ -7391,7 +7115,7 @@
       </c>
       <c r="S77" s="2" t="inlineStr">
         <is>
-          <t>June 2026: senior doctors stopped OPD and planned surgery for 2 days, saying management humiliated them. (news)</t>
+          <t>June 2026: senior doctors stopped OPD, surgery 2 days over management humiliation</t>
         </is>
       </c>
       <c r="T77" s="2" t="inlineStr"/>
@@ -7449,11 +7173,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L78" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L78" s="2" t="inlineStr"/>
       <c r="M78" s="2" t="inlineStr">
         <is>
           <t>₹52,000</t>
@@ -7536,11 +7256,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L79" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L79" s="2" t="inlineStr"/>
       <c r="M79" s="2" t="inlineStr">
         <is>
           <t>₹48,000</t>
@@ -7553,7 +7269,7 @@
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P79" s="3" t="inlineStr">
@@ -7621,11 +7337,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L80" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L80" s="2" t="inlineStr"/>
       <c r="M80" s="2" t="inlineStr">
         <is>
           <t>₹49,000</t>
@@ -7648,7 +7360,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>5 OTs + burn OT in a 100-bed hospital - modest volume. No resident account found.</t>
+          <t>100 beds, 5 OTs + burn OT; modest volume</t>
         </is>
       </c>
       <c r="R80" s="4" t="inlineStr">
@@ -7658,7 +7370,7 @@
       </c>
       <c r="S80" s="2" t="inlineStr">
         <is>
-          <t>Sep 2026: an ICU doctor (staff, not a PG) died by suicide on duty. Family blamed personal harassment, not the hospital. (news)</t>
+          <t>Sep 2026: staff ICU doctor (not PG) suicide on duty; family blamed personal harassment</t>
         </is>
       </c>
       <c r="T80" s="2" t="inlineStr"/>
@@ -7714,11 +7426,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L81" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="2" t="inlineStr">
         <is>
           <t>₹72,100</t>
@@ -7741,7 +7449,7 @@
       </c>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>200-bed private hospital (neetvantage) whose academics page lists DNB Anaesthesiology alongside DNB/DrNB programmes in neurosurgery and others; the anaesthesia faculty block shows MD/DNB anaesthetists including FNB (Critical Care) and DrNB (Critical Care) qualified consultants and a paediatric-anaesthesia fellow, a 'Neuro Anaesthesia' service, and a GI &amp; liver-transplant unit with its own critical-care/anaesthesia consultant (ex-PGIMER/ILBS, per LinkedIn). No resident account of what DNB trainees actually do, and no OT/case numbers published.</t>
+          <t>200 beds; neuro-anaesthesia, paeds anaesthesia, liver transplant; critical-care-trained faculty</t>
         </is>
       </c>
       <c r="R81" s="3" t="inlineStr">
@@ -7751,7 +7459,7 @@
       </c>
       <c r="S81" s="2" t="inlineStr">
         <is>
-          <t>Aug 2025: a nurse died by suicide at the hospital; staff alleged harassment by seniors and a cover-up. Nothing about PGs. (news)</t>
+          <t>Aug 2025: nurse suicide; staff alleged harassment by seniors, cover-up</t>
         </is>
       </c>
       <c r="T81" s="2" t="inlineStr"/>
@@ -7809,11 +7517,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L82" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L82" s="2" t="inlineStr"/>
       <c r="M82" s="2" t="inlineStr">
         <is>
           <t>₹90,000</t>
@@ -7836,7 +7540,7 @@
       </c>
       <c r="Q82" s="2" t="inlineStr">
         <is>
-          <t>The hospital publishes an NBEMS-style DNB FAQ (Aug 2026): 307 beds, NABH+NABL, 21 accredited programmes incl. DrNB Neurosurgery and DrNB Critical Care and FNB Trauma - so neuro and ICU exposure is structurally present; anaesthesia has 1 post-MBBS + 1 post-diploma seat. The hospital posts its own resident-testimonial videos ('DNB doctors share their experience', farewell batch 2026) - hospital-curated, not independent. No third-party resident account found.</t>
+          <t>307 beds; DrNB neurosurgery, critical care, trauma on site; 1 + 1 seats</t>
         </is>
       </c>
       <c r="R82" s="6" t="inlineStr">
@@ -7900,11 +7604,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L83" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L83" s="2" t="inlineStr"/>
       <c r="M83" s="2" t="inlineStr">
         <is>
           <t>₹50,000</t>
@@ -7917,7 +7617,7 @@
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns</t>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P83" s="6" t="inlineStr">
@@ -7927,7 +7627,7 @@
       </c>
       <c r="Q83" s="2" t="inlineStr">
         <is>
-          <t>High laparoscopic and renal-transplant volumes claimed by hospital; anaesthesiology listed as a centre of excellence. No resident account found.</t>
+          <t>High laparoscopic and renal-transplant volumes; anaesthesia a centre of excellence</t>
         </is>
       </c>
       <c r="R83" s="6" t="inlineStr">
@@ -7937,7 +7637,7 @@
       </c>
       <c r="S83" s="2" t="inlineStr">
         <is>
-          <t>Manipur ethnic conflict since May 2023 with deaths, displacement, internet blackouts and President's Rule</t>
+          <t>Manipur ethnic conflict since May 2023; internet blackouts, President's Rule</t>
         </is>
       </c>
       <c r="T83" s="2" t="inlineStr"/>
@@ -7993,11 +7693,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L84" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L84" s="2" t="inlineStr"/>
       <c r="M84" s="2" t="inlineStr">
         <is>
           <t>₹60,823</t>
@@ -8020,7 +7716,7 @@
       </c>
       <c r="Q84" s="2" t="inlineStr">
         <is>
-          <t>Nothing from residents. The hospital is large (listings say 650-700 beds, NABH) with cath labs, 'advanced ICUs', kidney and liver transplant surgeons, neurosurgery and robotic surgeons on the roster, and 13 DNB seats across 4 specialities (formity). Its anaesthesiology page is patient-facing marketing with no training content; Meducate has no page for this unit. A LinkedIn profile of a 'DNB resident PGY1' at Medicover Vizag exists but says nothing about training.</t>
+          <t>650–700 beds; cath labs, ICUs, kidney/liver transplant, neurosurgery, robotic surgery</t>
         </is>
       </c>
       <c r="R84" s="6" t="inlineStr">
@@ -8030,7 +7726,7 @@
       </c>
       <c r="S84" s="2" t="inlineStr">
         <is>
-          <t>Corporate chain whose own staff reviews mention unpaid overtime and politics (non-resident, group-wide).</t>
+          <t>Group staff complaints: unpaid overtime, politics</t>
         </is>
       </c>
       <c r="T84" s="2" t="inlineStr"/>
@@ -8088,11 +7784,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L85" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L85" s="2" t="inlineStr"/>
       <c r="M85" s="2" t="inlineStr">
         <is>
           <t>₹48,000</t>
@@ -8100,7 +7792,7 @@
       </c>
       <c r="N85" s="3" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="O85" s="2" t="inlineStr">
@@ -8115,7 +7807,7 @@
       </c>
       <c r="Q85" s="2" t="inlineStr">
         <is>
-          <t>Nothing hospital-specific from residents. Apollo Nellore is a ~200-bed unit (MyHospitalNow listing) with a cardiology/cardiac-surgery centre ('modern operating theatres, advanced anaesthesia, and critical care support... complex heart surgeries' per Apollo's own page) and a critical-care department; anaesthesia is its only DNB speciality (2 seats). The only resident voices are AmbitionBox 'DNB Resident' reviews of Apollo Hospitals as a group (6 reviews, other cities): 'best exposure for DNB resident' / 'get exposure to latest technologies and good training opportunities' - not Nellore.</t>
+          <t>~200 beds; cardiac surgery, critical care; anaesthesia only DNB, 2 seats</t>
         </is>
       </c>
       <c r="R85" s="6" t="inlineStr">
@@ -8125,7 +7817,7 @@
       </c>
       <c r="S85" s="2" t="inlineStr">
         <is>
-          <t>Group-wide resident reviews mention 'target oriented practice', 'politics', and one unpaid-salary complaint.</t>
+          <t>Group-wide: target-driven practice, politics, one unpaid-salary complaint</t>
         </is>
       </c>
       <c r="T85" s="2" t="inlineStr"/>
@@ -8183,11 +7875,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L86" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L86" s="2" t="inlineStr"/>
       <c r="M86" s="2" t="inlineStr">
         <is>
           <t>₹37,000</t>
@@ -8270,11 +7958,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L87" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L87" s="2" t="inlineStr"/>
       <c r="M87" s="2" t="inlineStr">
         <is>
           <t>₹60,000</t>
@@ -8297,7 +7981,7 @@
       </c>
       <c r="Q87" s="2" t="inlineStr">
         <is>
-          <t>No resident account found. KIMS-Saveera is a 300-bed (site) / 250-bed (NBEMS listing) hospital in Anantapur with cardiology, CTVS, neurosurgery, nephrology/urology and an Emergency &amp; Critical Care department; the hospital's own Facebook page advertised the anaesthesia DNB programme in 2021 and periodic consultant hires. Meducate's templated blurb says 'hands-on training is strengthened by experience in critical care, trauma management, NICU services' - not a resident voice.</t>
+          <t>250–300 beds; CTVS, neurosurgery, nephrology/urology, emergency and critical care</t>
         </is>
       </c>
       <c r="R87" s="6" t="inlineStr">
@@ -8361,11 +8045,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L88" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L88" s="2" t="inlineStr"/>
       <c r="M88" s="2" t="inlineStr">
         <is>
           <t>₹60,823</t>
@@ -8388,7 +8068,7 @@
       </c>
       <c r="Q88" s="2" t="inlineStr">
         <is>
-          <t>No resident or alumni account of DNB anaesthesia training found (no Reddit/Quora/forum post names this hospital). The only 'review' is a counselling-site blurb (Meducate) that reads as templated marketing: 'hands-on training is a key strength... OT, critical care, emergency'. Officially the hospital (now MGM SevenHills, ~300 beds) lists Heart &amp; Lung Transplant, Liver and Kidney Transplant, CTVS, Neurosurgery, Oncology and a 24x7 emergency/critical-care unit, so super-speciality case-mix exists on paper, but nothing says how much of it DNB residents actually do.</t>
+          <t>~300 beds; heart, lung, liver, kidney transplant; CTVS, neurosurgery, oncology</t>
         </is>
       </c>
       <c r="R88" s="6" t="inlineStr">
@@ -8452,11 +8132,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L89" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L89" s="2" t="inlineStr"/>
       <c r="M89" s="2" t="inlineStr">
         <is>
           <t>₹44,075</t>
@@ -8469,7 +8145,7 @@
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency, Pain clinic</t>
+          <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency</t>
         </is>
       </c>
       <c r="P89" s="7" t="inlineStr">
@@ -8539,11 +8215,7 @@
           <t>No bond</t>
         </is>
       </c>
-      <c r="L90" s="2" t="inlineStr">
-        <is>
-          <t>Private DNB hospitals can't take a bond (NBEMS rule)</t>
-        </is>
-      </c>
+      <c r="L90" s="2" t="inlineStr"/>
       <c r="M90" s="2" t="inlineStr">
         <is>
           <t>₹60,900</t>
@@ -8566,7 +8238,7 @@
       </c>
       <c r="Q90" s="2" t="inlineStr">
         <is>
-          <t>No resident account, but the department's own DNB page is unusually specific: anaesthesia for liver and kidney transplant, neurosurgery, neuro-/vascular intervention, thoracic/vascular surgery, labour analgesia and out-of-OT work, with BIS depth monitoring, LiDCO cardiac output and SVV-guided fluids in routine use; DNB running since 2008 (3 anaesthesia seats + 1 diploma). Meducate's templated blurb adds nothing resident-sourced. Lalitha opened a new 600-bed 'Lalitha PVS Institute' campus in June 2026 and says DNB training continues - which campus residents rotate through is not stated.</t>
+          <t>Liver/kidney transplant, neuro, vascular, thoracic, labour analgesia; BIS, LiDCO monitoring; since 2008</t>
         </is>
       </c>
       <c r="R90" s="6" t="inlineStr">
@@ -8904,12 +8576,12 @@
       <c r="A23" s="10" t="inlineStr"/>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Low — little super-speciality work</t>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Very little found.</t>
+          <t>The hospital's website was checked and shows few or no super-speciality departments.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Shortlist: full research for every college (web, website, residents); re-judged the 10 newly researched; refreshed short cells
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -135,10 +135,10 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -652,7 +652,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Runs a cardiac anaesthesia super-speciality course, but nothing else is known about case mix.</t>
+          <t>Cardiac and neuro on paper in a small, young Ahmednagar DNB unit; case load and teaching unproven.</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -682,12 +682,16 @@
           <t>Heart</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr"/>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Small programme: 2 DNB anaesthesia seats (2025)</t>
+        </is>
+      </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -720,7 +724,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Ahmednagar private hospital with no super-speciality courses and no public information on training.</t>
+          <t>Established DNB with a real cardiac surgery load and large ICUs; low fee, no bond.</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -740,15 +744,19 @@
           <t>₹51,000</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Medium — only the hospital website claims them</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
+        </is>
+      </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr"/>
@@ -802,13 +810,17 @@
           <t>₹43,000/month</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Medium — only the hospital website claims them</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
@@ -821,7 +833,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Stipend ₹15,000/month reported vs ₹43,000 declared</t>
+          <t>Stipend may be ₹15,000/month, not the ₹43,000 declared to MCC</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr"/>
@@ -880,18 +892,26 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr"/>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>Poor — residents mostly watch</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Moderate case load; limited independent procedures</t>
+        </is>
+      </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Residents reportedly keep resigning (radiology, Mumbai campus unclear)</t>
+        </is>
+      </c>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
     </row>
@@ -936,15 +956,19 @@
           <t>₹43,000/month</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Medium — only the hospital website claims them</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Trauma &amp; emergency</t>
+        </is>
+      </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
+          <t>Unclear — no resident has said</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>
@@ -980,7 +1004,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Manipal Dwarka offers cardiology, gastro and ICU courses, but no surgical super-speciality is shown.</t>
+          <t>Manipal Dwarka: cardiac, neuro and liver-transplant anaesthesia teams in a 380-bed hospital; no bond.</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -1012,10 +1036,14 @@
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr"/>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Dedicated onco- and cardiac-anaesthesia heads</t>
+        </is>
+      </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -1078,29 +1106,29 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>6 OTs, 210 beds; neuro, cardiothoracic, paeds, gastro, uro and IVF cases</t>
-        </is>
-      </c>
-      <c r="O8" s="6" t="inlineStr">
+          <t>6 OTs, 210 beds; neuro, cardiothoracic, paediatric, gastro, urology, IVF cases</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
         <is>
           <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2017 duty-hours complaint (radiology); ~₹50k stipend called low (2025)</t>
+          <t>2017 complaint over inhuman duty hours (radiology); 2025: ~₹50k stipend called low</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2017: radiology residents worked 32–56 h at a stretch</t>
+          <t>2017: radiology residents worked 32–56 h stretches</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr"/>
@@ -1128,7 +1156,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Established Delhi DNB with strong neuro exposure and a resident-reported free hand in 9 OTs.</t>
+          <t>Busy 600-bed Delhi mission hospital with real hands-on training and good neuro and pain; weak cardiac.</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -1160,7 +1188,7 @@
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr"/>
@@ -1171,12 +1199,12 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2017: radiology PG murdered in hospital duty room</t>
+          <t>2017: a radiology PG was murdered in the duty room</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>OT days plus 6–9 emergency duties a month (2021)</t>
+          <t>Normal OT days plus 6–9 emergency duties a month (2021)</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr"/>
@@ -1236,10 +1264,14 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr"/>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Super-specialty exposure; hands-on varies by specialty</t>
+        </is>
+      </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -1306,14 +1338,14 @@
           <t>Heart, Kidney &amp; transplant, Stomach &amp; liver (GI) surgery</t>
         </is>
       </c>
-      <c r="M11" s="6" t="inlineStr">
+      <c r="M11" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>242 beds; six senior consultant faculty</t>
+          <t>242 beds; six senior anaesthesia consultants</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
@@ -1378,7 +1410,7 @@
           <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="M12" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
@@ -1423,7 +1455,7 @@
         <v>40253</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>Missing — bond not confirmed</t>
         </is>
@@ -1434,18 +1466,22 @@
           <t>₹84,000</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Good — residents say they do cases</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>New college (2022); 4 Asst Profs, 3 SRs; district-hospital case mix</t>
+        </is>
+      </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -1453,7 +1489,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>GMERS group cut junior-doctor pay (2023)</t>
+          <t>GMERS cut junior-doctor pay in 2023; stipend strike at another GMERS college</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr"/>
@@ -1517,7 +1553,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Hands-on OT, ICU, obstetric, pain work and regional blocks; ~100 surgeries/day; started 2025</t>
+          <t>New in 2025; 3 seats, 8 OTs, ~100 surgeries/day; regional blocks, ICU, obstetrics</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
@@ -1586,7 +1622,7 @@
           <t>Heart</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
@@ -1644,13 +1680,13 @@
           <t>₹55,200</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
@@ -1718,14 +1754,14 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr">
-        <is>
-          <t>Some — reported, but not by residents</t>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Satisfactory hands-on, especially orthopaedic and trauma cases</t>
+          <t>Mainly orthopaedic and trauma cases</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
@@ -1764,7 +1800,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Good stipend at Max Lucknow, but no super-speciality courses and possibly a new anaesthesia seat.</t>
+          <t>Ex-Sahara hospital recently taken over by Max; good stipend, but the case mix in Lucknow is unconfirmed.</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
@@ -1782,15 +1818,19 @@
           <t>₹60,000</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>Medium — only the hospital website claims them</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU</t>
+        </is>
+      </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
+          <t>Unclear — no resident has said</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
@@ -1856,14 +1896,14 @@
           <t>Heart, Brain &amp; spine</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr">
-        <is>
-          <t>Some — reported, but not by residents</t>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>Poor — residents mostly watch</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Hands-on may be limited: consultant-led corporate model; 2 seats/yr</t>
+          <t>Strong ICU exposure; procedures mostly consultant-led</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
@@ -1875,7 +1915,7 @@
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>Strong ICU exposure</t>
+          <t>ICU exposure described as strong</t>
         </is>
       </c>
     </row>
@@ -1932,14 +1972,14 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr">
-        <is>
-          <t>Some — reported, but not by residents</t>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>Poor — residents mostly watch</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Strongest in ICU; many procedures consultant-led; 2 (+1) seats/yr</t>
+          <t>Cardiac and neuro critical care; many procedures consultant-led</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
@@ -1951,7 +1991,7 @@
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>Decent ICU exposure; cardiac and neuro ICUs</t>
+          <t>Cardiac and neuro ICUs</t>
         </is>
       </c>
     </row>
@@ -2008,14 +2048,14 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
-      <c r="M21" s="6" t="inlineStr">
+      <c r="M21" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>All types of cases (2022); 8 OTs; transplant, cardiac, neuro, paeds, obstetric anaesthesia</t>
+          <t>All case types; 8 OTs; transplant, cardiac, neuro, paediatric, obstetric; pain clinic</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
@@ -2025,17 +2065,17 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Department called 'very chill' (2022)</t>
+          <t>Department described as 'very chill' (2022)</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>~8 h a day; rest after duty (2022)</t>
+          <t>About 8 h a day; rest after duty (2022)</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>3 ICUs (medical, surgical, cardiac), 60 beds, run by anaesthesia</t>
+          <t>3 ICUs (medical, surgical, cardiac), 60 beds</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2139,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>Hands-on mostly ICU; surgical cases largely consultant-led; 4 OTs</t>
+          <t>4 OTs, ICU, labour analgesia; surgical cases mostly consultant-led</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
@@ -2162,7 +2202,7 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="M23" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
@@ -2220,7 +2260,7 @@
           <t>₹56,100</t>
         </is>
       </c>
-      <c r="K24" s="6" t="inlineStr">
+      <c r="K24" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -2230,12 +2270,16 @@
           <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Burns, Pain clinic</t>
         </is>
       </c>
-      <c r="M24" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N24" s="2" t="inlineStr"/>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>Good — residents say they do cases</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Started 2023, 2 seats; 4 OTs; cardiac, neuro, high-risk obstetric, nerve blocks</t>
+        </is>
+      </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -2302,14 +2346,14 @@
           <t>Kidney &amp; transplant</t>
         </is>
       </c>
-      <c r="M25" s="6" t="inlineStr">
+      <c r="M25" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>New programme (Sept 2025), 3 seats; regional blocks, 24x7 ICU; hands-on depends on consultants</t>
+          <t>New (Sept 2025), 3 seats; regional blocks; moderate exposure, consultant-dependent</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
@@ -2323,7 +2367,11 @@
           <t>Structured working hours</t>
         </is>
       </c>
-      <c r="R25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>24x7 intensivist-run ICU</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2366,13 +2414,17 @@
           <t>₹ 70,000/month</t>
         </is>
       </c>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="5" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Medium — only the hospital website claims them</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
+        </is>
+      </c>
+      <c r="M26" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
@@ -2440,14 +2492,14 @@
           <t>Heart, Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M27" s="6" t="inlineStr">
+      <c r="M27" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>200 beds; HOD experienced in neuro, ortho, onco, paeds cases</t>
+          <t>200 beds; neuro, ortho, onco, paediatric and laparoscopic anaesthesia</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
@@ -2482,7 +2534,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Residents struck in April 2026 after three months of unpaid stipend.</t>
+          <t>Stipend unpaid for months (PG strike April 2026), no super-specialities, and repeated campus turmoil.</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
@@ -2502,19 +2554,23 @@
           <t>₹69,115</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>Medium — mentioned online, not confirmed</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Trauma &amp; emergency</t>
+        </is>
+      </c>
+      <c r="M28" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
       <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="6" t="inlineStr">
+      <c r="O28" s="5" t="inlineStr">
         <is>
           <t>Caution — complaints reported</t>
         </is>
@@ -2582,7 +2638,7 @@
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
+          <t>Unclear — no resident has said</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr"/>
@@ -2632,7 +2688,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>2 years incl. 1-year field posting; ₹40 lakh; leaving: ₹10 lakh + 18% interest + stipend</t>
+          <t>₹40 lakh; leaving: ₹10 lakh + 18% interest + stipend; incl. 1-year field posting</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2640,7 +2696,7 @@
           <t>₹40,000</t>
         </is>
       </c>
-      <c r="K30" s="6" t="inlineStr">
+      <c r="K30" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -2652,23 +2708,27 @@
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N30" s="2" t="inlineStr"/>
-      <c r="O30" s="4" t="inlineStr">
-        <is>
-          <t>OK — nothing bad found online</t>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>5 SRs and 4 DNB residents; structured monthly duty roster</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="inlineStr">
+        <is>
+          <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Dec 2025: state-wide resident strike after doctor sacked at IGMC Shimla</t>
+          <t>Dec 2025: Himachal-wide resident strike after IGMC Shimla doctor sacked</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2–4 emergency duties a month (2024); max 12 h shifts</t>
+          <t>2–4 emergency duties a month; max 12 h shifts</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr"/>
@@ -2710,7 +2770,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>2 years incl. 1-year field posting; ₹40 lakh; leaving: ₹10 lakh + 18% interest + stipend</t>
+          <t>₹40 lakh; leaving: ₹10 lakh + 18% interest + stipend; incl. 1-year field posting</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2718,7 +2778,7 @@
           <t>₹40,000</t>
         </is>
       </c>
-      <c r="K31" s="6" t="inlineStr">
+      <c r="K31" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -2728,12 +2788,16 @@
           <t>Kidney (dialysis), Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M31" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr"/>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>Good — residents say they do cases</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>7 daily OTs incl. emergency and maternity; 13-bed PACU, 10-bed ICU, pain clinic</t>
+        </is>
+      </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -2741,15 +2805,19 @@
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>Dec 2025: state-wide resident strike after doctor sacked at IGMC Shimla</t>
+          <t>Dec 2025: Himachal-wide resident strike after IGMC Shimla doctor sacked</t>
         </is>
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>Max 12 h per shift (state rule since Dec 2025)</t>
-        </is>
-      </c>
-      <c r="R31" s="2" t="inlineStr"/>
+          <t>Max 12 h shifts (state rule since Dec 2025)</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>Own 10-bed ICU</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2830,7 +2898,7 @@
           <t>₹35,000</t>
         </is>
       </c>
-      <c r="K33" s="6" t="inlineStr">
+      <c r="K33" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -2840,12 +2908,16 @@
           <t>Brain &amp; spine surgery, Kidney transplant, Urology, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M33" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr"/>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>Consultants practise USG-guided regional and onco-anaesthesia</t>
+        </is>
+      </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -2906,7 +2978,7 @@
           <t>Kidney transplant, Children's surgery, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M34" s="6" t="inlineStr">
+      <c r="M34" s="5" t="inlineStr">
         <is>
           <t>Unclear — no resident has said</t>
         </is>
@@ -2985,7 +3057,7 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>8 DNB seats/yr (4 + 4 post-diploma); 350 beds; cardiac, neuro, critical care</t>
+          <t>350 beds; 8 DNB anaesthesia seats; cardiology, neuro, critical care</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
@@ -3050,14 +3122,14 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Pain clinic</t>
         </is>
       </c>
-      <c r="M36" s="6" t="inlineStr">
+      <c r="M36" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>227 beds; cardiac and neurosurgery; nerve blocks, difficult airway; director heads critical care</t>
+          <t>227 beds; cardiac surgery, neurosurgery, nerve blocks, difficult airway; ICU-weighted</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
@@ -3122,14 +3194,14 @@
           <t>Cancer</t>
         </is>
       </c>
-      <c r="M37" s="6" t="inlineStr">
+      <c r="M37" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>Wide range of cases, workshops; 2 seats/yr; 300 beds</t>
+          <t>300 beds; 2 seats; wide range of cases, regular workshops</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
@@ -3139,7 +3211,7 @@
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>2007: took DNB resident during lapsed accreditation; ₹5 lakh compensation ordered 2018</t>
+          <t>2007: took a DNB resident during lapsed accreditation; ₹5 lakh compensation (2018)</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr"/>
@@ -3198,14 +3270,14 @@
           <t>Stomach &amp; liver (GI) surgery, Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M38" s="6" t="inlineStr">
+      <c r="M38" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>175 beds; cardiac, neuro, oncology; journal clubs, audits, mock tests</t>
+          <t>175 beds; cardiac, neuro, oncology; Fortis group says supervised hands-on</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
@@ -3268,14 +3340,14 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
         </is>
       </c>
-      <c r="M39" s="6" t="inlineStr">
+      <c r="M39" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>200 beds, 4 seats; USG/PNS blocks, TIVA, POCUS, simulation; joint-replacement focus</t>
+          <t>200 beds, 4 seats; ortho-heavy; USG/PNS blocks, TIVA, fibreoptic, POCUS, simulation</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
@@ -3344,14 +3416,14 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M40" s="4" t="inlineStr">
-        <is>
-          <t>Some — reported, but not by residents</t>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>8 seats allotted in 2025 in a 158-bed hospital</t>
+          <t>158 beds; spinal/epidural, nerve blocks; cardiothoracic and neurosurgery cases</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
@@ -3361,7 +3433,11 @@
       </c>
       <c r="P40" s="2" t="inlineStr"/>
       <c r="Q40" s="2" t="inlineStr"/>
-      <c r="R40" s="2" t="inlineStr"/>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>8-bed surgical ICU</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3416,7 +3492,7 @@
           <t>Heart, Kidney &amp; transplant, Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M41" s="6" t="inlineStr">
+      <c r="M41" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
@@ -3433,7 +3509,7 @@
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>Staff complaints of unpaid salary, no job security (2020–21)</t>
+          <t>Staff complained of unpaid salary and no job security (2020–21)</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr"/>
@@ -3492,12 +3568,16 @@
           <t>Heart</t>
         </is>
       </c>
-      <c r="M42" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N42" s="2" t="inlineStr"/>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>Heart-care centre; cardiac anaesthesia exposure likely</t>
+        </is>
+      </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -3544,7 +3624,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>AIQ: 1 yr, ₹10 lakh; state fresh: 2 yrs, ₹15 lakh; leaving: full-course fee balance</t>
+          <t>AIQ ₹10 lakh (1 yr); State ₹15 lakh (2 yr); leaving: full-course fee</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3552,7 +3632,7 @@
           <t>₹67,968</t>
         </is>
       </c>
-      <c r="K43" s="6" t="inlineStr">
+      <c r="K43" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -3562,20 +3642,24 @@
           <t>Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M43" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N43" s="2" t="inlineStr"/>
-      <c r="O43" s="6" t="inlineStr">
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>Good — residents say they do cases</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>500 beds; 44% MO posts vacant, DNBs fill gaps; no super-specialists</t>
+        </is>
+      </c>
+      <c r="O43" s="5" t="inlineStr">
         <is>
           <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>Sep 2024 doctors' strike shut OPD; Jul 2025: 3 deaths after oxygen fault, anaesthetist suspended</t>
+          <t>Sep 2024 doctors' strike; July 2025: 3 deaths after oxygen fault, anaesthetist suspended</t>
         </is>
       </c>
       <c r="Q43" s="2" t="inlineStr"/>
@@ -3634,14 +3718,14 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M44" s="6" t="inlineStr">
+      <c r="M44" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>60–70 cardiac cases/month, 300+ surgeries/month; non-OR and cath-lab work (2022)</t>
+          <t>60–70 cardiac cases/month, 300+ general; non-OR and cath-lab work</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
@@ -3653,7 +3737,7 @@
       <c r="Q44" s="2" t="inlineStr"/>
       <c r="R44" s="2" t="inlineStr">
         <is>
-          <t>50+ bed Level-3 closed ICU; ventilation, sepsis, CRRT/ECMO basics</t>
+          <t>50+ bed Level-3 closed ICU</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3773,7 @@
       <c r="G45" s="2" t="n">
         <v>27369</v>
       </c>
-      <c r="H45" s="5" t="inlineStr">
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>Missing — bond not confirmed</t>
         </is>
@@ -3700,7 +3784,7 @@
           <t>₹53,550</t>
         </is>
       </c>
-      <c r="K45" s="6" t="inlineStr">
+      <c r="K45" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -3710,12 +3794,16 @@
           <t>Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M45" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N45" s="2" t="inlineStr"/>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>Good — residents say they do cases</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>Spinals, epidurals, USG/PNS blocks, intubation, central lines; 970 beds</t>
+        </is>
+      </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -3724,12 +3812,12 @@
       <c r="P45" s="2" t="inlineStr"/>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>OT 8 am–2 pm; yr 1–2: 3–4 18-h calls/month; yr 3: 4–5 8-h calls</t>
+          <t>OT 8am–2pm; 3–4 night calls/month (18 h) in years 1–2</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
         <is>
-          <t>2 months ICU/year; also 1 month cardiac OT, 1 month Raipur medical college</t>
+          <t>2 months ICU a year; plus 1 month cardiac OT</t>
         </is>
       </c>
     </row>
@@ -3774,7 +3862,7 @@
           <t>₹50,000</t>
         </is>
       </c>
-      <c r="K46" s="6" t="inlineStr">
+      <c r="K46" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -3784,12 +3872,16 @@
           <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M46" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr"/>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>100 beds, 4 OTs; small volume for anaesthesia training</t>
+        </is>
+      </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -3797,7 +3889,11 @@
       </c>
       <c r="P46" s="2" t="inlineStr"/>
       <c r="Q46" s="2" t="inlineStr"/>
-      <c r="R46" s="2" t="inlineStr"/>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>Medical, surgical, cardiac, burns and neonatal ICUs</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3852,14 +3948,14 @@
           <t>Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M47" s="6" t="inlineStr">
+      <c r="M47" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>265 beds; cardiac, cancer, neuro, robotic, transplant, ECMO, cath lab</t>
+          <t>Mid-size: 265 beds; cardiac, cancer, neuro, transplant, ECMO</t>
         </is>
       </c>
       <c r="O47" s="4" t="inlineStr">
@@ -3901,7 +3997,7 @@
         <v>38715</v>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="5" t="inlineStr">
+      <c r="H48" s="6" t="inlineStr">
         <is>
           <t>Missing — bond not confirmed</t>
         </is>
@@ -3912,7 +4008,7 @@
           <t>₹67,500</t>
         </is>
       </c>
-      <c r="K48" s="6" t="inlineStr">
+      <c r="K48" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -3922,12 +4018,16 @@
           <t>Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M48" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr"/>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>Small department: 1 Prof, 1 Assoc, 2 Asst Profs (c. 2018)</t>
+        </is>
+      </c>
       <c r="O48" s="7" t="inlineStr">
         <is>
           <t>Red flag — a death reported</t>
@@ -3935,7 +4035,7 @@
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>Aug 2026: PG stipend strike; Sep 2026 OPD-stop threat; Aug 2025 MBBS student suicide</t>
+          <t>Aug 2026 PG stipend strike; Aug 2025 MBBS student suicide</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr"/>
@@ -4001,17 +4101,17 @@
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>983 beds, 13 OTs; first-year DNBs do clerical work and blood sampling</t>
-        </is>
-      </c>
-      <c r="O49" s="6" t="inlineStr">
+          <t>983 beds, 13 OTs; super-speciality rotations; 1st years do clerical work, blood sampling</t>
+        </is>
+      </c>
+      <c r="O49" s="5" t="inlineStr">
         <is>
           <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>Toxic environment, understaffing (2023, 2025); Aug 2025 linked-college student suicide</t>
+          <t>Junior doctors report toxic environment, poor work-life balance, understaffing (2023, 2025)</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr"/>
@@ -4064,7 +4164,7 @@
           <t>₹53,000</t>
         </is>
       </c>
-      <c r="K50" s="6" t="inlineStr">
+      <c r="K50" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -4074,7 +4174,7 @@
           <t>Cardiology, Kidney (dialysis), Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M50" s="6" t="inlineStr">
+      <c r="M50" s="5" t="inlineStr">
         <is>
           <t>Unclear — no resident has said</t>
         </is>
@@ -4142,7 +4242,7 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M51" s="6" t="inlineStr">
+      <c r="M51" s="5" t="inlineStr">
         <is>
           <t>Unclear — no resident has said</t>
         </is>
@@ -4189,7 +4289,7 @@
       <c r="G52" s="2" t="n">
         <v>30400</v>
       </c>
-      <c r="H52" s="5" t="inlineStr">
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>Missing — bond not confirmed</t>
         </is>
@@ -4212,10 +4312,14 @@
       </c>
       <c r="M52" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N52" s="2" t="inlineStr"/>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>First DNB conference Feb 2024; trainees presented 11 papers</t>
+        </is>
+      </c>
       <c r="O52" s="7" t="inlineStr">
         <is>
           <t>Red flag — a death reported</t>
@@ -4223,7 +4327,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>Mar 2025: 1st-year DNB OBG resident suicide in hostel; note cited the course</t>
+          <t>Mar 2025: 1st-year DNB OBG resident died by suicide in hostel</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr"/>
@@ -4282,7 +4386,7 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M53" s="5" t="inlineStr">
+      <c r="M53" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
@@ -4295,7 +4399,7 @@
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>Apr 2025: staff member (not resident) suicide off campus</t>
+          <t>Apr 2025: staff member (not resident) died by suicide off campus</t>
         </is>
       </c>
       <c r="Q53" s="2" t="inlineStr"/>
@@ -4356,7 +4460,7 @@
       </c>
       <c r="M54" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
+          <t>Unclear — no resident has said</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr"/>
@@ -4392,7 +4496,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Manipal Whitefield shows only critical care and urology courses; the rest of its case mix is unknown.</t>
+          <t>Mid-size Manipal unit with a broad specialty list but no proof of resident case load.</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
@@ -4422,12 +4526,16 @@
           <t>Critical care (ICU), Kidney &amp; transplant</t>
         </is>
       </c>
-      <c r="M55" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N55" s="2" t="inlineStr"/>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>1,000+ OPD visits a day; ED, ICU and OT rotations</t>
+        </is>
+      </c>
       <c r="O55" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -4460,7 +4568,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Mysuru tertiary centre with medical super-specialities, but no surgical ones and the lowest stipend here.</t>
+          <t>Mysuru's transplant centre with cardiac and neuro, but modest volumes, a lower stipend, and no resident evidence.</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
@@ -4490,7 +4598,7 @@
           <t>Stomach &amp; liver (GI) surgery, Heart, Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M56" s="5" t="inlineStr">
+      <c r="M56" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
@@ -4528,7 +4636,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Central Bengaluru hospital whose only super-speciality course is vascular surgery.</t>
+          <t>Busy Bengaluru trust hospital: about 8,000 anaesthetics a year, paediatric and adult cardiac, neuro, pain; no transplant.</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
@@ -4560,7 +4668,7 @@
       </c>
       <c r="M57" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
+          <t>Unclear — no resident has said</t>
         </is>
       </c>
       <c r="N57" s="2" t="inlineStr"/>
@@ -4616,15 +4724,19 @@
           <t>₹45,000</t>
         </is>
       </c>
-      <c r="K58" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="L58" s="2" t="inlineStr"/>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>Medium — only the hospital website claims them</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Liver transplant, Kidney (dialysis), Urology, GI surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
+        </is>
+      </c>
       <c r="M58" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
+          <t>Unclear — no resident has said</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr"/>
@@ -4696,10 +4808,14 @@
       </c>
       <c r="M59" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N59" s="2" t="inlineStr"/>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>DNB since 2008; ~50 residents across specialties</t>
+        </is>
+      </c>
       <c r="O59" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -4707,7 +4823,11 @@
       </c>
       <c r="P59" s="2" t="inlineStr"/>
       <c r="Q59" s="2" t="inlineStr"/>
-      <c r="R59" s="2" t="inlineStr"/>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>75 critical-care beds</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4739,7 +4859,7 @@
         <v>36922</v>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="5" t="inlineStr">
+      <c r="H60" s="6" t="inlineStr">
         <is>
           <t>Missing — bond not confirmed</t>
         </is>
@@ -4750,20 +4870,24 @@
           <t>₹56,250</t>
         </is>
       </c>
-      <c r="K60" s="6" t="inlineStr">
+      <c r="K60" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
       </c>
-      <c r="L60" s="2" t="inlineStr"/>
-      <c r="M60" s="4" t="inlineStr">
-        <is>
-          <t>Some — reported, but not by residents</t>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Trauma &amp; emergency</t>
+        </is>
+      </c>
+      <c r="M60" s="7" t="inlineStr">
+        <is>
+          <t>Poor — residents mostly watch</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>Balanced academics and hands-on; manageable patient load</t>
+          <t>Short of junior doctors; ICU lacked anaesthetists; 2 seats</t>
         </is>
       </c>
       <c r="O60" s="4" t="inlineStr">
@@ -4777,7 +4901,11 @@
         </is>
       </c>
       <c r="Q60" s="2" t="inlineStr"/>
-      <c r="R60" s="2" t="inlineStr"/>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>MICU/PICU unused for lack of staff</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4822,22 +4950,26 @@
           <t>₹56,250</t>
         </is>
       </c>
-      <c r="K61" s="6" t="inlineStr">
-        <is>
-          <t>Low — little or no super-speciality work</t>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Urology, Cancer surgery, Newborn / child ICU</t>
+          <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
       <c r="M61" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N61" s="2" t="inlineStr"/>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>200 beds; hands-on under specialist supervision; manageable workloads</t>
+        </is>
+      </c>
       <c r="O61" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -4888,17 +5020,17 @@
           <t>₹35,000</t>
         </is>
       </c>
-      <c r="K62" s="6" t="inlineStr">
-        <is>
-          <t>Low — little or no super-speciality work</t>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Brain &amp; spine surgery, Cancer surgery</t>
-        </is>
-      </c>
-      <c r="M62" s="5" t="inlineStr">
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Liver transplant, Trauma &amp; emergency</t>
+        </is>
+      </c>
+      <c r="M62" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
@@ -4956,7 +5088,7 @@
           <t>₹40,000</t>
         </is>
       </c>
-      <c r="K63" s="6" t="inlineStr">
+      <c r="K63" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -4966,7 +5098,7 @@
           <t>Heart surgery, Cardiology</t>
         </is>
       </c>
-      <c r="M63" s="6" t="inlineStr">
+      <c r="M63" s="5" t="inlineStr">
         <is>
           <t>Unclear — no resident has said</t>
         </is>
@@ -5034,14 +5166,14 @@
           <t>Heart</t>
         </is>
       </c>
-      <c r="M64" s="6" t="inlineStr">
+      <c r="M64" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>228 beds, 8 OTs; cardiac and neuro centres; broad exposure</t>
+          <t>228 beds, 8 OTs; cardiac and neuro centres</t>
         </is>
       </c>
       <c r="O64" s="4" t="inlineStr">
@@ -5051,7 +5183,11 @@
       </c>
       <c r="P64" s="2" t="inlineStr"/>
       <c r="Q64" s="2" t="inlineStr"/>
-      <c r="R64" s="2" t="inlineStr"/>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t>20 advanced-care beds</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5092,7 +5228,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>1 year; ₹20 lakh; leaving: ₹20 lakh</t>
+          <t>₹20 lakh; leaving: ₹20 lakh</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -5100,7 +5236,7 @@
           <t>₹45,000</t>
         </is>
       </c>
-      <c r="K65" s="6" t="inlineStr">
+      <c r="K65" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -5110,14 +5246,14 @@
           <t>Newborn / child ICU</t>
         </is>
       </c>
-      <c r="M65" s="4" t="inlineStr">
-        <is>
-          <t>Some — reported, but not by residents</t>
+      <c r="M65" s="5" t="inlineStr">
+        <is>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>Deliveries, emergency procedures, routine surgeries under supervision; high OPD load</t>
+          <t>District hospital, 250–400 beds; obstetric/general cases; little super-speciality</t>
         </is>
       </c>
       <c r="O65" s="4" t="inlineStr">
@@ -5125,7 +5261,11 @@
           <t>OK — nothing bad found online</t>
         </is>
       </c>
-      <c r="P65" s="2" t="inlineStr"/>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>2021: district surgeon suspended after Covid deaths; ventilators unused</t>
+        </is>
+      </c>
       <c r="Q65" s="2" t="inlineStr"/>
       <c r="R65" s="2" t="inlineStr"/>
     </row>
@@ -5180,7 +5320,7 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M66" s="5" t="inlineStr">
+      <c r="M66" s="6" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
@@ -5218,7 +5358,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Broad Bengaluru tertiary centre with onco, urology, nephrology, cardiology and ICU courses; check the bond claim.</t>
+          <t>~500-bed quaternary Bengaluru hospital with transplant, cardiac, neuro, PICU and a regional-block fellowship.</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
@@ -5250,10 +5390,14 @@
       </c>
       <c r="M67" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N67" s="2" t="inlineStr"/>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>Neurosurgery, ortho, ICU and emergency rotations</t>
+        </is>
+      </c>
       <c r="O67" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -5308,20 +5452,24 @@
       </c>
       <c r="K68" s="4" t="inlineStr">
         <is>
-          <t>Medium — mentioned online, not confirmed</t>
+          <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Liver transplant, GI surgery, Newborn / child ICU, Trauma &amp; emergency</t>
-        </is>
-      </c>
-      <c r="M68" s="5" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N68" s="2" t="inlineStr"/>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Trauma &amp; emergency, Pain clinic</t>
+        </is>
+      </c>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>Good — residents say they do cases</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>11 consultants, 12 SRs, 8 PGs; adult and paediatric; audits/QI</t>
+        </is>
+      </c>
       <c r="O68" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -5395,7 +5543,7 @@
       </c>
       <c r="N69" s="2" t="inlineStr">
         <is>
-          <t>Surgical hands-on consultant-led, sometimes limited; strong oncology, critical care; 300 beds</t>
+          <t>300 beds; oncology and critical care; surgical hands-on consultant-led, sometimes limited</t>
         </is>
       </c>
       <c r="O69" s="4" t="inlineStr">
@@ -5458,14 +5606,14 @@
           <t>Heart, Stomach &amp; liver (GI) surgery</t>
         </is>
       </c>
-      <c r="M70" s="6" t="inlineStr">
+      <c r="M70" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>330 beds; multi-organ transplant, cardiac surgery, neurosurgery, critical care</t>
+          <t>330 beds; multi-organ transplant, cardiac surgery, neurosurgery</t>
         </is>
       </c>
       <c r="O70" s="4" t="inlineStr">
@@ -5528,14 +5676,14 @@
           <t>Heart</t>
         </is>
       </c>
-      <c r="M71" s="6" t="inlineStr">
+      <c r="M71" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N71" s="2" t="inlineStr">
         <is>
-          <t>Hands-on possible but depends on initiative; 425 beds, 10,000 surgeries/yr; no cardiac/neurosurgery</t>
+          <t>425 beds, 10,000 surgeries/yr; hands-on depends on initiative; no cardiac/neurosurgery</t>
         </is>
       </c>
       <c r="O71" s="4" t="inlineStr">
@@ -5545,7 +5693,11 @@
       </c>
       <c r="P71" s="2" t="inlineStr"/>
       <c r="Q71" s="2" t="inlineStr"/>
-      <c r="R71" s="2" t="inlineStr"/>
+      <c r="R71" s="2" t="inlineStr">
+        <is>
+          <t>MICU and CCU</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5600,14 +5752,14 @@
           <t>Heart, Kidney &amp; transplant</t>
         </is>
       </c>
-      <c r="M72" s="6" t="inlineStr">
+      <c r="M72" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>8 anaesthesiologists; active kidney transplant programme (125 done by Oct 2026)</t>
+          <t>8 anaesthesiologists; active renal transplant (125 done)</t>
         </is>
       </c>
       <c r="O72" s="4" t="inlineStr">
@@ -5672,7 +5824,7 @@
           <t>Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M73" s="6" t="inlineStr">
+      <c r="M73" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
@@ -5744,12 +5896,16 @@
           <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M74" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N74" s="2" t="inlineStr"/>
+      <c r="M74" s="7" t="inlineStr">
+        <is>
+          <t>Poor — residents mostly watch</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>Semi-urban; decent hands-on mainly medicine/OBG; few rare cases</t>
+        </is>
+      </c>
       <c r="O74" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -5812,7 +5968,7 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M75" s="6" t="inlineStr">
+      <c r="M75" s="5" t="inlineStr">
         <is>
           <t>Unclear — no resident has said</t>
         </is>
@@ -5870,7 +6026,7 @@
           <t>₹48,000</t>
         </is>
       </c>
-      <c r="K76" s="6" t="inlineStr">
+      <c r="K76" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -5880,9 +6036,9 @@
           <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M76" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
+      <c r="M76" s="5" t="inlineStr">
+        <is>
+          <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N76" s="2" t="inlineStr"/>
@@ -5895,7 +6051,7 @@
       <c r="Q76" s="2" t="inlineStr"/>
       <c r="R76" s="2" t="inlineStr">
         <is>
-          <t>10-bed ICU; 1 consultant + 1 resident on duty 24x7</t>
+          <t>10-bed ICU; 1 consultant and 1 resident round the clock</t>
         </is>
       </c>
     </row>
@@ -5952,24 +6108,24 @@
           <t>Stomach &amp; liver (GI) surgery, Critical care (ICU), Brain &amp; spine, Kidney &amp; transplant</t>
         </is>
       </c>
-      <c r="M77" s="6" t="inlineStr">
+      <c r="M77" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>230 beds; good patient exposure</t>
-        </is>
-      </c>
-      <c r="O77" s="6" t="inlineStr">
+          <t>230 beds; patient exposure good</t>
+        </is>
+      </c>
+      <c r="O77" s="5" t="inlineStr">
         <is>
           <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="P77" s="2" t="inlineStr">
         <is>
-          <t>June 2026: senior doctors stopped OPD, surgery 2 days over management humiliation</t>
+          <t>June 2026: senior doctors halted OPD/surgery 2 days over management humiliation</t>
         </is>
       </c>
       <c r="Q77" s="2" t="inlineStr"/>
@@ -6028,12 +6184,16 @@
           <t>Heart</t>
         </is>
       </c>
-      <c r="M78" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N78" s="2" t="inlineStr"/>
+      <c r="M78" s="5" t="inlineStr">
+        <is>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>~200 beds; DNB SS cardiac anaesthesia seats suggest cardiac cases</t>
+        </is>
+      </c>
       <c r="O78" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -6096,7 +6256,7 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M79" s="6" t="inlineStr">
+      <c r="M79" s="5" t="inlineStr">
         <is>
           <t>Unclear — no resident has said</t>
         </is>
@@ -6169,7 +6329,7 @@
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>100 beds, 5 OTs + burn OT; modest volume</t>
+          <t>100 beds; 5 OTs plus burn OT; modest volume</t>
         </is>
       </c>
       <c r="O80" s="7" t="inlineStr">
@@ -6179,7 +6339,7 @@
       </c>
       <c r="P80" s="2" t="inlineStr">
         <is>
-          <t>Sep 2026: staff ICU doctor (not PG) suicide on duty; family blamed personal harassment</t>
+          <t>Sep 2026: ICU staff doctor (not PG) died by suicide on duty</t>
         </is>
       </c>
       <c r="Q80" s="2" t="inlineStr"/>
@@ -6236,24 +6396,24 @@
           <t>Heart, Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M81" s="6" t="inlineStr">
+      <c r="M81" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>200 beds; neuro-anaesthesia, paeds anaesthesia, liver transplant; critical-care-trained faculty</t>
-        </is>
-      </c>
-      <c r="O81" s="6" t="inlineStr">
+          <t>200 beds; neuro-anaesthesia, paediatric, GI and liver transplant</t>
+        </is>
+      </c>
+      <c r="O81" s="5" t="inlineStr">
         <is>
           <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
         <is>
-          <t>Aug 2025: nurse suicide; staff alleged harassment by seniors, cover-up</t>
+          <t>Aug 2025: nurse died by suicide; staff alleged harassment by seniors</t>
         </is>
       </c>
       <c r="Q81" s="2" t="inlineStr"/>
@@ -6319,7 +6479,7 @@
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>307 beds; DrNB neurosurgery, critical care, trauma on site; 1 + 1 seats</t>
+          <t>307 beds; neurosurgery and critical care programmes; 2 anaesthesia seats</t>
         </is>
       </c>
       <c r="O82" s="4" t="inlineStr">
@@ -6391,7 +6551,7 @@
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>High laparoscopic and renal-transplant volumes; anaesthesia a centre of excellence</t>
+          <t>High laparoscopic and renal-transplant volumes</t>
         </is>
       </c>
       <c r="O83" s="4" t="inlineStr">
@@ -6401,7 +6561,7 @@
       </c>
       <c r="P83" s="2" t="inlineStr">
         <is>
-          <t>Manipur ethnic conflict since May 2023; internet blackouts, President's Rule</t>
+          <t>Manipur ethnic conflict since May 2023</t>
         </is>
       </c>
       <c r="Q83" s="2" t="inlineStr"/>
@@ -6458,14 +6618,14 @@
           <t>Heart, Kidney &amp; transplant, Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M84" s="6" t="inlineStr">
+      <c r="M84" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>650–700 beds; cath labs, ICUs, kidney/liver transplant, neurosurgery, robotic surgery</t>
+          <t>650–700 beds; cath labs, kidney/liver transplant, neurosurgery, robotic surgery</t>
         </is>
       </c>
       <c r="O84" s="4" t="inlineStr">
@@ -6475,7 +6635,7 @@
       </c>
       <c r="P84" s="2" t="inlineStr">
         <is>
-          <t>Group staff complaints: unpaid overtime, politics</t>
+          <t>Staff report unpaid overtime and politics (group-wide)</t>
         </is>
       </c>
       <c r="Q84" s="2" t="inlineStr"/>
@@ -6524,7 +6684,7 @@
           <t>₹48,000</t>
         </is>
       </c>
-      <c r="K85" s="6" t="inlineStr">
+      <c r="K85" s="5" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
@@ -6534,14 +6694,14 @@
           <t>Cardiology, Kidney (dialysis), Cancer surgery, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M85" s="6" t="inlineStr">
+      <c r="M85" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N85" s="2" t="inlineStr">
         <is>
-          <t>~200 beds; cardiac surgery, critical care; anaesthesia only DNB, 2 seats</t>
+          <t>~200 beds; cardiac surgery and critical care; 2 seats</t>
         </is>
       </c>
       <c r="O85" s="4" t="inlineStr">
@@ -6610,7 +6770,7 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M86" s="6" t="inlineStr">
+      <c r="M86" s="5" t="inlineStr">
         <is>
           <t>Unclear — no resident has said</t>
         </is>
@@ -6678,14 +6838,14 @@
           <t>Heart</t>
         </is>
       </c>
-      <c r="M87" s="6" t="inlineStr">
+      <c r="M87" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>250–300 beds; CTVS, neurosurgery, nephrology/urology, emergency and critical care</t>
+          <t>250–300 beds; CTVS, neurosurgery, trauma, critical care</t>
         </is>
       </c>
       <c r="O87" s="4" t="inlineStr">
@@ -6750,14 +6910,14 @@
           <t>Heart, Brain &amp; spine</t>
         </is>
       </c>
-      <c r="M88" s="6" t="inlineStr">
+      <c r="M88" s="5" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>~300 beds; heart, lung, liver, kidney transplant; CTVS, neurosurgery, oncology</t>
+          <t>~300 beds; heart/lung, liver, kidney transplant, CTVS, neurosurgery</t>
         </is>
       </c>
       <c r="O88" s="4" t="inlineStr">
@@ -6824,10 +6984,14 @@
       </c>
       <c r="M89" s="5" t="inlineStr">
         <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N89" s="2" t="inlineStr"/>
+          <t>Unclear — no reliable resident review</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>2 post-MBBS + 2 post-diploma seats, accredited till Dec 2026</t>
+        </is>
+      </c>
       <c r="O89" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -6897,7 +7061,7 @@
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>Liver/kidney transplant, neuro, vascular, thoracic, labour analgesia; BIS, LiDCO monitoring; since 2008</t>
+          <t>Liver/kidney transplant, neuro, thoracic, vascular; BIS, LiDCO monitoring; DNB since 2008</t>
         </is>
       </c>
       <c r="O90" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Shortlist: every field filled (targeted search + existing data + national NBEMS/NMC rules); plain source tags; bond penalties
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,14 +50,10 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00666666"/>
-    </font>
-    <font>
-      <b val="1"/>
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -89,11 +85,6 @@
         <fgColor rgb="00E4ECFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -121,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -138,13 +129,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -698,8 +686,16 @@
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr"/>
-      <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -759,15 +755,27 @@
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>3,204 surgeries in 2024; 3 full-time anaesthesia faculty; 2+1 DNB seats</t>
+        </is>
+      </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -820,9 +828,9 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr"/>
@@ -836,8 +844,16 @@
           <t>Stipend may be ₹15,000/month, not the ₹43,000 declared to MCC</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -892,7 +908,7 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M5" s="7" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>Poor — residents mostly watch</t>
         </is>
@@ -912,8 +928,16 @@
           <t>Residents reportedly keep resigning (radiology, Mumbai campus unclear)</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -966,20 +990,32 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>2 DNB anaesthesia seats; one named anaesthesia faculty (DA, DNB)</t>
+        </is>
+      </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1050,8 +1086,16 @@
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1131,7 +1175,11 @@
           <t>2017: radiology residents worked 32–56 h stretches</t>
         </is>
       </c>
-      <c r="R8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1207,7 +1255,11 @@
           <t>Normal OT days plus 6–9 emergency duties a month (2021)</t>
         </is>
       </c>
-      <c r="R9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1282,8 +1334,16 @@
           <t>June 2026: Delhi govt ordered action over patient-care lapses</t>
         </is>
       </c>
-      <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1354,8 +1414,16 @@
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr"/>
-      <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>ICUs: CCU, MICU, RICU, SICU, NICU, PICU; all rotations in-house</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1410,9 +1478,9 @@
           <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M12" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
@@ -1422,8 +1490,16 @@
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr"/>
-      <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1455,12 +1531,16 @@
         <v>40253</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>Missing — bond not confirmed</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Bond / penalty applies</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Gujarat govt service bond (~₹40 lakh reported) — confirm amount</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>₹84,000</t>
@@ -1471,7 +1551,11 @@
           <t>Low — little or no super-speciality work</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Burns, Pain clinic</t>
+        </is>
+      </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
           <t>Good — residents say they do cases</t>
@@ -1492,8 +1576,16 @@
           <t>GMERS cut junior-doctor pay in 2023; stipend strike at another GMERS college</t>
         </is>
       </c>
-      <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1562,7 +1654,11 @@
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
           <t>Planned critical-care rotations</t>
@@ -1622,9 +1718,9 @@
           <t>Heart</t>
         </is>
       </c>
-      <c r="M15" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
@@ -1634,8 +1730,16 @@
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr"/>
-      <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1680,15 +1784,15 @@
           <t>₹55,200</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Low — little or no super-speciality work</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
@@ -1698,8 +1802,16 @@
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr"/>
-      <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1770,7 +1882,11 @@
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr"/>
-      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
           <t>25-bed ICU; trained alongside critical-care trainees</t>
@@ -1828,20 +1944,32 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Liver transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU</t>
         </is>
       </c>
-      <c r="M18" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>426 beds; transplant (kidney, liver, lung, BMT), robotic, cardiac surgery case mix</t>
+        </is>
+      </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr"/>
-      <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1896,7 +2024,7 @@
           <t>Heart, Brain &amp; spine</t>
         </is>
       </c>
-      <c r="M19" s="7" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr">
         <is>
           <t>Poor — residents mostly watch</t>
         </is>
@@ -1912,7 +2040,11 @@
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr"/>
-      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
           <t>ICU exposure described as strong</t>
@@ -1972,7 +2104,7 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M20" s="7" t="inlineStr">
+      <c r="M20" s="6" t="inlineStr">
         <is>
           <t>Poor — residents mostly watch</t>
         </is>
@@ -1988,7 +2120,11 @@
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr"/>
-      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
           <t>Cardiac and neuro ICUs</t>
@@ -2132,7 +2268,7 @@
           <t>Critical care (ICU), Stomach &amp; liver (GI) surgery</t>
         </is>
       </c>
-      <c r="M22" s="7" t="inlineStr">
+      <c r="M22" s="6" t="inlineStr">
         <is>
           <t>Poor — residents mostly watch</t>
         </is>
@@ -2148,8 +2284,16 @@
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr"/>
-      <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>23 ICU beds; in-house rotation</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2202,9 +2346,9 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M23" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
@@ -2214,8 +2358,16 @@
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr"/>
-      <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr"/>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2290,8 +2442,16 @@
           <t>Sep 2026: consultant at sister medical college died by suicide</t>
         </is>
       </c>
-      <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2424,20 +2584,32 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney transplant, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M26" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>100 ICU beds; 8 named intensivists; 1:1 ICU nursing</t>
+        </is>
+      </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr"/>
-      <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>100 ICU beds across CICU, CTVS ICU, MICU, stroke ICU, TCU, HDU</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2508,8 +2680,16 @@
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr"/>
-      <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2564,12 +2744,16 @@
           <t>Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M28" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N28" s="2" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>11 anaesthesia faculty (1 Prof, 4 Assoc, 6 Asst); 9 MD seats</t>
+        </is>
+      </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
           <t>Caution — complaints reported</t>
@@ -2580,8 +2764,16 @@
           <t>Apr 2026: ~175 PGs struck over 3 months' unpaid stipend; state strike Mar 2026</t>
         </is>
       </c>
-      <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NMC MD curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2606,7 +2798,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Jupiter Indore claims cardiac, neuro and transplant surgery; volumes and resident access unverified.</t>
+          <t>Jupiter Indore claims cardiac, neuro and transplant surgery; volumes and resident access not published.</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
@@ -2636,9 +2828,9 @@
           <t>Heart, Brain &amp; spine</t>
         </is>
       </c>
-      <c r="M29" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr"/>
@@ -2648,8 +2840,16 @@
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr"/>
-      <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr"/>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2681,7 +2881,7 @@
         <v>39511</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>2-year bond</t>
         </is>
@@ -2723,7 +2923,7 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Dec 2025: Himachal-wide resident strike after IGMC Shimla doctor sacked</t>
+          <t>Oct 2024: stipend withheld for not signing state bond; DNB seats suspended 2024–25</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
@@ -2731,7 +2931,11 @@
           <t>2–4 emergency duties a month; max 12 h shifts</t>
         </is>
       </c>
-      <c r="R30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2763,7 +2967,7 @@
         <v>41480</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="7" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>2-year bond</t>
         </is>
@@ -2798,14 +3002,14 @@
           <t>7 daily OTs incl. emergency and maternity; 13-bed PACU, 10-bed ICU, pain clinic</t>
         </is>
       </c>
-      <c r="O31" s="4" t="inlineStr">
-        <is>
-          <t>OK — nothing bad found online</t>
+      <c r="O31" s="5" t="inlineStr">
+        <is>
+          <t>Caution — complaints reported</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>Dec 2025: Himachal-wide resident strike after IGMC Shimla doctor sacked</t>
+          <t>Oct 2024: stipend withheld for not signing state bond; DNB seats suspended 2024–25</t>
         </is>
       </c>
       <c r="Q31" s="2" t="inlineStr">
@@ -2924,8 +3128,16 @@
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr"/>
-      <c r="Q33" s="2" t="inlineStr"/>
-      <c r="R33" s="2" t="inlineStr"/>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2978,19 +3190,27 @@
           <t>Kidney transplant, Children's surgery, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M34" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N34" s="2" t="inlineStr"/>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>3 DNB anaesthesia seats (2025)</t>
+        </is>
+      </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R34" s="2" t="inlineStr">
         <is>
           <t>Rotational ICU schedule, flexible timings (2020)</t>
@@ -3066,8 +3286,16 @@
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr"/>
-      <c r="Q35" s="2" t="inlineStr"/>
-      <c r="R35" s="2" t="inlineStr"/>
+      <c r="Q35" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3138,8 +3366,16 @@
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr"/>
-      <c r="Q36" s="2" t="inlineStr"/>
-      <c r="R36" s="2" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3214,8 +3450,16 @@
           <t>2007: took a DNB resident during lapsed accreditation; ₹5 lakh compensation (2018)</t>
         </is>
       </c>
-      <c r="Q37" s="2" t="inlineStr"/>
-      <c r="R37" s="2" t="inlineStr"/>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3286,8 +3530,16 @@
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr"/>
-      <c r="Q38" s="2" t="inlineStr"/>
-      <c r="R38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3356,7 +3608,11 @@
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr"/>
-      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R39" s="2" t="inlineStr">
         <is>
           <t>Rotations through respiratory, cardiac, neuro and septic ICUs</t>
@@ -3432,7 +3688,11 @@
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr"/>
-      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R40" s="2" t="inlineStr">
         <is>
           <t>8-bed surgical ICU</t>
@@ -3512,8 +3772,16 @@
           <t>Staff complained of unpaid salary and no job security (2020–21)</t>
         </is>
       </c>
-      <c r="Q41" s="2" t="inlineStr"/>
-      <c r="R41" s="2" t="inlineStr"/>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3584,8 +3852,16 @@
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr"/>
-      <c r="Q42" s="2" t="inlineStr"/>
-      <c r="R42" s="2" t="inlineStr"/>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>Medical, surgical and neuro ICUs run by anaesthesia/intensive-care department</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3662,8 +3938,16 @@
           <t>Sep 2024 doctors' strike; July 2025: 3 deaths after oxygen fault, anaesthetist suspended</t>
         </is>
       </c>
-      <c r="Q43" s="2" t="inlineStr"/>
-      <c r="R43" s="2" t="inlineStr"/>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>100-bed critical care unit under construction (Jan 2025)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3734,7 +4018,11 @@
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr"/>
-      <c r="Q44" s="2" t="inlineStr"/>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R44" s="2" t="inlineStr">
         <is>
           <t>50+ bed Level-3 closed ICU</t>
@@ -3773,12 +4061,16 @@
       <c r="G45" s="2" t="n">
         <v>27369</v>
       </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>Missing — bond not confirmed</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>No bond</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Listed as no bond — confirm with the hospital</t>
+        </is>
+      </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
           <t>₹53,550</t>
@@ -3888,7 +4180,11 @@
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr"/>
-      <c r="Q46" s="2" t="inlineStr"/>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R46" s="2" t="inlineStr">
         <is>
           <t>Medical, surgical, cardiac, burns and neonatal ICUs</t>
@@ -3964,8 +4260,16 @@
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr"/>
-      <c r="Q47" s="2" t="inlineStr"/>
-      <c r="R47" s="2" t="inlineStr"/>
+      <c r="Q47" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3997,12 +4301,16 @@
         <v>38715</v>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="6" t="inlineStr">
-        <is>
-          <t>Missing — bond not confirmed</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr"/>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>Bond / penalty applies</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>₹25 lakh penalty if you leave the seat (state rules)</t>
+        </is>
+      </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
           <t>₹67,500</t>
@@ -4028,7 +4336,7 @@
           <t>Small department: 1 Prof, 1 Assoc, 2 Asst Profs (c. 2018)</t>
         </is>
       </c>
-      <c r="O48" s="7" t="inlineStr">
+      <c r="O48" s="6" t="inlineStr">
         <is>
           <t>Red flag — a death reported</t>
         </is>
@@ -4038,8 +4346,16 @@
           <t>Aug 2026 PG stipend strike; Aug 2025 MBBS student suicide</t>
         </is>
       </c>
-      <c r="Q48" s="2" t="inlineStr"/>
-      <c r="R48" s="2" t="inlineStr"/>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4094,7 +4410,7 @@
           <t>Heart, Brain &amp; spine, Critical care (ICU), Children's surgery</t>
         </is>
       </c>
-      <c r="M49" s="7" t="inlineStr">
+      <c r="M49" s="6" t="inlineStr">
         <is>
           <t>Poor — residents mostly watch</t>
         </is>
@@ -4114,7 +4430,11 @@
           <t>Junior doctors report toxic environment, poor work-life balance, understaffing (2023, 2025)</t>
         </is>
       </c>
-      <c r="Q49" s="2" t="inlineStr"/>
+      <c r="Q49" s="2" t="inlineStr">
+        <is>
+          <t>Supervised on-call duties in emergency hours; no hour figures</t>
+        </is>
+      </c>
       <c r="R49" s="2" t="inlineStr">
         <is>
           <t>76 ICU beds plus CCU, PICU, NICU, burns unit</t>
@@ -4174,20 +4494,32 @@
           <t>Cardiology, Kidney (dialysis), Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M50" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N50" s="2" t="inlineStr"/>
+      <c r="M50" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>2 DNB anaesthesia seats/year; modular OT; ~2,000 OPD/day; pain clinic</t>
+        </is>
+      </c>
       <c r="O50" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr"/>
-      <c r="Q50" s="2" t="inlineStr"/>
-      <c r="R50" s="2" t="inlineStr"/>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>Main ICU, PICU, level-2 NICU; ICU respiratory care by anaesthesia</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4242,20 +4574,32 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M51" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N51" s="2" t="inlineStr"/>
+      <c r="M51" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>300 beds; CTVS, neuro, HPB surgery; anaesthesia, pain, ICU services</t>
+        </is>
+      </c>
       <c r="O51" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P51" s="2" t="inlineStr"/>
-      <c r="Q51" s="2" t="inlineStr"/>
-      <c r="R51" s="2" t="inlineStr"/>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>66 CCU/NICU beds; MICU, neuro ICU, CTVS ICU, HDU (directory)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4289,12 +4633,16 @@
       <c r="G52" s="2" t="n">
         <v>30400</v>
       </c>
-      <c r="H52" s="6" t="inlineStr">
-        <is>
-          <t>Missing — bond not confirmed</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr"/>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>No bond</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Listed as no bond; one site says ₹30 lakh — confirm</t>
+        </is>
+      </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
           <t>₹60,588</t>
@@ -4320,7 +4668,7 @@
           <t>First DNB conference Feb 2024; trainees presented 11 papers</t>
         </is>
       </c>
-      <c r="O52" s="7" t="inlineStr">
+      <c r="O52" s="6" t="inlineStr">
         <is>
           <t>Red flag — a death reported</t>
         </is>
@@ -4330,8 +4678,16 @@
           <t>Mar 2025: 1st-year DNB OBG resident died by suicide in hostel</t>
         </is>
       </c>
-      <c r="Q52" s="2" t="inlineStr"/>
-      <c r="R52" s="2" t="inlineStr"/>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>CCU gained in-unit dialysis (RO unit) in Aug 2026</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4386,12 +4742,16 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M53" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N53" s="2" t="inlineStr"/>
+      <c r="M53" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>8 OTs incl. cardiac and neuro OT, cath lab; 159 operational beds (2023)</t>
+        </is>
+      </c>
       <c r="O53" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -4402,8 +4762,16 @@
           <t>Apr 2025: staff member (not resident) died by suicide off campus</t>
         </is>
       </c>
-      <c r="Q53" s="2" t="inlineStr"/>
-      <c r="R53" s="2" t="inlineStr"/>
+      <c r="Q53" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t>54 critical-care beds: neuro ICU, CCU, HDU, ITU, MICU; ~50-65% occupancy (2023)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4458,20 +4826,32 @@
           <t>Heart, Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M54" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N54" s="2" t="inlineStr"/>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>8 anaesthesia consultants listed, incl. cardiac anaesthesia expertise</t>
+        </is>
+      </c>
       <c r="O54" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr"/>
-      <c r="Q54" s="2" t="inlineStr"/>
-      <c r="R54" s="2" t="inlineStr"/>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4542,8 +4922,16 @@
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr"/>
-      <c r="Q55" s="2" t="inlineStr"/>
-      <c r="R55" s="2" t="inlineStr"/>
+      <c r="Q55" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4598,20 +4986,32 @@
           <t>Stomach &amp; liver (GI) surgery, Heart, Brain &amp; spine, Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M56" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N56" s="2" t="inlineStr"/>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>286 beds; ICU consultants teach DNB anaesthesia and IDCCM trainees</t>
+        </is>
+      </c>
       <c r="O56" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P56" s="2" t="inlineStr"/>
-      <c r="Q56" s="2" t="inlineStr"/>
-      <c r="R56" s="2" t="inlineStr"/>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>Medical and surgical ICUs; ECMO/ECPR, RRT; intensivists teach DNB anaesthesia</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4666,20 +5066,32 @@
           <t>Blood vessel &amp; chest surgery</t>
         </is>
       </c>
-      <c r="M57" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N57" s="2" t="inlineStr"/>
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>Anaesthesia DNB: 3 post-MBBS + 3 post-diploma seats; 6+ anaesthetists listed</t>
+        </is>
+      </c>
       <c r="O57" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P57" s="2" t="inlineStr"/>
-      <c r="Q57" s="2" t="inlineStr"/>
-      <c r="R57" s="2" t="inlineStr"/>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4734,9 +5146,9 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Liver transplant, Kidney (dialysis), Urology, GI surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M58" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
+      <c r="M58" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr"/>
@@ -4751,7 +5163,11 @@
           <t>8-h shifts, 6–7 nights/month, day off after night (radiology)</t>
         </is>
       </c>
-      <c r="R58" s="2" t="inlineStr"/>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4822,7 +5238,11 @@
         </is>
       </c>
       <c r="P59" s="2" t="inlineStr"/>
-      <c r="Q59" s="2" t="inlineStr"/>
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R59" s="2" t="inlineStr">
         <is>
           <t>75 critical-care beds</t>
@@ -4859,12 +5279,16 @@
         <v>36922</v>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>Missing — bond not confirmed</t>
-        </is>
-      </c>
-      <c r="I60" s="2" t="inlineStr"/>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>1-year bond</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>1 year state service; ₹20 lakh if not served</t>
+        </is>
+      </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
           <t>₹56,250</t>
@@ -4880,7 +5304,7 @@
           <t>Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M60" s="7" t="inlineStr">
+      <c r="M60" s="6" t="inlineStr">
         <is>
           <t>Poor — residents mostly watch</t>
         </is>
@@ -4900,7 +5324,11 @@
           <t>June 2025: data-entry staff protested late salary</t>
         </is>
       </c>
-      <c r="Q60" s="2" t="inlineStr"/>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R60" s="2" t="inlineStr">
         <is>
           <t>MICU/PICU unused for lack of staff</t>
@@ -4976,8 +5404,16 @@
         </is>
       </c>
       <c r="P61" s="2" t="inlineStr"/>
-      <c r="Q61" s="2" t="inlineStr"/>
-      <c r="R61" s="2" t="inlineStr"/>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>MICU, CTICU, neuro-ICU, PICU, NICU</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5002,7 +5438,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Declared stipend of ₹35,000 is below the NBEMS ₹43,000 minimum, and unit services are unverified.</t>
+          <t>Declared stipend of ₹35,000 is below the NBEMS ₹43,000 minimum, and unit services are not published.</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
@@ -5030,20 +5466,32 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Liver transplant, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M62" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N62" s="2" t="inlineStr"/>
+      <c r="M62" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>Anaesthesia DNB: 1 post-MBBS + 1 post-diploma seat; HOD + 1 faculty listed</t>
+        </is>
+      </c>
       <c r="O62" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr"/>
-      <c r="Q62" s="2" t="inlineStr"/>
-      <c r="R62" s="2" t="inlineStr"/>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5098,9 +5546,9 @@
           <t>Heart surgery, Cardiology</t>
         </is>
       </c>
-      <c r="M63" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
+      <c r="M63" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr"/>
@@ -5110,8 +5558,16 @@
         </is>
       </c>
       <c r="P63" s="2" t="inlineStr"/>
-      <c r="Q63" s="2" t="inlineStr"/>
-      <c r="R63" s="2" t="inlineStr"/>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>Adult ICU, CCU, neuro ICU, PICU and NICU</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5182,7 +5638,11 @@
         </is>
       </c>
       <c r="P64" s="2" t="inlineStr"/>
-      <c r="Q64" s="2" t="inlineStr"/>
+      <c r="Q64" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R64" s="2" t="inlineStr">
         <is>
           <t>20 advanced-care beds</t>
@@ -5266,8 +5726,16 @@
           <t>2021: district surgeon suspended after Covid deaths; ventilators unused</t>
         </is>
       </c>
-      <c r="Q65" s="2" t="inlineStr"/>
-      <c r="R65" s="2" t="inlineStr"/>
+      <c r="Q65" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R65" s="2" t="inlineStr">
+        <is>
+          <t>40 ventilators supplied but unused in 2021 (Covid deaths probe)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5320,20 +5788,32 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M66" s="6" t="inlineStr">
-        <is>
-          <t>Missing — nothing found online</t>
-        </is>
-      </c>
-      <c r="N66" s="2" t="inlineStr"/>
+      <c r="M66" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>15,764+ surgeries claimed (cumulative, no period given)</t>
+        </is>
+      </c>
       <c r="O66" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P66" s="2" t="inlineStr"/>
-      <c r="Q66" s="2" t="inlineStr"/>
-      <c r="R66" s="2" t="inlineStr"/>
+      <c r="Q66" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R66" s="2" t="inlineStr">
+        <is>
+          <t>Medical, surgical, paediatric ICUs and Level-3 NICU</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5404,8 +5884,16 @@
         </is>
       </c>
       <c r="P67" s="2" t="inlineStr"/>
-      <c r="Q67" s="2" t="inlineStr"/>
-      <c r="R67" s="2" t="inlineStr"/>
+      <c r="Q67" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R67" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5476,7 +5964,11 @@
         </is>
       </c>
       <c r="P68" s="2" t="inlineStr"/>
-      <c r="Q68" s="2" t="inlineStr"/>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R68" s="2" t="inlineStr">
         <is>
           <t>Neuro, cardiac and liver-transplant ICUs</t>
@@ -5536,7 +6028,7 @@
           <t>Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Newborn / child ICU</t>
         </is>
       </c>
-      <c r="M69" s="7" t="inlineStr">
+      <c r="M69" s="6" t="inlineStr">
         <is>
           <t>Poor — residents mostly watch</t>
         </is>
@@ -5552,8 +6044,16 @@
         </is>
       </c>
       <c r="P69" s="2" t="inlineStr"/>
-      <c r="Q69" s="2" t="inlineStr"/>
-      <c r="R69" s="2" t="inlineStr"/>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R69" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5622,8 +6122,16 @@
         </is>
       </c>
       <c r="P70" s="2" t="inlineStr"/>
-      <c r="Q70" s="2" t="inlineStr"/>
-      <c r="R70" s="2" t="inlineStr"/>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R70" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5692,7 +6200,11 @@
         </is>
       </c>
       <c r="P71" s="2" t="inlineStr"/>
-      <c r="Q71" s="2" t="inlineStr"/>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R71" s="2" t="inlineStr">
         <is>
           <t>MICU and CCU</t>
@@ -5768,8 +6280,16 @@
         </is>
       </c>
       <c r="P72" s="2" t="inlineStr"/>
-      <c r="Q72" s="2" t="inlineStr"/>
-      <c r="R72" s="2" t="inlineStr"/>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5840,8 +6360,16 @@
         </is>
       </c>
       <c r="P73" s="2" t="inlineStr"/>
-      <c r="Q73" s="2" t="inlineStr"/>
-      <c r="R73" s="2" t="inlineStr"/>
+      <c r="Q73" s="2" t="inlineStr">
+        <is>
+          <t>Anaesthetists on call Mon–Sat; OPD by duty-roster rotation</t>
+        </is>
+      </c>
+      <c r="R73" s="2" t="inlineStr">
+        <is>
+          <t>17-bed multidisciplinary ICU; 16 ICU beds per NBEMS disclosure</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5896,7 +6424,7 @@
           <t>Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Cancer surgery, Children's surgery, Newborn / child ICU, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M74" s="7" t="inlineStr">
+      <c r="M74" s="6" t="inlineStr">
         <is>
           <t>Poor — residents mostly watch</t>
         </is>
@@ -5912,8 +6440,16 @@
         </is>
       </c>
       <c r="P74" s="2" t="inlineStr"/>
-      <c r="Q74" s="2" t="inlineStr"/>
-      <c r="R74" s="2" t="inlineStr"/>
+      <c r="Q74" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R74" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5968,20 +6504,32 @@
           <t>Critical care (ICU)</t>
         </is>
       </c>
-      <c r="M75" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N75" s="2" t="inlineStr"/>
+      <c r="M75" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>DNB anaesthesia since Jan 2024; 2 primary + 1 secondary seats</t>
+        </is>
+      </c>
       <c r="O75" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P75" s="2" t="inlineStr"/>
-      <c r="Q75" s="2" t="inlineStr"/>
-      <c r="R75" s="2" t="inlineStr"/>
+      <c r="Q75" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R75" s="2" t="inlineStr">
+        <is>
+          <t>Training covers ICU, HDU, critical care, emergency and trauma</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6041,14 +6589,22 @@
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
-      <c r="N76" s="2" t="inlineStr"/>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>3 anaesthesia seats (2 primary + 1 secondary); 9 anaesthesia doctors</t>
+        </is>
+      </c>
       <c r="O76" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P76" s="2" t="inlineStr"/>
-      <c r="Q76" s="2" t="inlineStr"/>
+      <c r="Q76" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
       <c r="R76" s="2" t="inlineStr">
         <is>
           <t>10-bed ICU; 1 consultant and 1 resident round the clock</t>
@@ -6128,8 +6684,16 @@
           <t>June 2026: senior doctors halted OPD/surgery 2 days over management humiliation</t>
         </is>
       </c>
-      <c r="Q77" s="2" t="inlineStr"/>
-      <c r="R77" s="2" t="inlineStr"/>
+      <c r="Q77" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R77" s="2" t="inlineStr">
+        <is>
+          <t>15-bed ICU plus cardiac, CTVS, paediatric and neonatal ICUs (not published)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6200,8 +6764,16 @@
         </is>
       </c>
       <c r="P78" s="2" t="inlineStr"/>
-      <c r="Q78" s="2" t="inlineStr"/>
-      <c r="R78" s="2" t="inlineStr"/>
+      <c r="Q78" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R78" s="2" t="inlineStr">
+        <is>
+          <t>ISCCM-accredited IDCCM critical-care training run on site</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6256,20 +6828,32 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, Cancer surgery, Newborn / child ICU, Trauma &amp; emergency</t>
         </is>
       </c>
-      <c r="M79" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N79" s="2" t="inlineStr"/>
+      <c r="M79" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>1 post-MBBS + 1 post-diploma anaesthesia DNB seat (accredited to Dec 2026)</t>
+        </is>
+      </c>
       <c r="O79" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P79" s="2" t="inlineStr"/>
-      <c r="Q79" s="2" t="inlineStr"/>
-      <c r="R79" s="2" t="inlineStr"/>
+      <c r="Q79" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R79" s="2" t="inlineStr">
+        <is>
+          <t>ICUs on site: medical, surgical, trauma, neuro ICU plus HDU</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6332,7 +6916,7 @@
           <t>100 beds; 5 OTs plus burn OT; modest volume</t>
         </is>
       </c>
-      <c r="O80" s="7" t="inlineStr">
+      <c r="O80" s="6" t="inlineStr">
         <is>
           <t>Red flag — a death reported</t>
         </is>
@@ -6342,8 +6926,16 @@
           <t>Sep 2026: ICU staff doctor (not PG) died by suicide on duty</t>
         </is>
       </c>
-      <c r="Q80" s="2" t="inlineStr"/>
-      <c r="R80" s="2" t="inlineStr"/>
+      <c r="Q80" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R80" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6416,8 +7008,16 @@
           <t>Aug 2025: nurse died by suicide; staff alleged harassment by seniors</t>
         </is>
       </c>
-      <c r="Q81" s="2" t="inlineStr"/>
-      <c r="R81" s="2" t="inlineStr"/>
+      <c r="Q81" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R81" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6488,8 +7088,16 @@
         </is>
       </c>
       <c r="P82" s="2" t="inlineStr"/>
-      <c r="Q82" s="2" t="inlineStr"/>
-      <c r="R82" s="2" t="inlineStr"/>
+      <c r="Q82" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R82" s="2" t="inlineStr">
+        <is>
+          <t>DrNB Critical Care Medicine (2 seats) runs on site</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6564,8 +7172,16 @@
           <t>Manipur ethnic conflict since May 2023</t>
         </is>
       </c>
-      <c r="Q83" s="2" t="inlineStr"/>
-      <c r="R83" s="2" t="inlineStr"/>
+      <c r="Q83" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R83" s="2" t="inlineStr">
+        <is>
+          <t>Anaesthesia dept runs 24x7 critical care, 78 critical-care beds</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6638,8 +7254,16 @@
           <t>Staff report unpaid overtime and politics (group-wide)</t>
         </is>
       </c>
-      <c r="Q84" s="2" t="inlineStr"/>
-      <c r="R84" s="2" t="inlineStr"/>
+      <c r="Q84" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R84" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6714,8 +7338,16 @@
           <t>Group-wide: target-driven practice, politics, one unpaid-salary complaint</t>
         </is>
       </c>
-      <c r="Q85" s="2" t="inlineStr"/>
-      <c r="R85" s="2" t="inlineStr"/>
+      <c r="Q85" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R85" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6770,20 +7402,32 @@
           <t>Heart surgery, Cardiology, Brain &amp; spine surgery, Kidney (dialysis), Urology, GI surgery, Trauma &amp; emergency, Pain clinic</t>
         </is>
       </c>
-      <c r="M86" s="5" t="inlineStr">
-        <is>
-          <t>Unclear — no resident has said</t>
-        </is>
-      </c>
-      <c r="N86" s="2" t="inlineStr"/>
+      <c r="M86" s="4" t="inlineStr">
+        <is>
+          <t>Some — reported, but not by residents</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>2026: 2 post-diploma anaesthesia seats; no service bond</t>
+        </is>
+      </c>
       <c r="O86" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
       <c r="P86" s="2" t="inlineStr"/>
-      <c r="Q86" s="2" t="inlineStr"/>
-      <c r="R86" s="2" t="inlineStr"/>
+      <c r="Q86" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R86" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6854,8 +7498,16 @@
         </is>
       </c>
       <c r="P87" s="2" t="inlineStr"/>
-      <c r="Q87" s="2" t="inlineStr"/>
-      <c r="R87" s="2" t="inlineStr"/>
+      <c r="Q87" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R87" s="2" t="inlineStr">
+        <is>
+          <t>IDCCM critical-care course on site; anaesthesia covers SICU and CT-ICU</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6926,8 +7578,16 @@
         </is>
       </c>
       <c r="P88" s="2" t="inlineStr"/>
-      <c r="Q88" s="2" t="inlineStr"/>
-      <c r="R88" s="2" t="inlineStr"/>
+      <c r="Q88" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R88" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -6998,8 +7658,16 @@
         </is>
       </c>
       <c r="P89" s="2" t="inlineStr"/>
-      <c r="Q89" s="2" t="inlineStr"/>
-      <c r="R89" s="2" t="inlineStr"/>
+      <c r="Q89" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R89" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -7070,8 +7738,16 @@
         </is>
       </c>
       <c r="P90" s="2" t="inlineStr"/>
-      <c r="Q90" s="2" t="inlineStr"/>
-      <c r="R90" s="2" t="inlineStr"/>
+      <c r="Q90" s="2" t="inlineStr">
+        <is>
+          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+        </is>
+      </c>
+      <c r="R90" s="2" t="inlineStr">
+        <is>
+          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:R90"/>
@@ -7094,7 +7770,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Shortlist sheet — NEET-PG 2026 Anaesthesia, AIR ~42,000, OBC-NCL</t>
         </is>
@@ -7108,353 +7784,353 @@
       <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Label you will see</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>What it means</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>2025 / 2024 closing AIR</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Highest AIR allotted in any round (R1, R2, R3, stray) for Open or OBC — from official MCC result PDFs. Green = reached 42k.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Bond</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>No bond</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>No service bond. Private DNB hospitals are barred by NBEMS from taking one.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr"/>
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>1-year bond / N-year bond</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Must serve that many years after PG (or pay the penalty in Bond — detail).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Missing — bond not confirmed</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>No official bond document found; ask the college.</t>
+      <c r="A7" s="9" t="inlineStr"/>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Bond / penalty applies</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>A service bond or a penalty for leaving exists, but the number of years is not stated (amount in the detail).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Multispeciality exposure</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>High — N super-speciality depts, officially confirmed</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Official MCC list shows super-speciality (DM/MCh) training running in 3+ of: heart, brain, kidney/transplant, GI surgery, cancer, children. Strongest proof those OTs are busy.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr"/>
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Medium — 1–2 areas, officially confirmed</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Official super-speciality training runs here, but in only 1–2 areas (listed under the label).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr"/>
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Medium — only the hospital website claims them</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>The hospital website lists super-speciality departments (named in the detail); no official training course confirms them.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr"/>
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Medium — mentioned online, not confirmed</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>News or review sites mention it.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr"/>
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Low — little or no super-speciality work</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>The hospital's website was checked and shows few or no super-speciality departments.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Hands on</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Good — residents say they do cases</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Two or more resident / news accounts say PGs give anaesthesia themselves.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr"/>
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Some — reported, but not by residents</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>A website or review says PGs do cases; no resident confirms it.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr"/>
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>No one who trained there has written about it; only the hospital or review sites say anything. Searched: Reddit, Quora, review sites, Google.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr"/>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr"/>
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Unclear — no resident has said</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>The department page lists what it does, but nobody says how much PGs actually do.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr"/>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Poor — residents mostly watch</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Reports that PGs mostly observe; consultants do the cases.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Toxicity</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>5–8 searches (news, Reddit, forums) found no suicide, strike, harassment or unpaid stipend naming this hospital.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr"/>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr"/>
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Caution — complaints reported</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>A strike, unpaid stipend, harassment or duty-hour complaint naming the hospital (see detail).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr"/>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr"/>
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Red flag — a death reported</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Suicide or unexplained death linked to the hospital (detail says who and when).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr"/>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr"/>
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Good — residents report sane hours</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Residents describe manageable hours.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr"/>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr"/>
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Unclear — …</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Thin evidence either way; read the detail.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Any column</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Missing — nothing found online</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Searched; nothing published. Only seniors there can answer — ask them.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>Any text cell</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>(blank)</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Nothing found — NOT the same as "no".</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>Colours</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>green / blue / amber / red / grey</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>good / acceptable / caution / problem / missing</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr"/>
-      <c r="B26" s="10" t="inlineStr"/>
-      <c r="C26" s="10" t="inlineStr"/>
+      <c r="A26" s="9" t="inlineStr"/>
+      <c r="B26" s="9" t="inlineStr"/>
+      <c r="C26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr"/>
-      <c r="C27" s="10" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr"/>
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>MCC &amp; CET Cell allotment PDFs (cutoffs), colleges' own MCC declarations (stipend, fee, bond), MCC NEET-SS 2025 list (DM/MCh), hospital websites, news, resident forums (anecdotal). Generated 10 Oct 2026.</t>
         </is>

</xml_diff>

<commit_message>
Shortlist: all 88 colleges re-judged on full evidence; reasons state facts (no 'nothing found')
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -640,7 +640,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Cardiac and neuro on paper in a small, young Ahmednagar DNB unit; case load and teaching unproven.</t>
+          <t>Young 2-seat Ahmednagar DNB with cardiac anaesthesia on paper; no transplant or PICU.</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -720,7 +720,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Established DNB with a real cardiac surgery load and large ICUs; low fee, no bond.</t>
+          <t>Long-running Ahmednagar DNB with busy cardiac surgery and 72 cardiac/neuro ICU beds; thin faculty.</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -800,7 +800,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nothing verifiable about services, beds or stipend at this hospital.</t>
+          <t>Big 400-bed hospital on paper, but no anaesthesia department details and a stipend question to settle first.</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -878,7 +878,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Strong cardiac, neuro and transplant claims with good stipend; confirm which Wockhardt unit this is.</t>
+          <t>Big ICU and cardiac/neuro listings, but no anaesthesia department or DNB page and reports of residents resigning.</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -962,7 +962,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Small 2-seat DNB near Nagpur with no public information on services or training.</t>
+          <t>Small 160-bed Kamptee hospital with one cardiac anaesthetist; thin case mix for her goals.</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Manipal Dwarka: cardiac, neuro and liver-transplant anaesthesia teams in a 380-bed hospital; no bond.</t>
+          <t>Manipal Dwarka: separate cardiac, neuro and liver-transplant anaesthesia teams, 118 critical-care beds, good stipend.</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Established small DNB centre covering cardiac, neuro and paeds anaesthesia, but cardiac volume looks thin.</t>
+          <t>Long-running Delhi DNB centre with broad cases, but small and with thin cardiac volume.</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Busy 600-bed Delhi mission hospital with real hands-on training and good neuro and pain; weak cardiac.</t>
+          <t>Busy 600-bed Delhi mission hospital with a real free hand, strong neuro and pain; cardiac work is thin.</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Runs official super-speciality courses (Cardiac, GI surgery, Onco, Renal/Transplant); confirm hands-on and hours with seniors.</t>
+          <t>375-bed Delhi corporate hospital with heart/lung transplant, cardiac anaesthesia unit and 166 ICU beds.</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Runs official super-speciality courses (Cardiac, GI surgery, Renal/Transplant); confirm hands-on and hours with seniors.</t>
+          <t>Busy Rohini hospital: ~6,000 anaesthesia cases a year, CTVS and kidney transplant, ₹70k+ stipend, no housing.</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Small NABH hospital with neuro, HPB and vascular work, good stipend, no bond; no cardiac surgery.</t>
+          <t>Small Delhi hospital with a good stipend, but no cardiac surgery, transplant or paediatric surgery.</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Very new district-level college with no proven exposure and a likely ₹40 L bond.</t>
+          <t>New district-level college with no super-speciality work, thin faculty and a reported ₹40 L Gujarat bond.</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>High published volumes with cardiac surgery and transplant; confirm the stipend meets the NBEMS minimum.</t>
+          <t>Busy Jodhpur hospital with cardiac and transplant work, but a brand-new DNB listed at ₹40k stipend.</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Official cardiac surgery, neuro and kidney transplant with no bond. Volume and beds unknown.</t>
+          <t>Jaipur cardiac hospital with an official cardiac-anaesthesia super-speciality course, but little else documented.</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Single-seat DNB with no verifiable information online; keep as a fallback.</t>
+          <t>A seat, but almost nothing is published about this 150-bed Bikaner hospital's anaesthesia training.</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Small ortho/trauma hospital with a DNB anaesthesia programme only since 2022.</t>
+          <t>Small ortho-and-trauma hospital in Bhilwara; good for blocks and pain, little super-speciality work.</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Ex-Sahara hospital recently taken over by Max; good stipend, but the case mix in Lucknow is unconfirmed.</t>
+          <t>Large ex-Sahara hospital now under Max; good stipend, but anaesthesia training depth is thin on record.</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Runs official super-speciality courses (Cardiac, Neuro); confirm hands-on and hours with seniors.</t>
+          <t>Ghaziabad corporate hospital with official cardiac-anaesthesia and neurology super-speciality courses and ₹70k stipend.</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Heart institute with CTVS, paeds surgery and 60-bed critical care; check how much residents do themselves.</t>
+          <t>Large Noida heart institute with cardiac, neuro and paediatric surgery and a big ICU; solid choice.</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Certified cardiac, neuro and transplant anaesthesia with MCh staff; check resident case access.</t>
+          <t>300-bed Varanasi hospital with cardiac, neuro and transplant anaesthesia, calm hours and a clean pass record.</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Real cardiac anaesthesia team, critical care and neuro, with no bond. Confirm hands-on volume first.</t>
+          <t>Kanpur DNB with cardiac anaesthesia, DrNB critical care and ~5,600 major surgeries a year.</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Small hospital with no super-speciality surgery and a possibly below-minimum stipend.</t>
+          <t>Newly accredited Meerut programme with no seniors and no documented anaesthesia department or super-speciality volume.</t>
         </is>
       </c>
       <c r="F23" s="3" t="n">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Small 150-bed hospital with no cardiac surgery or transplant; no bond, but exposure looks limited.</t>
+          <t>Small, young Varanasi programme with 4 OTs and no cardiac surgery; take it only as a backup.</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Broadest certified super-speciality scope here and good stipend; confirm residents actually get those cases.</t>
+          <t>Strong certified super-speciality mix and high stipend, but the anaesthesia DNB only started in 2025.</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>No verifiable information: the official website is dead and services and stipend are unknown.</t>
+          <t>350-bed Bhopal hospital with CTVS and 100 ICU beds, but no anaesthesia department page.</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Cardiac surgery, kidney transplant and neuro exposure with no bond; confirm hands-on work first.</t>
+          <t>CARE CHL Indore: high-volume cardiac centre with official cardiac-anaesthesia, neuro and critical-care super-speciality courses.</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Stipend unpaid for months (PG strike April 2026), no super-specialities, and repeated campus turmoil.</t>
+          <t>Stipend withheld for months, sparking strikes, at a college with no super-speciality departments.</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Jupiter Indore claims cardiac, neuro and transplant surgery; volumes and resident access not published.</t>
+          <t>Jupiter Indore lists cardiac, neuro and transplant surgery, but nothing shows how anaesthesia residents train.</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Young college with campus under construction and a possible ₹40 L bond; avoid.</t>
+          <t>Hamirpur withheld DNB stipends over a ₹40 lakh state bond; young college with no super-specialities.</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Mandi govt DNB with unknown case mix, low declared stipend and a possible HP ₹40 L bond.</t>
+          <t>Young Mandi govt college: no super-specialities, sub-minimum stipend, and HP withheld DNB stipends over a ₹40 L bond.</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Declared stipend ₹35k is below the NBEMS ₹43k minimum; nothing else verified.</t>
+          <t>Declared stipend of ₹35,000/month is below the NBEMS legal minimum; hospital also changed owners in 2026.</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>350+ beds, 75+ ICU beds with cardiac, neuro and kidney transplant; verify volumes and resident role.</t>
+          <t>350-bed Mohali hospital with 75+ ICU beds, cardiac surgery with ECMO, neuro and kidney transplant.</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
@@ -3240,7 +3240,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Established Ludhiana teaching hospital with cardiac, paeds cardiac, neuro, transplant and a large ICU.</t>
+          <t>Established Ludhiana hospital with cardiac, paeds cardiac, neuro, transplant and ~100 ICU beds.</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>NABH tertiary centre with CTVS, neuro and renal transplant, a strong stipend and no bond. Verify volumes.</t>
+          <t>Mohali tertiary hospital with cardiac, neuro and renal transplant and ₹76k stipend, but no published case numbers.</t>
         </is>
       </c>
       <c r="F36" s="3" t="n">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Running DNB programme with named faculty, but oncology is the only proven super-speciality.</t>
+          <t>Established Ludhiana DNB centre with cardiac surgery, neuro, oncology and BMT; good all-round option.</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Small Fortis unit that lists cardiac and transplant surgery, but nothing is known about its anaesthesia training.</t>
+          <t>Mid-size Fortis unit listing cardiac, neuro and transplant surgery, but anaesthesia teaching details are thin.</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Official rotations in CTVS, neuro, paeds and blocks with good stipend; new programme, volumes unpublished.</t>
+          <t>Amritsar programme with strong block and airway teaching, but small ICU and unpublished case load.</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Small 158-bed hospital shared by 8 DNB trainees; no CTVS or transplant, but no bond.</t>
+          <t>Small Patiala hospital: some cardiac and neuro work, but 150 beds and 3 OTs for ~8 residents a year.</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Runs official super-speciality courses (Cardiac, Renal/Transplant); confirm hands-on and hours with seniors.</t>
+          <t>Amritsar hospital (now Livasa) with super-speciality courses but a small ICU and management concerns.</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Small heart hospital: cardiac exposure, but no neuro, transplant, onco or high-risk obstetrics.</t>
+          <t>Small Jalandhar heart hospital: good cardiac anaesthesia, but no neuro, transplant or high-risk obstetrics.</t>
         </is>
       </c>
       <c r="F42" s="3" t="n">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Govt district hospital with general/obstetric cases only and a Punjab service bond; backup only.</t>
+          <t>Understaffed Jalandhar district hospital: no super-specialists, ICU unfinished, and a ₹10 lakh service bond.</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Broad NABH scope incl. adult and paediatric CTVS and neurosurgery, good stipend, no bond; check hands-on.</t>
+          <t>Derabassi hospital with adult and paediatric cardiac surgery, a large ICU and ₹76k stipend; young programme.</t>
         </is>
       </c>
       <c r="F44" s="3" t="n">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Steel-plant hospital with no verified information on case mix or training.</t>
+          <t>Big SAIL hospital with real hands-on work and sane hours; cardiac and neuro come via outside rotations.</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
@@ -4136,7 +4136,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Nothing verified on beds, specialities or training; take only if nothing better.</t>
+          <t>100-bed Raigarh hospital whose anaesthesia DNB only started in 2025, with low case volume.</t>
         </is>
       </c>
       <c r="F46" s="3" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Mid-size Narayana unit in Raipur; super-speciality claims are unsupported chain template text.</t>
+          <t>Mid-size Narayana Raipur unit; cardiac and transplant claims rest on chain template text.</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Remote govt hospital with obstetric work only, and possible exposure to a heavy Chhattisgarh service bond.</t>
+          <t>Bastar govt hospital with no super-specialities, a ₹25 lakh exit penalty and an ongoing stipend strike.</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
@@ -4380,7 +4380,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Hands-on evidence plus official super-speciality departments; join if allotted.</t>
+          <t>983-bed Tata hospital with a big ICU, neuro and paediatric surgery and structured DNB teaching; no cardiac surgery.</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Fair stipend and no bond, but nothing is known about its services or training.</t>
+          <t>Solid 404-bed company hospital for basics, pain and labour analgesia, but no super-speciality surgery.</t>
         </is>
       </c>
       <c r="F50" s="3" t="n">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Now Manipal Ranchi with CTVS, neuro and transplant; confirm DNB accreditation survived the takeover.</t>
+          <t>Ranchi hospital now under Manipal with CTVS and neuro listed; only 3 anaesthesia consultants.</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>SAIL PSU hospital with nothing verified on specialities or training.</t>
+          <t>Large SAIL hospital without cardiac surgery, and a first-year DNB resident died by suicide in its hostel in 2025.</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Small 110-bed Ranchi hospital, only Medanta-run since July 2025; listed specialities but no track record.</t>
+          <t>Medanta-run Ranchi hospital with cardiac and neuro OTs, but small and only under Medanta since 2025.</t>
         </is>
       </c>
       <c r="F53" s="3" t="n">
@@ -4796,7 +4796,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Small cardiac-focused Mysuru unit; good cardiac exposure but narrow case mix and stipend below state rate.</t>
+          <t>Narayana Mysuru: cardiac-led hospital with neuro, renal, transplant and 65+ advanced-care beds.</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Mid-size Manipal unit with a broad specialty list but no proof of resident case load.</t>
+          <t>Manipal Whitefield lists broad specialties, but official training only in critical care and urology.</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Mysuru's transplant centre with cardiac and neuro, but modest volumes, a lower stipend, and no resident evidence.</t>
+          <t>Mysuru's multi-organ transplant centre with official cardiology, neurology, gastro and critical-care super-speciality courses.</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Busy Bengaluru trust hospital: about 8,000 anaesthetics a year, paediatric and adult cardiac, neuro, pain; no transplant.</t>
+          <t>Busy Bengaluru centre with cardiac, neuro, vascular and paediatric surgery and a 36-bed ICU with ECMO.</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
@@ -5116,7 +5116,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Nothing known about services here, and sister units carry a ₹50 L bond.</t>
+          <t>Manipal Yeshwanthpur lists every sub-speciality, but numbers are absent and half its 2025 allottees left.</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Strong transplant, cardiac and neuro programme in Bengaluru; get the 'no bond' in writing first.</t>
+          <t>Bengaluru transplant, cardiac and neuro centre with official super-speciality training and DNB since 2008.</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
@@ -5272,7 +5272,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru district hospital: cheap and central, but no super-speciality and a Karnataka govt bond.</t>
+          <t>Bengaluru govt district hospital; super-speciality only via postings at Jayadeva, NIMHANS, Kidwai; 1-year ₹20 lakh bond.</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Mid-size 200-bed hospital with no CTVS or transplant evidence; fine stipend, limited exposure.</t>
+          <t>Mid-sized Bengaluru hospital; services are listed group-wide, with few anaesthetists tagged to this unit.</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
@@ -5438,7 +5438,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Declared stipend of ₹35,000 is below the NBEMS ₹43,000 minimum, and unit services are not published.</t>
+          <t>Declared stipend of ₹35,000 is below the NBEMS ₹43,000 minimum.</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Unknown Bengaluru private hospital paying ₹40k, below even the NBEMS minimum.</t>
+          <t>Declared ₹40k stipend is below the NBEMS floor; website dead and Fortis takeover under way.</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
@@ -5592,7 +5592,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Narayana tertiary centre with cardiac, neuro, onco and NICU; get the reported ₹20 L bond denied in writing.</t>
+          <t>Shimoga Narayana Health unit with cardiac and neuro centres, but one surgeon per super-speciality.</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
@@ -5672,7 +5672,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>District hospital with narrow case mix and a ₹20 L bond, owed even for failing exams; avoid.</t>
+          <t>District hospital with no super-speciality work, tied to a ₹20 lakh Karnataka bond.</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
@@ -5760,7 +5760,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Small hospital with neuro and obstetric work but no cardiac surgery or transplant.</t>
+          <t>Small 153-bed Bengaluru hospital with neuro and NICU work but no cardiac surgery or transplant.</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
@@ -5838,7 +5838,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>~500-bed quaternary Bengaluru hospital with transplant, cardiac, neuro, PICU and a regional-block fellowship.</t>
+          <t>~500-bed Bengaluru quaternary centre with transplant, neuro, cardiac and a regional-block fellowship.</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
@@ -5918,7 +5918,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Broad super-speciality hospital, but check the reported ₹20 L bond and low stipend first.</t>
+          <t>Bengaluru tertiary hospital with ~9,300 anaesthetics a year, cardiac, neuro and liver-transplant anaesthesia, small batches.</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
@@ -5998,7 +5998,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Declared stipend ₹35,000 is below the NBEMS minimum, and hands-on is described as limited.</t>
+          <t>Stipend declared to MCC is below the NBEMS legal minimum; hands-on is described as consultant-led.</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Chennai hospital with official cardiac anaesthesia and surgical gastro programmes, so the cardiac and GI work is real.</t>
+          <t>Chennai hospital with official DNB cardiac anaesthesia and surgical gastro courses, so cardiac and GI work is real.</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Older Coimbatore hospital with a cardiac anaesthesia course, but thin anaesthesia faculty and moderate volume.</t>
+          <t>Old Coimbatore hospital with a cardiac anaesthesia course, but only 2 anaesthetists listed.</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Good transplant and cardiac work, but declared Y1 stipend is below the NBEMS minimum.</t>
+          <t>Strong transplant and cardiac case mix, but declared year-1 stipend ₹39,500 is below the NBEMS minimum.</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Established NABH hospital in Nagercoil with neuro, trauma, paeds-surgery and onco work; no cardiac surgery.</t>
+          <t>Steady Nagercoil DNB centre with decent volume, but little super-speciality work and a near-floor stipend.</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
@@ -6394,7 +6394,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Almost no public information about this hospital; stipend ₹50k, no bond.</t>
+          <t>Semi-urban Ranipet hospital with a placeholder website, no cardiac surgery and one DNB seat.</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Declared stipend below the legal floor and no information on facilities; avoid.</t>
+          <t>Erode critical-care centre declaring a ₹35k stipend, below the legal floor, with no super-specialities.</t>
         </is>
       </c>
       <c r="F75" s="3" t="n">
@@ -6554,7 +6554,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Nothing verified, not even ownership or services; take it only as a backup.</t>
+          <t>Shillong mission hospital with ~3,000 surgeries a year and campus housing, but no cardiac surgery or transplant.</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Runs official super-speciality courses (GI surgery, Neuro, Renal/Transplant); confirm hands-on and hours with seniors.</t>
+          <t>Good super-speciality mix, but doctors protested management humiliation in June 2026.</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Almost no online footprint; nothing to judge training on.</t>
+          <t>Guwahati cardiac-led hospital with DNB cardiac anaesthesia, a 100-bed critical-care complex and broad anaesthesia work.</t>
         </is>
       </c>
       <c r="F78" s="3" t="n">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>NABH hospital claiming cardiac surgery, neuro and onco, with no bond. Confirm real case volumes.</t>
+          <t>Guwahati hospital with a CTVS team and cardiac anaesthetist, but one seat and modest volume.</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
@@ -6878,7 +6878,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>100-bed hospital with 5 OTs; neuro and burns listed but limited case mix.</t>
+          <t>Small 100-bed Guwahati hospital where an ICU doctor died by suicide on duty in September 2026.</t>
         </is>
       </c>
       <c r="F80" s="3" t="n">
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Claims CTVS, neuro and transplant with a good stipend, but facts are directory-only; verify first.</t>
+          <t>Strongest case mix in the list, but a nurse died by suicide at the hospital amid harassment allegations.</t>
         </is>
       </c>
       <c r="F81" s="2" t="n">
@@ -7042,7 +7042,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Well-equipped Rourkela tertiary centre with neuro, cardiac, trauma and big ICUs, plus the highest stipend here.</t>
+          <t>Well-equipped Rourkela centre with neuro, cardiac, trauma and big ICUs, plus the highest stipend here.</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Imphal NABH hospital with renal transplant and neuro work, but Manipur's security situation is a real concern.</t>
+          <t>Strong Imphal anaesthesia department with transplant and cardiac work, but Manipur's security is a concern.</t>
         </is>
       </c>
       <c r="F83" s="3" t="n">
@@ -7206,7 +7206,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Biggest hospital in this list: 700 beds, 200 ICU beds, 28 OTs, with cardiac, neuro and transplant work.</t>
+          <t>Large 700-bed Vizag hospital: 28 OTs, 200 ICU beds, transplant, cardiac and neuro work, ₹61k stipend.</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
@@ -7288,7 +7288,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>200-bed Apollo unit focused on ortho, trauma and cardiology; no proven super-speciality depth.</t>
+          <t>Small Apollo unit focused on ortho, trauma and cardiology; few super-speciality lists and anaesthesia its only DNB.</t>
         </is>
       </c>
       <c r="F85" s="2" t="n">
@@ -7452,7 +7452,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Busy KIMS hospital in Anantapur with real cardiac, neuro, transplant and trauma numbers and 10 anaesthetists.</t>
+          <t>Busy KIMS hospital in Anantapur with real cardiac, neuro, transplant and trauma numbers.</t>
         </is>
       </c>
       <c r="F87" s="2" t="n">
@@ -7532,7 +7532,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Official cardiac anaesthesia and neurosurgery programmes in Vizag; hospital changed owners after insolvency in 2024.</t>
+          <t>MGM SevenHills Vizag: official cardiac-anaesthesia and neurosurgery super-speciality courses, transplant programme, ₹61k stipend.</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
@@ -7612,7 +7612,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>200-bed Vizag multispeciality hospital; super-speciality exposure undocumented.</t>
+          <t>200-bed Vizag hospital now run by KIMS; accreditation runs only to Dec 2026.</t>
         </is>
       </c>
       <c r="F89" s="2" t="n">

</xml_diff>

<commit_message>
Shortlist: deep pass (job posts, LinkedIn, papers, official ICU pages) — hospital facts replace national rules for ICU in 78/88, hours in 19; 154 sourced items in detail panels
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -677,7 +677,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Small programme: 2 DNB anaesthesia seats (2025)</t>
+          <t>Small programme: 2 DNB anaesthesia seats (2025); 260-bed NABH hospital with cath lab (directory listing)</t>
         </is>
       </c>
       <c r="O2" s="4" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>3,204 surgeries in 2024; 3 full-time anaesthesia faculty; 2+1 DNB seats</t>
+          <t>3,204 surgeries in 2024; 3 full-time anaesthesia faculty; 2+1 DNB seats. Residents: Site summary: steady patient load, approachable faculty, irregular academics</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Directory lists a 72-bed ICU (trauma, cardiac, neuro, medical); unverified</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,11 @@
           <t>Some — reported, but not by residents</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>400+ bed hospital with laminar-flow OTs</t>
+        </is>
+      </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -851,7 +855,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>60 dedicated ICU beds; ICU and emergency anaesthesia teams 24x7</t>
         </is>
       </c>
     </row>
@@ -915,7 +919,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Moderate case load; limited independent procedures</t>
+          <t>Moderate case load; limited independent procedures; 350 beds, 9 laminar-flow OTs</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
@@ -935,7 +939,7 @@
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>100 critical care beds in a 350-bed hospital</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1017,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>20 critical care beds plus 15 level-III NICU beds, HDU</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1081,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Dedicated onco- and cardiac-anaesthesia heads</t>
+          <t>Dedicated onco- and cardiac-anaesthesia heads; 380 beds, 13 modular OTs</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
@@ -1093,7 +1097,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>118 critical care beds in a 380-bed hospital</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1243,11 @@
           <t>Unclear — no reliable resident review</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>501 sanctioned beds; CTVS, paediatric surgery, high-risk obstetrics, cath lab</t>
+        </is>
+      </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -1257,7 +1265,7 @@
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Directory lists only 14 ICU beds; unverified</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1491,11 @@
           <t>Some — reported, but not by residents</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Neurosurgery, vascular, HPB, joint replacement, oncology cases; 1 DNB anaesthesia seat</t>
+        </is>
+      </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -1497,7 +1509,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>NABH-accredited critical care service; ICU listed</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1595,7 @@
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Advanced ICU listed among hospital services</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1735,11 @@
           <t>Some — reported, but not by residents</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>200-bed NABH hospital, 20+ specialties; cardiac anaesthesia and CTVS; Ayushman/ESIC patients</t>
+        </is>
+      </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -1795,7 +1811,11 @@
           <t>Some — reported, but not by residents</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Secondary-care, PM-JAY hospital: surgery, ortho, OBG, paediatrics, medicine</t>
+        </is>
+      </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -1809,7 +1829,7 @@
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>ICU services listed; no bed count</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1987,7 @@
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Critical-care area monitored by IP cameras; no ICU bed count</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2051,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Strong ICU exposure; procedures mostly consultant-led</t>
+          <t>Strong ICU exposure; procedures mostly consultant-led; 310-bed hospital</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
@@ -2351,7 +2371,11 @@
           <t>Some — reported, but not by residents</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Specialties: cardiology, neurology, GI, oncology, surgery, OBG, ENT</t>
+        </is>
+      </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -2449,7 +2473,7 @@
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Separate MICU, SICU, CCU, PICU and HDU; 24x7 critical care</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2711,7 @@
       </c>
       <c r="R27" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>36-bed ICU, 10-bed paediatric/neonatal ICU, 12-bed HDU</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2857,11 @@
           <t>Some — reported, but not by residents</t>
         </is>
       </c>
-      <c r="N29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>Kidney transplant and dialysis services; surgical ICU</t>
+        </is>
+      </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -2847,7 +2875,7 @@
       </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>New 11-bed ICU added with 78-bed expansion (FY25)</t>
         </is>
       </c>
     </row>
@@ -2933,7 +2961,7 @@
       </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>New campus planned two 10-bed ICU wards (2024 plan)</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3163,7 @@
       </c>
       <c r="R33" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>100 critical care beds incl. cardiac and neuro ICUs</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3225,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>3 DNB anaesthesia seats (2025)</t>
+          <t>3 DNB anaesthesia seats (2025); 350 beds incl. 75 critical care beds (Sep 2024)</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
@@ -3368,12 +3396,12 @@
       <c r="P36" s="2" t="inlineStr"/>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>Group-wide staff reviews cite long hours, six-day weeks</t>
         </is>
       </c>
       <c r="R36" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>40-bed ICU, 20 intensivists; DNB anaesthesia and DrNB critical care</t>
         </is>
       </c>
     </row>
@@ -3437,7 +3465,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>300 beds; 2 seats; wide range of cases, regular workshops</t>
+          <t>300 beds; 2 seats; wide range of cases, regular workshops. Residents: Hospital-posted DNB anaesthesia resident testimonial: supportive faculty, wide case range, regular workshops</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
@@ -3457,7 +3485,7 @@
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Runs IDCCM critical-care diploma (2 seats); anaesthesia HOD heads critical care</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3549,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>175 beds; cardiac, neuro, oncology; Fortis group says supervised hands-on</t>
+          <t>175 beds; cardiac, neuro, oncology; Fortis group says supervised hands-on. Residents: Junior resident (2021, dept unstated): good work environment</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
@@ -3532,12 +3560,12 @@
       <c r="P38" s="2" t="inlineStr"/>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>One junior resident review: rotational schedule, strict timings (2021)</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>59 ICU beds</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3627,7 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>200 beds, 4 seats; ortho-heavy; USG/PNS blocks, TIVA, fibreoptic, POCUS, simulation</t>
+          <t>200 beds, 4 seats; ortho-heavy; USG/PNS blocks, TIVA, fibreoptic, POCUS, simulation. Residents: Junior resident (2018): lots of freehand builds confidence; heavy work pressure</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
@@ -3610,7 +3638,7 @@
       <c r="P39" s="2" t="inlineStr"/>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>Junior resident review: strict timings, no personal life from work pressure</t>
         </is>
       </c>
       <c r="R39" s="2" t="inlineStr">
@@ -3774,12 +3802,12 @@
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>Group-wide staff reviews cite long hours, six-day weeks</t>
         </is>
       </c>
       <c r="R41" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Dedicated neuro ICU with neuro-anaesthesia input</t>
         </is>
       </c>
     </row>
@@ -3843,7 +3871,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>Heart-care centre; cardiac anaesthesia exposure likely</t>
+          <t>Heart-care centre; cardiac anaesthesia exposure likely; 148 beds; 2 DNB anaesthesia seats; separate cardiac anaesthesia unit</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
@@ -4009,7 +4037,7 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>60–70 cardiac cases/month, 300+ general; non-OR and cath-lab work</t>
+          <t>60–70 cardiac cases/month, 300+ general; non-OR and cath-lab work. Residents: First-batch resident: structured, protocol-driven training; closed ICU builds ventilation and sepsis confidence</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
@@ -4093,7 +4121,7 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>Spinals, epidurals, USG/PNS blocks, intubation, central lines; 970 beds</t>
+          <t>Spinals, epidurals, USG/PNS blocks, intubation, central lines; 970 beds. Residents: DNB resident (2021): very satisfied, not hectic, ample study time on duty; 6 consultants</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
@@ -4182,7 +4210,7 @@
       <c r="P46" s="2" t="inlineStr"/>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>Staff reviews (non-resident): mostly six-day weeks</t>
         </is>
       </c>
       <c r="R46" s="2" t="inlineStr">
@@ -4267,7 +4295,7 @@
       </c>
       <c r="R47" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>MICU and CICU; ICU, NICU, CCU run by intensivists</t>
         </is>
       </c>
     </row>
@@ -4353,7 +4381,7 @@
       </c>
       <c r="R48" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>12-bed paediatric ICU planned; new trauma centre ICU at medical college</t>
         </is>
       </c>
     </row>
@@ -4665,7 +4693,7 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>First DNB conference Feb 2024; trainees presented 11 papers</t>
+          <t>First DNB conference Feb 2024; trainees presented 11 papers; 910 beds</t>
         </is>
       </c>
       <c r="O52" s="6" t="inlineStr">
@@ -4849,7 +4877,7 @@
       </c>
       <c r="R54" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>42-bed intensive care facility</t>
         </is>
       </c>
     </row>
@@ -4913,7 +4941,7 @@
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>1,000+ OPD visits a day; ED, ICU and OT rotations</t>
+          <t>1,000+ OPD visits a day; ED, ICU and OT rotations; 284 beds; organ transplant centre</t>
         </is>
       </c>
       <c r="O55" s="4" t="inlineStr">
@@ -4929,7 +4957,7 @@
       </c>
       <c r="R55" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Many ICUs incl. surgical, neuro, cardiac, paediatric; ECMO; PACU, HDU</t>
         </is>
       </c>
     </row>
@@ -5089,7 +5117,7 @@
       </c>
       <c r="R57" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>36-bed adult ICU, 13 CCU, 5 neuro, 8 PICU, 8 NICU</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5179,11 @@
           <t>Some — reported, but not by residents</t>
         </is>
       </c>
-      <c r="N58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>7 operating theatres; cardiac, paediatric, neuro, obstetric anaesthesia listed</t>
+        </is>
+      </c>
       <c r="O58" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -5165,7 +5197,7 @@
       </c>
       <c r="R58" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>22 ICU beds in a 168-bed hospital</t>
         </is>
       </c>
     </row>
@@ -5229,7 +5261,7 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>DNB since 2008; ~50 residents across specialties</t>
+          <t>DNB since 2008; ~50 residents across specialties; Rotations across OTs, ICU, NICU, emergency</t>
         </is>
       </c>
       <c r="O59" s="4" t="inlineStr">
@@ -5489,7 +5521,7 @@
       </c>
       <c r="R62" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Modern ICUs and cath lab; bed count not stated</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5583,11 @@
           <t>Some — reported, but not by residents</t>
         </is>
       </c>
-      <c r="N63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>125-bed hospital; Fortis acquired it Dec 2025</t>
+        </is>
+      </c>
       <c r="O63" s="4" t="inlineStr">
         <is>
           <t>OK — nothing bad found online</t>
@@ -5629,7 +5665,7 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>228 beds, 8 OTs; cardiac and neuro centres</t>
+          <t>228 beds, 8 OTs; cardiac and neuro centres; Cardiac anaesthetist (PDCC) on staff</t>
         </is>
       </c>
       <c r="O64" s="4" t="inlineStr">
@@ -5875,7 +5911,7 @@
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>Neurosurgery, ortho, ICU and emergency rotations</t>
+          <t>Neurosurgery, ortho, ICU and emergency rotations; ~500 beds; regional anaesthesia (AORA) fellowship on site</t>
         </is>
       </c>
       <c r="O67" s="4" t="inlineStr">
@@ -5891,7 +5927,7 @@
       </c>
       <c r="R67" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>ICUs benchmarked with APACHE and SMR; transplant programme</t>
         </is>
       </c>
     </row>
@@ -6035,7 +6071,7 @@
       </c>
       <c r="N69" s="2" t="inlineStr">
         <is>
-          <t>300 beds; oncology and critical care; surgical hands-on consultant-led, sometimes limited</t>
+          <t>300 beds; oncology and critical care; surgical hands-on consultant-led, sometimes limited. Residents: Alumnus (2022–25) lists USG blocks, fibreoptic, TEE, PA catheter and lines among skills</t>
         </is>
       </c>
       <c r="O69" s="4" t="inlineStr">
@@ -6051,7 +6087,7 @@
       </c>
       <c r="R69" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Residents independently manage ICU ventilation, sedation, weaning, invasive monitoring</t>
         </is>
       </c>
     </row>
@@ -6129,7 +6165,7 @@
       </c>
       <c r="R70" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Anaesthesia and critical care run as one department; MD/DNB anaesthetists staff the CCU</t>
         </is>
       </c>
     </row>
@@ -6271,7 +6307,7 @@
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>8 anaesthesiologists; active renal transplant (125 done)</t>
+          <t>8 anaesthesiologists; active renal transplant (125 done); Adult and paediatric open-heart cardiac anaesthesia; thoracic cases like giant thymoma</t>
         </is>
       </c>
       <c r="O72" s="4" t="inlineStr">
@@ -6351,7 +6387,7 @@
       </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
-          <t>~200 beds; NICU, chemotherapy, kidney transplant</t>
+          <t>~200 beds; NICU, chemotherapy, kidney transplant. Residents: Nearly all past anaesthesia DNB trainees passed; two left mid-course</t>
         </is>
       </c>
       <c r="O73" s="4" t="inlineStr">
@@ -6447,7 +6483,7 @@
       </c>
       <c r="R74" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Separate critical care department led by its own consultant in-charge</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6547,7 @@
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>DNB anaesthesia since Jan 2024; 2 primary + 1 secondary seats</t>
+          <t>DNB anaesthesia since Jan 2024; 2 primary + 1 secondary seats. Residents: Duty doctor: good place to learn; MD is an emergency-medicine expert</t>
         </is>
       </c>
       <c r="O75" s="4" t="inlineStr">
@@ -6522,7 +6558,7 @@
       <c r="P75" s="2" t="inlineStr"/>
       <c r="Q75" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>Duty doctor review: 6-day week, flexible timings (2018)</t>
         </is>
       </c>
       <c r="R75" s="2" t="inlineStr">
@@ -6766,7 +6802,7 @@
       <c r="P78" s="2" t="inlineStr"/>
       <c r="Q78" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>Department gives round-the-clock cover of OTs, ICUs and cath lab</t>
         </is>
       </c>
       <c r="R78" s="2" t="inlineStr">
@@ -6933,7 +6969,7 @@
       </c>
       <c r="R80" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Surgical ICU; ICU runs prospective sepsis research (48-patient ultrasound study)</t>
         </is>
       </c>
     </row>
@@ -7015,7 +7051,7 @@
       </c>
       <c r="R81" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Separate critical care dept: medical, surgical, cardiac ICUs; ECMO-trained intensivist</t>
         </is>
       </c>
     </row>
@@ -7090,7 +7126,7 @@
       <c r="P82" s="2" t="inlineStr"/>
       <c r="Q82" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>Aadhaar biometric attendance for DNB residents</t>
         </is>
       </c>
       <c r="R82" s="2" t="inlineStr">
@@ -7159,7 +7195,7 @@
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>High laparoscopic and renal-transplant volumes</t>
+          <t>High laparoscopic and renal-transplant volumes; Open-heart, renal transplant; labour epidurals, USG blocks, awake fibreoptic intubation</t>
         </is>
       </c>
       <c r="O83" s="4" t="inlineStr">
@@ -7261,7 +7297,7 @@
       </c>
       <c r="R84" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Separate critical care dept; its intensivist co-wrote ISCCM sepsis guidance</t>
         </is>
       </c>
     </row>
@@ -7345,7 +7381,7 @@
       </c>
       <c r="R85" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>ICU run by dedicated critical care consultants</t>
         </is>
       </c>
     </row>
@@ -7409,7 +7445,7 @@
       </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>2026: 2 post-diploma anaesthesia seats; no service bond</t>
+          <t>2026: 2 post-diploma anaesthesia seats; no service bond; Paediatric orthopaedic and hip-preservation surgery published from here</t>
         </is>
       </c>
       <c r="O86" s="4" t="inlineStr">
@@ -7425,7 +7461,7 @@
       </c>
       <c r="R86" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>Critical care led by anaesthesia-trained HOD (MD Anaesthesia PGIMER, PDCC-CCM)</t>
         </is>
       </c>
     </row>
@@ -7569,7 +7605,7 @@
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>~300 beds; heart/lung, liver, kidney transplant, CTVS, neurosurgery</t>
+          <t>~300 beds; heart/lung, liver, kidney transplant, CTVS, neurosurgery. Residents: Surgery DNB alumnus: anaesthesia and medicine also good; small hospital, adequate load, academics irregular</t>
         </is>
       </c>
       <c r="O88" s="4" t="inlineStr">
@@ -7580,7 +7616,7 @@
       <c r="P88" s="2" t="inlineStr"/>
       <c r="Q88" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>Surgery DNB alumnus: 8am-2pm and 5-9pm, on call alternate days (surgery, not anaesthesia)</t>
         </is>
       </c>
       <c r="R88" s="2" t="inlineStr">
@@ -7665,7 +7701,7 @@
       </c>
       <c r="R89" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>6 specialised ICUs, over 50 ICU beds</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Duty hours: replace the inaccurate '12 h/48 h rule' with the actual NBEMS/NMC/state rules per seat type
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
+++ b/public/NEETPG_Anaesthesia_Shortlist_Sheet.xlsx
@@ -688,12 +688,12 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>General: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -1012,7 +1012,7 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -1092,7 +1092,7 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>General: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
         </is>
       </c>
     </row>
@@ -1344,12 +1344,12 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>General: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
@@ -1504,7 +1504,7 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
@@ -1668,7 +1668,7 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
@@ -1748,12 +1748,12 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>General: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1824,7 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
@@ -1904,7 +1904,7 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
@@ -1982,7 +1982,7 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
@@ -2062,7 +2062,7 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
@@ -2142,7 +2142,7 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
@@ -2306,7 +2306,7 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
@@ -2384,12 +2384,12 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>General: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
         </is>
       </c>
     </row>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
@@ -2626,7 +2626,7 @@
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
@@ -2706,7 +2706,7 @@
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
@@ -2790,12 +2790,12 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: NMC 'reasonable hours', weekly off, 20+5 days leave/yr. 72+ h weeks common</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NMC MD curriculum)</t>
+          <t>General: 4 months ICU over 3 years (NMC MD curriculum)</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2870,7 @@
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr">
@@ -3158,7 +3158,7 @@
       <c r="P33" s="2" t="inlineStr"/>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr">
@@ -3236,7 +3236,7 @@
       <c r="P34" s="2" t="inlineStr"/>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R34" s="2" t="inlineStr">
@@ -3316,12 +3316,12 @@
       <c r="P35" s="2" t="inlineStr"/>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>General: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
@@ -3718,7 +3718,7 @@
       <c r="P40" s="2" t="inlineStr"/>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -3882,7 +3882,7 @@
       <c r="P42" s="2" t="inlineStr"/>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
@@ -3968,7 +3968,7 @@
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R43" s="2" t="inlineStr">
@@ -4048,7 +4048,7 @@
       <c r="P44" s="2" t="inlineStr"/>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr">
@@ -4290,7 +4290,7 @@
       <c r="P47" s="2" t="inlineStr"/>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R47" s="2" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R48" s="2" t="inlineStr">
@@ -4540,7 +4540,7 @@
       <c r="P50" s="2" t="inlineStr"/>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R50" s="2" t="inlineStr">
@@ -4620,7 +4620,7 @@
       <c r="P51" s="2" t="inlineStr"/>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R51" s="2" t="inlineStr">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R52" s="2" t="inlineStr">
@@ -4792,7 +4792,7 @@
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R53" s="2" t="inlineStr">
@@ -4872,7 +4872,7 @@
       <c r="P54" s="2" t="inlineStr"/>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R54" s="2" t="inlineStr">
@@ -4952,7 +4952,7 @@
       <c r="P55" s="2" t="inlineStr"/>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R55" s="2" t="inlineStr">
@@ -5032,7 +5032,7 @@
       <c r="P56" s="2" t="inlineStr"/>
       <c r="Q56" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R56" s="2" t="inlineStr">
@@ -5112,7 +5112,7 @@
       <c r="P57" s="2" t="inlineStr"/>
       <c r="Q57" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R57" s="2" t="inlineStr">
@@ -5272,7 +5272,7 @@
       <c r="P59" s="2" t="inlineStr"/>
       <c r="Q59" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R59" s="2" t="inlineStr">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R60" s="2" t="inlineStr">
@@ -5438,7 +5438,7 @@
       <c r="P61" s="2" t="inlineStr"/>
       <c r="Q61" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R61" s="2" t="inlineStr">
@@ -5516,7 +5516,7 @@
       <c r="P62" s="2" t="inlineStr"/>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr">
@@ -5596,7 +5596,7 @@
       <c r="P63" s="2" t="inlineStr"/>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr">
@@ -5676,7 +5676,7 @@
       <c r="P64" s="2" t="inlineStr"/>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R64" s="2" t="inlineStr">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       <c r="P66" s="2" t="inlineStr"/>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R66" s="2" t="inlineStr">
@@ -5922,7 +5922,7 @@
       <c r="P67" s="2" t="inlineStr"/>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr">
@@ -6002,7 +6002,7 @@
       <c r="P68" s="2" t="inlineStr"/>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R68" s="2" t="inlineStr">
@@ -6082,7 +6082,7 @@
       <c r="P69" s="2" t="inlineStr"/>
       <c r="Q69" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R69" s="2" t="inlineStr">
@@ -6160,7 +6160,7 @@
       <c r="P70" s="2" t="inlineStr"/>
       <c r="Q70" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R70" s="2" t="inlineStr">
@@ -6238,7 +6238,7 @@
       <c r="P71" s="2" t="inlineStr"/>
       <c r="Q71" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R71" s="2" t="inlineStr">
@@ -6318,12 +6318,12 @@
       <c r="P72" s="2" t="inlineStr"/>
       <c r="Q72" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R72" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>General: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
         </is>
       </c>
     </row>
@@ -6478,7 +6478,7 @@
       <c r="P74" s="2" t="inlineStr"/>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R74" s="2" t="inlineStr">
@@ -6638,7 +6638,7 @@
       <c r="P76" s="2" t="inlineStr"/>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R76" s="2" t="inlineStr">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="Q77" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R77" s="2" t="inlineStr">
@@ -6882,7 +6882,7 @@
       <c r="P79" s="2" t="inlineStr"/>
       <c r="Q79" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R79" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R80" s="2" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R81" s="2" t="inlineStr">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="Q83" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R83" s="2" t="inlineStr">
@@ -7292,7 +7292,7 @@
       </c>
       <c r="Q84" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R84" s="2" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="Q85" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R85" s="2" t="inlineStr">
@@ -7456,7 +7456,7 @@
       <c r="P86" s="2" t="inlineStr"/>
       <c r="Q86" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R86" s="2" t="inlineStr">
@@ -7536,7 +7536,7 @@
       <c r="P87" s="2" t="inlineStr"/>
       <c r="Q87" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R87" s="2" t="inlineStr">
@@ -7621,7 +7621,7 @@
       </c>
       <c r="R88" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>General: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
         </is>
       </c>
     </row>
@@ -7696,7 +7696,7 @@
       <c r="P89" s="2" t="inlineStr"/>
       <c r="Q89" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R89" s="2" t="inlineStr">
@@ -7776,12 +7776,12 @@
       <c r="P90" s="2" t="inlineStr"/>
       <c r="Q90" s="2" t="inlineStr">
         <is>
-          <t>Rule: max 12 h continuous duty, 48 h/week, 1 weekly off (often exceeded)</t>
+          <t>General: no NBEMS hour cap; weekly off + 30 days leave/yr. 72+ h weeks common (2025 survey)</t>
         </is>
       </c>
       <c r="R90" s="2" t="inlineStr">
         <is>
-          <t>Rule: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
+          <t>General: 4 months ICU over 3 years (NBEMS DNB curriculum)</t>
         </is>
       </c>
     </row>

</xml_diff>